<commit_message>
Corregí el nombre de las pantallas
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/momuychayis/Documents/Python courses/Ventas_casa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F593614B-342A-DA40-A03C-3824B94848AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5836251-6390-1148-B9F5-CE4CB0AEC571}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2940" yWindow="600" windowWidth="24460" windowHeight="15880" xr2:uid="{CD00CDD9-C0C8-D147-B0FC-6E5A64DE4059}"/>
   </bookViews>
@@ -375,9 +375,6 @@
     <t xml:space="preserve">Mide </t>
   </si>
   <si>
-    <t>Pantalla inteligente de 50''</t>
-  </si>
-  <si>
     <t>Coqueta de cmuy buena madera, originalmente comprada en Sarchí. Lo pintamos hace algunos años para cambiarle el estilo.</t>
   </si>
   <si>
@@ -609,6 +606,9 @@
   </si>
   <si>
     <t>Pequeñita, ideal para poner el celular y libros.</t>
+  </si>
+  <si>
+    <t>Pantalla inteligente de 50 pulgadas</t>
   </si>
 </sst>
 </file>
@@ -1044,7 +1044,7 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B2" t="s">
         <v>7</v>
@@ -1090,7 +1090,7 @@
     </row>
     <row r="4" spans="1:10" ht="306" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B4" t="s">
         <v>7</v>
@@ -1099,24 +1099,24 @@
         <v>14</v>
       </c>
       <c r="D4" t="s">
+        <v>141</v>
+      </c>
+      <c r="E4" t="s">
         <v>142</v>
-      </c>
-      <c r="E4" t="s">
-        <v>143</v>
       </c>
       <c r="F4" s="2">
         <v>4000000</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="J4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B5" t="s">
         <v>7</v>
@@ -1125,7 +1125,7 @@
         <v>14</v>
       </c>
       <c r="D5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E5" t="s">
         <v>6</v>
@@ -1137,7 +1137,7 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B6" t="s">
         <v>7</v>
@@ -1146,10 +1146,10 @@
         <v>14</v>
       </c>
       <c r="D6" t="s">
+        <v>163</v>
+      </c>
+      <c r="E6" t="s">
         <v>164</v>
-      </c>
-      <c r="E6" t="s">
-        <v>165</v>
       </c>
       <c r="F6" s="2">
         <v>8300000</v>
@@ -1158,7 +1158,7 @@
     </row>
     <row r="7" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>112</v>
+        <v>186</v>
       </c>
       <c r="B7" t="s">
         <v>11</v>
@@ -1184,28 +1184,33 @@
     </row>
     <row r="8" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>167</v>
+        <v>186</v>
       </c>
       <c r="B8" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>14</v>
       </c>
       <c r="D8" t="s">
-        <v>169</v>
+        <v>19</v>
+      </c>
+      <c r="E8" t="s">
+        <v>15</v>
       </c>
       <c r="F8" s="2">
-        <v>170000</v>
+        <v>120000</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="J8" s="3"/>
+        <v>12</v>
+      </c>
+      <c r="H8" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="9" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B9" t="s">
         <v>7</v>
@@ -1214,41 +1219,36 @@
         <v>14</v>
       </c>
       <c r="D9" t="s">
+        <v>168</v>
+      </c>
+      <c r="F9" s="2">
+        <v>170000</v>
+      </c>
+      <c r="G9" s="5" t="s">
         <v>169</v>
-      </c>
-      <c r="F9" s="2">
-        <v>130000</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>170</v>
       </c>
       <c r="J9" s="3"/>
     </row>
     <row r="10" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>112</v>
+        <v>167</v>
       </c>
       <c r="B10" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>14</v>
       </c>
       <c r="D10" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" t="s">
-        <v>15</v>
+        <v>168</v>
       </c>
       <c r="F10" s="2">
-        <v>120000</v>
+        <v>130000</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="H10" t="s">
-        <v>51</v>
-      </c>
+        <v>169</v>
+      </c>
+      <c r="J10" s="3"/>
     </row>
     <row r="11" spans="1:10" ht="68" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
@@ -1270,7 +1270,7 @@
         <v>80000</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="37" customHeight="1" x14ac:dyDescent="0.2">
@@ -1304,7 +1304,7 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B13" t="s">
         <v>11</v>
@@ -1316,7 +1316,7 @@
         <v>20</v>
       </c>
       <c r="E13" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F13" s="2">
         <v>15000</v>
@@ -1327,7 +1327,7 @@
     </row>
     <row r="14" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B14" t="s">
         <v>11</v>
@@ -1336,7 +1336,7 @@
         <v>14</v>
       </c>
       <c r="D14" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E14" t="s">
         <v>109</v>
@@ -1345,7 +1345,7 @@
         <v>40000</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="H14" t="s">
         <v>32</v>
@@ -1366,7 +1366,7 @@
         <v>45000</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H15" t="s">
         <v>34</v>
@@ -1406,7 +1406,7 @@
         <v>100000</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="H17" t="s">
         <v>36</v>
@@ -1414,7 +1414,7 @@
     </row>
     <row r="18" spans="1:10" ht="102" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B18" t="s">
         <v>74</v>
@@ -1423,7 +1423,7 @@
         <v>14</v>
       </c>
       <c r="D18" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E18" t="s">
         <v>23</v>
@@ -1432,7 +1432,7 @@
         <v>120000</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
@@ -1455,7 +1455,7 @@
         <v>30000</v>
       </c>
       <c r="G19" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H19" t="s">
         <v>37</v>
@@ -1486,7 +1486,7 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B21" t="s">
         <v>74</v>
@@ -1495,7 +1495,7 @@
         <v>14</v>
       </c>
       <c r="D21" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E21" t="s">
         <v>109</v>
@@ -1504,7 +1504,7 @@
         <v>25000</v>
       </c>
       <c r="G21" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="68" x14ac:dyDescent="0.2">
@@ -1524,7 +1524,7 @@
         <v>120000</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H22" t="s">
         <v>39</v>
@@ -1696,7 +1696,7 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B30" t="s">
         <v>74</v>
@@ -1714,7 +1714,7 @@
         <v>25000</v>
       </c>
       <c r="G30" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.2">
@@ -1745,7 +1745,7 @@
     </row>
     <row r="32" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B32" t="s">
         <v>74</v>
@@ -1763,12 +1763,12 @@
         <v>10000</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="119" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B33" t="s">
         <v>74</v>
@@ -1786,7 +1786,7 @@
         <v>35000</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H33" t="s">
         <v>56</v>
@@ -1794,25 +1794,25 @@
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
+        <v>122</v>
+      </c>
+      <c r="B34" t="s">
         <v>123</v>
       </c>
-      <c r="B34" t="s">
+      <c r="C34" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D34" t="s">
         <v>124</v>
       </c>
-      <c r="C34" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D34" t="s">
-        <v>125</v>
-      </c>
       <c r="E34" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F34" s="2">
         <v>20000</v>
       </c>
       <c r="G34" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="H34" t="s">
         <v>63</v>
@@ -1820,36 +1820,36 @@
     </row>
     <row r="35" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
+        <v>130</v>
+      </c>
+      <c r="B35" t="s">
+        <v>136</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D35" t="s">
         <v>131</v>
       </c>
-      <c r="B35" t="s">
-        <v>137</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D35" t="s">
+      <c r="E35" t="s">
         <v>132</v>
-      </c>
-      <c r="E35" t="s">
-        <v>133</v>
       </c>
       <c r="F35" s="2">
         <v>15000</v>
       </c>
       <c r="G35" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H35" t="s">
         <v>65</v>
       </c>
       <c r="J35" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B36" t="s">
         <v>71</v>
@@ -1858,13 +1858,13 @@
         <v>14</v>
       </c>
       <c r="D36" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F36" s="2">
         <v>8000</v>
       </c>
       <c r="G36" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H36" t="s">
         <v>59</v>
@@ -1872,10 +1872,10 @@
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
+        <v>127</v>
+      </c>
+      <c r="B37" t="s">
         <v>128</v>
-      </c>
-      <c r="B37" t="s">
-        <v>129</v>
       </c>
       <c r="C37" s="4" t="s">
         <v>14</v>
@@ -1890,7 +1890,7 @@
         <v>10000</v>
       </c>
       <c r="G37" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H37" t="s">
         <v>64</v>
@@ -1898,10 +1898,10 @@
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B38" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C38" s="4" t="s">
         <v>14</v>
@@ -1916,7 +1916,7 @@
         <v>4000</v>
       </c>
       <c r="G38" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H38" t="s">
         <v>67</v>
@@ -1924,10 +1924,10 @@
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B39" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>14</v>
@@ -1942,7 +1942,7 @@
         <v>2000</v>
       </c>
       <c r="G39" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="H39" t="s">
         <v>68</v>
@@ -1950,7 +1950,7 @@
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B40" t="s">
         <v>71</v>
@@ -1962,7 +1962,7 @@
         <v>10000</v>
       </c>
       <c r="G40" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="H40" t="s">
         <v>69</v>
@@ -1970,10 +1970,10 @@
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B41" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>14</v>
@@ -1987,10 +1987,10 @@
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B42" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>14</v>
@@ -2062,7 +2062,7 @@
         <v>0</v>
       </c>
       <c r="G45" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="H45" t="s">
         <v>40</v>
@@ -2070,10 +2070,10 @@
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B46" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C46" s="4" t="s">
         <v>14</v>
@@ -2082,7 +2082,7 @@
         <v>0</v>
       </c>
       <c r="G46" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H46" t="s">
         <v>61</v>
@@ -2090,10 +2090,10 @@
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B47" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C47" s="4" t="s">
         <v>14</v>
@@ -2102,7 +2102,7 @@
         <v>0</v>
       </c>
       <c r="G47" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H47" t="s">
         <v>54</v>
@@ -2110,7 +2110,7 @@
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B48" t="s">
         <v>74</v>
@@ -2122,7 +2122,7 @@
         <v>0</v>
       </c>
       <c r="G48" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H48" t="s">
         <v>46</v>
@@ -2130,7 +2130,7 @@
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B49" t="s">
         <v>11</v>
@@ -2147,7 +2147,7 @@
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B50" t="s">
         <v>74</v>
@@ -2159,7 +2159,7 @@
         <v>0</v>
       </c>
       <c r="G50" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="H50" t="s">
         <v>49</v>
@@ -2167,10 +2167,10 @@
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B51" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C51" s="4" t="s">
         <v>14</v>
@@ -2184,7 +2184,7 @@
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B52" t="s">
         <v>71</v>
@@ -2196,7 +2196,7 @@
         <v>0</v>
       </c>
       <c r="G52" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H52" t="s">
         <v>55</v>

</xml_diff>

<commit_message>
Cambie los modelos a N/A en el excel
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/momuychayis/Documents/Python courses/Ventas_casa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5836251-6390-1148-B9F5-CE4CB0AEC571}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{826E957C-B5B4-B641-941A-C5D63225D9BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2940" yWindow="600" windowWidth="24460" windowHeight="15880" xr2:uid="{CD00CDD9-C0C8-D147-B0FC-6E5A64DE4059}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="189">
   <si>
     <t>Nombre</t>
   </si>
@@ -64,9 +64,6 @@
     <t>Referencia</t>
   </si>
   <si>
-    <t>50" Crystal UHD 4K CU7000 Smart TV</t>
-  </si>
-  <si>
     <t>https://www.samsung.com/latin/tvs/uhd-4k-tv/cu7000-50-inch-un50cu7000pxpa/</t>
   </si>
   <si>
@@ -80,9 +77,6 @@
   </si>
   <si>
     <t>Disponible</t>
-  </si>
-  <si>
-    <t>50" Crystal UHD 4K CU6000 Smart TV</t>
   </si>
   <si>
     <t>Coqueta</t>
@@ -609,6 +603,19 @@
   </si>
   <si>
     <t>Pantalla inteligente de 50 pulgadas</t>
+  </si>
+  <si>
+    <t>50in Crystal UHD 4K CU7000 Smart TV</t>
+  </si>
+  <si>
+    <t>50in Crystal UHD 4K CU6000 Smart TV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N/A
+</t>
+  </si>
+  <si>
+    <t>N/A</t>
   </si>
 </sst>
 </file>
@@ -1015,13 +1022,13 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>1</v>
@@ -1042,90 +1049,96 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B2" t="s">
         <v>7</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
+      </c>
+      <c r="D2" t="s">
+        <v>188</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>187</v>
       </c>
       <c r="F2" s="2">
         <v>25000</v>
       </c>
       <c r="H2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F3" s="2">
         <v>25000</v>
       </c>
       <c r="G3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="H3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="J3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="306" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B4" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D4" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E4" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="F4" s="2">
         <v>4000000</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J4" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B5" t="s">
         <v>7</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D5" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="E5" t="s">
         <v>6</v>
@@ -1137,19 +1150,19 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B6" t="s">
         <v>7</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D6" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E6" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="F6" s="2">
         <v>8300000</v>
@@ -1158,1048 +1171,1161 @@
     </row>
     <row r="7" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E7" t="s">
-        <v>9</v>
+        <v>185</v>
       </c>
       <c r="F7" s="2">
         <v>140000</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>184</v>
+      </c>
+      <c r="B8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" t="s">
         <v>186</v>
-      </c>
-      <c r="B8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D8" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" t="s">
-        <v>15</v>
       </c>
       <c r="F8" s="2">
         <v>120000</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H8" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B9" t="s">
         <v>7</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D9" t="s">
-        <v>168</v>
+        <v>166</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>187</v>
       </c>
       <c r="F9" s="2">
         <v>170000</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="J9" s="3"/>
     </row>
     <row r="10" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B10" t="s">
         <v>7</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D10" t="s">
-        <v>168</v>
+        <v>166</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>187</v>
       </c>
       <c r="F10" s="2">
         <v>130000</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="J10" s="3"/>
     </row>
     <row r="11" spans="1:10" ht="68" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B11" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D11" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F11" s="2">
         <v>80000</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E12" t="s">
         <v>27</v>
-      </c>
-      <c r="E12" t="s">
-        <v>29</v>
       </c>
       <c r="F12" s="2">
         <v>30000</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="H12" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="J12" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D13" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E13" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="F13" s="2">
         <v>15000</v>
       </c>
       <c r="H13" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>173</v>
+      </c>
+      <c r="B14" t="s">
+        <v>10</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" t="s">
         <v>175</v>
       </c>
-      <c r="B14" t="s">
-        <v>11</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D14" t="s">
-        <v>177</v>
-      </c>
       <c r="E14" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F14" s="2">
         <v>40000</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="H14" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B15" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D15" s="6"/>
+        <v>13</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>187</v>
+      </c>
       <c r="F15" s="2">
         <v>45000</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H15" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B16" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D16" t="s">
-        <v>20</v>
+        <v>18</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>187</v>
       </c>
       <c r="F16" s="2">
         <v>10000</v>
       </c>
       <c r="H16" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="119" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B17" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
+      </c>
+      <c r="D17" t="s">
+        <v>188</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>187</v>
       </c>
       <c r="F17" s="2">
         <v>100000</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H17" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="102" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B18" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D18" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F18" s="2">
         <v>120000</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B19" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D19" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E19" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F19" s="2">
         <v>30000</v>
       </c>
       <c r="G19" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H19" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="J19" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B20" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D20" t="s">
-        <v>79</v>
+        <v>77</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>187</v>
       </c>
       <c r="F20" s="2">
         <v>50000</v>
       </c>
       <c r="H20" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B21" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D21" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="E21" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F21" s="2">
         <v>25000</v>
       </c>
       <c r="G21" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="68" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B22" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D22" t="s">
-        <v>82</v>
+        <v>80</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>187</v>
       </c>
       <c r="F22" s="2">
         <v>120000</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H22" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B23" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
+      </c>
+      <c r="D23" t="s">
+        <v>188</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>187</v>
       </c>
       <c r="F23" s="2">
         <v>80000</v>
       </c>
       <c r="H23" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B24" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
+      </c>
+      <c r="D24" t="s">
+        <v>188</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>187</v>
       </c>
       <c r="F24" s="2">
         <v>15000</v>
       </c>
       <c r="G24" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H24" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B25" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D25" t="s">
-        <v>19</v>
+        <v>17</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>187</v>
       </c>
       <c r="F25" s="2">
         <v>250000</v>
       </c>
       <c r="H25" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B26" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D26" t="s">
-        <v>19</v>
+        <v>17</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>187</v>
       </c>
       <c r="F26" s="2">
         <v>150000</v>
       </c>
       <c r="G26" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H26" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
+        <v>95</v>
+      </c>
+      <c r="B27" t="s">
+        <v>10</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27" t="s">
+        <v>96</v>
+      </c>
+      <c r="E27" t="s">
         <v>97</v>
-      </c>
-      <c r="B27" t="s">
-        <v>11</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D27" t="s">
-        <v>98</v>
-      </c>
-      <c r="E27" t="s">
-        <v>99</v>
       </c>
       <c r="F27" s="2">
         <v>120000</v>
       </c>
       <c r="G27" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H27" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
+        <v>99</v>
+      </c>
+      <c r="B28" t="s">
+        <v>69</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D28" t="s">
+        <v>17</v>
+      </c>
+      <c r="E28" t="s">
         <v>101</v>
-      </c>
-      <c r="B28" t="s">
-        <v>71</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D28" t="s">
-        <v>19</v>
-      </c>
-      <c r="E28" t="s">
-        <v>103</v>
       </c>
       <c r="F28" s="2">
         <v>60000</v>
       </c>
       <c r="G28" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H28" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="J28" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B29" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D29" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E29" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F29" s="2">
         <v>60000</v>
       </c>
       <c r="G29" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="H29" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="J29" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B30" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D30" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E30" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F30" s="2">
         <v>25000</v>
       </c>
       <c r="G30" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B31" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D31" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E31" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F31" s="2">
         <v>35000</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="H31" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B32" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D32" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E32" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F32" s="2">
         <v>10000</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="119" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B33" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D33" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E33" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F33" s="2">
         <v>35000</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H33" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
+        <v>120</v>
+      </c>
+      <c r="B34" t="s">
+        <v>121</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D34" t="s">
         <v>122</v>
       </c>
-      <c r="B34" t="s">
-        <v>123</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D34" t="s">
+      <c r="E34" t="s">
         <v>124</v>
-      </c>
-      <c r="E34" t="s">
-        <v>126</v>
       </c>
       <c r="F34" s="2">
         <v>20000</v>
       </c>
       <c r="G34" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="H34" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="35" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
+        <v>128</v>
+      </c>
+      <c r="B35" t="s">
+        <v>134</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D35" t="s">
+        <v>129</v>
+      </c>
+      <c r="E35" t="s">
         <v>130</v>
-      </c>
-      <c r="B35" t="s">
-        <v>136</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D35" t="s">
-        <v>131</v>
-      </c>
-      <c r="E35" t="s">
-        <v>132</v>
       </c>
       <c r="F35" s="2">
         <v>15000</v>
       </c>
       <c r="G35" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="H35" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J35" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
+        <v>117</v>
+      </c>
+      <c r="B36" t="s">
+        <v>69</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D36" t="s">
         <v>119</v>
       </c>
-      <c r="B36" t="s">
-        <v>71</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D36" t="s">
-        <v>121</v>
+      <c r="E36" s="5" t="s">
+        <v>187</v>
       </c>
       <c r="F36" s="2">
         <v>8000</v>
       </c>
       <c r="G36" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="H36" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B37" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D37" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E37" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F37" s="2">
         <v>10000</v>
       </c>
       <c r="G37" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="H37" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B38" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D38" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E38" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F38" s="2">
         <v>4000</v>
       </c>
       <c r="G38" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="H38" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B39" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D39" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E39" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F39" s="2">
         <v>2000</v>
       </c>
       <c r="G39" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="H39" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B40" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
+      </c>
+      <c r="D40" t="s">
+        <v>188</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>187</v>
       </c>
       <c r="F40" s="2">
         <v>10000</v>
       </c>
       <c r="G40" t="s">
+        <v>148</v>
+      </c>
+      <c r="H40" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
         <v>150</v>
       </c>
-      <c r="H40" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
-        <v>152</v>
-      </c>
       <c r="B41" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
+      </c>
+      <c r="D41" t="s">
+        <v>188</v>
+      </c>
+      <c r="E41" s="5" t="s">
+        <v>187</v>
       </c>
       <c r="F41" s="2">
         <v>0</v>
       </c>
       <c r="H41" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B42" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
+      </c>
+      <c r="D42" t="s">
+        <v>188</v>
+      </c>
+      <c r="E42" s="5" t="s">
+        <v>187</v>
       </c>
       <c r="F42" s="2">
         <v>0</v>
       </c>
       <c r="H42" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B43" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D43" t="s">
-        <v>20</v>
+        <v>18</v>
+      </c>
+      <c r="E43" s="5" t="s">
+        <v>187</v>
       </c>
       <c r="F43" s="2">
         <v>0</v>
       </c>
       <c r="H43" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B44" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D44" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E44" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F44" s="2">
         <v>0</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B45" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D45" t="s">
-        <v>84</v>
+        <v>82</v>
+      </c>
+      <c r="E45" s="5" t="s">
+        <v>187</v>
       </c>
       <c r="F45" s="2">
         <v>0</v>
       </c>
       <c r="G45" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="H45" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B46" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
+      </c>
+      <c r="D46" t="s">
+        <v>188</v>
+      </c>
+      <c r="E46" s="5" t="s">
+        <v>187</v>
       </c>
       <c r="F46" s="2">
         <v>0</v>
       </c>
       <c r="G46" t="s">
+        <v>153</v>
+      </c>
+      <c r="H46" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
         <v>155</v>
       </c>
-      <c r="H46" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
-        <v>157</v>
-      </c>
       <c r="B47" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
+      </c>
+      <c r="D47" t="s">
+        <v>188</v>
+      </c>
+      <c r="E47" s="5" t="s">
+        <v>187</v>
       </c>
       <c r="F47" s="2">
         <v>0</v>
       </c>
       <c r="G47" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="H47" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B48" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
+      </c>
+      <c r="D48" t="s">
+        <v>188</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>187</v>
       </c>
       <c r="F48" s="2">
         <v>0</v>
       </c>
       <c r="G48" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="H48" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B49" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
+      </c>
+      <c r="D49" t="s">
+        <v>188</v>
+      </c>
+      <c r="E49" s="5" t="s">
+        <v>187</v>
       </c>
       <c r="F49" s="2">
         <v>0</v>
       </c>
       <c r="H49" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B50" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
+      </c>
+      <c r="D50" t="s">
+        <v>188</v>
+      </c>
+      <c r="E50" s="5" t="s">
+        <v>187</v>
       </c>
       <c r="F50" s="2">
         <v>0</v>
       </c>
       <c r="G50" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="H50" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B51" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
+      </c>
+      <c r="D51" t="s">
+        <v>188</v>
+      </c>
+      <c r="E51" s="5" t="s">
+        <v>187</v>
       </c>
       <c r="F51" s="2">
         <v>0</v>
       </c>
       <c r="H51" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B52" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
+      </c>
+      <c r="D52" t="s">
+        <v>188</v>
+      </c>
+      <c r="E52" s="5" t="s">
+        <v>187</v>
       </c>
       <c r="F52" s="2">
         <v>0</v>
       </c>
       <c r="G52" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="H52" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Excel modificado con fotos y más info
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/momuychayis/Documents/Python courses/Ventas_casa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC789695-E72C-BD4C-8AA8-9A6900C770A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C0EE6D0-0C20-C847-8A36-C6B7E0C66429}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2940" yWindow="600" windowWidth="24460" windowHeight="15880" xr2:uid="{CD00CDD9-C0C8-D147-B0FC-6E5A64DE4059}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{CD00CDD9-C0C8-D147-B0FC-6E5A64DE4059}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="219">
   <si>
     <t>Nombre</t>
   </si>
@@ -97,9 +97,6 @@
     <t>TF-2006-R</t>
   </si>
   <si>
-    <t>3 velocidades -viene con control</t>
-  </si>
-  <si>
     <t>No aplica</t>
   </si>
   <si>
@@ -296,9 +293,6 @@
   </si>
   <si>
     <t>Secadora 20kg</t>
-  </si>
-  <si>
-    <t>Lavadora frontal 20kg</t>
   </si>
   <si>
     <t>Cruiser</t>
@@ -366,12 +360,6 @@
 Mide 170cm de alto x 80cm de ancho x 31cm de profundidad.</t>
   </si>
   <si>
-    <t xml:space="preserve">Mide </t>
-  </si>
-  <si>
-    <t>Coqueta de cmuy buena madera, originalmente comprada en Sarchí. Lo pintamos hace algunos años para cambiarle el estilo.</t>
-  </si>
-  <si>
     <t>Bancos miden 30x30x77cm de alto</t>
   </si>
   <si>
@@ -498,27 +486,9 @@
     <t>Raqueta mata bichos</t>
   </si>
   <si>
-    <t>Esta en perfecto estado, solo tiene muchos años de uso constante</t>
-  </si>
-  <si>
-    <t>Practicamente nuevo</t>
-  </si>
-  <si>
-    <t>El portaretratos gira, pero se le quebró el vidriecito de uno de los lados</t>
-  </si>
-  <si>
     <t>Portaretratos</t>
   </si>
   <si>
-    <t>Es la mesa que hemos tenido por años. La parte blanca es un papel de contacto que tiene casi desde nueva. Se puede quitar sin ningún problema. Solemos usar las sillas con los cobertores que nos hizo mi mamá, pero en alguna de las mudanzas desapareció el 4to cobertor</t>
-  </si>
-  <si>
-    <t>Era un mueble que habíamos comprado en pequeño mundo o walmart. Es muy útil como alacena o simplemente almacenamiento de chunches.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ideal para picar el chile, cebolla y ajo para el arroz </t>
-  </si>
-  <si>
     <t>Multistrada 950 2017</t>
   </si>
   <si>
@@ -534,88 +504,250 @@
     <t>Ducati</t>
   </si>
   <si>
-    <t>Bicicleta de montaña</t>
-  </si>
-  <si>
-    <t>Bicicleta de montaña talla S</t>
-  </si>
-  <si>
     <t>Scot</t>
   </si>
   <si>
-    <t>Tiene muy poco uso. Se venden con mantenimiento hecho por un ciclo.</t>
+    <t xml:space="preserve">Cama king + colchon </t>
+  </si>
+  <si>
+    <t>Innomuebles</t>
+  </si>
+  <si>
+    <t>Linda y amplica cama con luces a cada lado del respaldar. 
+El colchón es marca jirón. Sigue en buen estado excepto por rasguños en algunos bordes gracias a los michis -.-</t>
+  </si>
+  <si>
+    <t>Cama individual con múltiples compartimentos. La cama está hecha de melamina y tiene un colchón confortable.
+Casi no se usa pues es el del cuarto de visitas.
+Mide approx. 110x218cmx112cm</t>
+  </si>
+  <si>
+    <t>Ventilador con niebla de agua</t>
+  </si>
+  <si>
+    <t>Tiene rueditas, control remoto y se le puede añadir agua para crear una niebla fresca.</t>
+  </si>
+  <si>
+    <t>Basic Living</t>
+  </si>
+  <si>
+    <t>Ventilador de pie</t>
+  </si>
+  <si>
+    <t>DSF-1809B</t>
+  </si>
+  <si>
+    <t>Escritorio de vidrio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Altura fija, mide 110cmx70cm x 75cm de alto. </t>
+  </si>
+  <si>
+    <t>Mueble con dos repisas</t>
+  </si>
+  <si>
+    <t>Mueble de melamina y metal.</t>
+  </si>
+  <si>
+    <t>Mesita de noche</t>
+  </si>
+  <si>
+    <t>Pequeñita, ideal para poner el celular y libros.</t>
+  </si>
+  <si>
+    <t>Pantalla inteligente de 50 pulgadas</t>
+  </si>
+  <si>
+    <t>50in Crystal UHD 4K CU7000 Smart TV</t>
+  </si>
+  <si>
+    <t>50in Crystal UHD 4K CU6000 Smart TV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N/A
+</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Talla M
+Tiene muy poco uso. Se venden con mantenimiento hecho por un ciclo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mountain Bike Scot Scale 980 </t>
+  </si>
+  <si>
+    <t>Mountain Bike Scot 740</t>
+  </si>
+  <si>
+    <t xml:space="preserve">740
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scale 980
+</t>
+  </si>
+  <si>
+    <t>Talla S
+Tiene muy poco uso. Se venden con mantenimiento hecho por un ciclo.</t>
+  </si>
+  <si>
+    <t>Zandona</t>
+  </si>
+  <si>
+    <t xml:space="preserve">X-treme
+</t>
+  </si>
+  <si>
+    <t>– Certificado CE EN 1621-1. NIVEL DE PROTECCION 2
+– Doble articulación para máxima libertad de movimiento.
+– Compuesto por una estructura externa deformable que  disipa el impacto y esta hecha de un compuesto plástico ligero.
+– Acolchado interior suave y confortable.
+– Perfecta estabilidad.
+– La articulación alcanza unos 90 °, lo que permite un cómodo movimiento de la pierna.
+– Hecho en Italia.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-Kiometraje: 108000km
+-Techo panorámico
+-AWD
+-Automático
+-Asientos impecables (siempre cubiertos para evitar daños)
+-Marchamo incluido, traspaso corre por cuenta del comprador.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-Kilometraje: 56000km
+Incluye:
+1. Pantalla inteligente Chigee AIO-5 lite
+2. Cámara trasera y delantera
+3. Medidor de presión de llantas
+4. Defensas SW-Motech
+5. Tank bag marca Ducati
+6. Baúl Ducati (problema de cierre, usa un candado :) )
+7.Marchamo incluido, traspaso corre por cuenta del comprador.
+</t>
+  </si>
+  <si>
+    <t>Coqueta de muy buena madera, originalmente comprada en Sarchí. Lo pintamos hace algunos años para cambiarle el estilo.</t>
+  </si>
+  <si>
+    <t>Batido con tazon y dos aspas, se ha usado una vez :)</t>
+  </si>
+  <si>
+    <t>Venddo</t>
+  </si>
+  <si>
+    <t>https://store.steelcase.com/seating/office-chairs/steelcase-series-1</t>
+  </si>
+  <si>
+    <t>Silla ergónomica de excelente calidad.
+En excelentes condiciones, solo una pequeña mancha en el asiento</t>
+  </si>
+  <si>
+    <t>Lavadora carga frontal 20kg</t>
+  </si>
+  <si>
+    <t>Mide 68cm ancho x 100cm de profundida x 77cm de alto.
+Excelente para lavar todo tipo de telas.
+Ciclos incluidos son normal, alergénico, esterilizar, ropa de cama, carga pesada, vapor, lavado rápido, delicados, planchado permante y enjuagar/centtrifugar.</t>
+  </si>
+  <si>
+    <t>Mide 68cm ancho x 100cm de profundida x 77cm de alto
+Ciclos incluyen esterilizar, delicados, planchado permanente, ropa de cama, normal, carga pesada, secado rápido, tiempo de secado, atemperar, antiarrugas.
+Incluye un accesorio para poder secar las tenis sin que giren con el tambor.</t>
+  </si>
+  <si>
+    <t>Gratis</t>
+  </si>
+  <si>
+    <t>Gratis
+3 velocidades -viene con control</t>
+  </si>
+  <si>
+    <t>Gratis
+Esta en perfecto estado, solo tiene muchos años de uso constante</t>
+  </si>
+  <si>
+    <t>Gratis
+Practicamente nuevo</t>
+  </si>
+  <si>
+    <t>Gratis
+El portaretratos gira, pero se le quebró el vidriecito de uno de los lados</t>
+  </si>
+  <si>
+    <t>Gratis
+Es la mesa que hemos tenido por años. La parte blanca es un papel de contacto que tiene casi desde nueva. Se puede quitar sin ningún problema. Solemos usar las sillas con los cobertores que nos hizo mi mamá, pero en alguna de las mudanzas desapareció el 4to cobertor</t>
+  </si>
+  <si>
+    <t>Gratis
+Era un mueble que habíamos comprado en pequeño mundo o walmart. Es muy útil como alacena o simplemente almacenamiento de chunches.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gratis
+Ideal para picar el chile, cebolla y ajo para el arroz </t>
+  </si>
+  <si>
+    <t>Black and Decker</t>
+  </si>
+  <si>
+    <t>Parrilla de gas</t>
+  </si>
+  <si>
+    <t>Incluye cilindro de gas
+4 quemadores 
+Térmometro incorporado en la tapa
+Mesas lateriales
+Con ruedas para moverlo fácilmente</t>
+  </si>
+  <si>
+    <t>Expert Grill</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>parrilla1.jpeg, parrilla2.jpeg, parrilla3.jpeg, parrilla4.jpeg</t>
+  </si>
+  <si>
+    <t>Alimentador automático para gatos o perros pequeños</t>
+  </si>
+  <si>
+    <t>Incluye cámara y micrófono, se puede controlar por aplicación mediante conexión wifi.</t>
+  </si>
+  <si>
+    <t>NHA-PC10</t>
+  </si>
+  <si>
+    <t>alimentador1.jpeg, alimentador2.jpeg</t>
+  </si>
+  <si>
+    <t>pantallaArriba1.jpeg, pantallaArriba2.jpeg, pantallaArriba3.jpeg</t>
+  </si>
+  <si>
+    <t>MuebleRepisas.jpeg</t>
+  </si>
+  <si>
+    <t>MesitaNoche.jpeg</t>
+  </si>
+  <si>
+    <t>CoquetaOrig.jpeg</t>
+  </si>
+  <si>
+    <t>monstra1.jpeg,monstra2.jpeg,monstra3.jpeg,monstra4.jpeg,monstra5.jpeg</t>
+  </si>
+  <si>
+    <t>vespa1.jpeg,vespa2.jpeg,vespa3.jpeg, vespa4.jpeg, vespa5.jpeg, vespaAccesories.jpeg</t>
   </si>
   <si>
     <t xml:space="preserve">Poco kilómetraje (3200KM)
 Ha tenido la revisión de los 1000KM y la segunda revisión por tiempo (cambio de aceite, revisión de discos de freno y  revisión general). Ambos hechos en la agencia.
 Encendido con llave por proximidad, pantalla y conexión a bluetooth con el teléfono a través de la aplicación de Vespa.
-Completamente equipada con racks delantero y trasero, baúl, parabrisas, defensas traseras, puños y alfombra, las cuales suman alrededor de 2000 doláres.
+Completamente equipada con racks delantero y trasero, baúl, parabrisas, defensas traseras, puños y alfombra.
 Marchamo incluido, traspaso corre por cuenta del comprador.
 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cama king + colchon </t>
-  </si>
-  <si>
-    <t>Innomuebles</t>
-  </si>
-  <si>
-    <t>Linda y amplica cama con luces a cada lado del respaldar. 
-El colchón es marca jirón. Sigue en buen estado excepto por rasguños en algunos bordes gracias a los michis -.-</t>
-  </si>
-  <si>
-    <t>Cama individual con múltiples compartimentos. La cama está hecha de melamina y tiene un colchón confortable.
-Casi no se usa pues es el del cuarto de visitas.
-Mide approx. 110x218cmx112cm</t>
-  </si>
-  <si>
-    <t>Ventilador con niebla de agua</t>
-  </si>
-  <si>
-    <t>Tiene rueditas, control remoto y se le puede añadir agua para crear una niebla fresca.</t>
-  </si>
-  <si>
-    <t>Basic Living</t>
-  </si>
-  <si>
-    <t>Ventilador de pie</t>
-  </si>
-  <si>
-    <t>DSF-1809B</t>
-  </si>
-  <si>
-    <t>Escritorio de vidrio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Altura fija, mide 110cmx70cm x 75cm de alto. </t>
-  </si>
-  <si>
-    <t>Mueble con dos repisas</t>
-  </si>
-  <si>
-    <t>Mueble de melamina y metal.</t>
-  </si>
-  <si>
-    <t>Mesita de noche</t>
-  </si>
-  <si>
-    <t>Pequeñita, ideal para poner el celular y libros.</t>
-  </si>
-  <si>
-    <t>Pantalla inteligente de 50 pulgadas</t>
-  </si>
-  <si>
-    <t>50in Crystal UHD 4K CU7000 Smart TV</t>
-  </si>
-  <si>
-    <t>50in Crystal UHD 4K CU6000 Smart TV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N/A
-</t>
-  </si>
-  <si>
-    <t>N/A</t>
   </si>
 </sst>
 </file>
@@ -678,7 +810,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -688,6 +820,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1003,10 +1138,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60AABAA7-0A6C-104B-82C9-83D30D50B2A2}">
-  <dimension ref="A1:J52"/>
+  <dimension ref="A1:J54"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="32.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="39.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="23.6640625" bestFit="1" customWidth="1"/>
@@ -1022,7 +1157,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C1" t="s">
         <v>12</v>
@@ -1049,9 +1184,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="356" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B2" t="s">
         <v>7</v>
@@ -1060,21 +1195,24 @@
         <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="F2" s="2">
-        <v>25000</v>
+        <v>40000</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>183</v>
       </c>
       <c r="H2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
@@ -1083,27 +1221,27 @@
         <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E3" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F3" s="2">
         <v>25000</v>
       </c>
       <c r="G3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="H3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J3" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="306" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="289" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="B4" t="s">
         <v>7</v>
@@ -1112,24 +1250,27 @@
         <v>13</v>
       </c>
       <c r="D4" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="E4" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="F4" s="2">
         <v>4000000</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>168</v>
+        <v>218</v>
+      </c>
+      <c r="H4" t="s">
+        <v>217</v>
       </c>
       <c r="J4" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="221" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="B5" t="s">
         <v>7</v>
@@ -1138,7 +1279,7 @@
         <v>13</v>
       </c>
       <c r="D5" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
       <c r="E5" t="s">
         <v>6</v>
@@ -1146,11 +1287,16 @@
       <c r="F5" s="2">
         <v>3500000</v>
       </c>
-      <c r="G5" s="5"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="G5" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="H5" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="153" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="B6" t="s">
         <v>7</v>
@@ -1159,19 +1305,21 @@
         <v>13</v>
       </c>
       <c r="D6" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="E6" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
       <c r="F6" s="2">
         <v>8300000</v>
       </c>
-      <c r="G6" s="5"/>
+      <c r="G6" s="7" t="s">
+        <v>184</v>
+      </c>
     </row>
     <row r="7" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>184</v>
+        <v>170</v>
       </c>
       <c r="B7" t="s">
         <v>10</v>
@@ -1183,7 +1331,7 @@
         <v>17</v>
       </c>
       <c r="E7" t="s">
-        <v>185</v>
+        <v>171</v>
       </c>
       <c r="F7" s="2">
         <v>140000</v>
@@ -1191,13 +1339,16 @@
       <c r="G7" s="5" t="s">
         <v>11</v>
       </c>
+      <c r="H7" t="s">
+        <v>212</v>
+      </c>
       <c r="J7" s="3" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>184</v>
+        <v>170</v>
       </c>
       <c r="B8" t="s">
         <v>10</v>
@@ -1209,7 +1360,7 @@
         <v>17</v>
       </c>
       <c r="E8" t="s">
-        <v>186</v>
+        <v>172</v>
       </c>
       <c r="F8" s="2">
         <v>120000</v>
@@ -1218,12 +1369,12 @@
         <v>11</v>
       </c>
       <c r="H8" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="B9" t="s">
         <v>7</v>
@@ -1232,22 +1383,22 @@
         <v>13</v>
       </c>
       <c r="D9" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="F9" s="2">
-        <v>170000</v>
+        <v>220000</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="J9" s="3"/>
     </row>
-    <row r="10" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="B10" t="s">
         <v>7</v>
@@ -1256,16 +1407,16 @@
         <v>13</v>
       </c>
       <c r="D10" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="F10" s="2">
-        <v>130000</v>
+        <v>180000</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="J10" s="3"/>
     </row>
@@ -1274,56 +1425,56 @@
         <v>14</v>
       </c>
       <c r="B11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F11" s="2">
         <v>80000</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="37" customHeight="1" x14ac:dyDescent="0.2">
+        <v>186</v>
+      </c>
+      <c r="H11" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="102" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>26</v>
+        <v>203</v>
       </c>
       <c r="B12" t="s">
-        <v>10</v>
+        <v>130</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D12" t="s">
+        <v>205</v>
+      </c>
+      <c r="E12" t="s">
+        <v>206</v>
+      </c>
+      <c r="F12" s="2">
+        <v>60000</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="H12" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="37" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>25</v>
-      </c>
-      <c r="E12" t="s">
-        <v>27</v>
-      </c>
-      <c r="F12" s="2">
-        <v>30000</v>
-      </c>
-      <c r="G12" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="H12" t="s">
-        <v>45</v>
-      </c>
-      <c r="J12" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>176</v>
       </c>
       <c r="B13" t="s">
         <v>10</v>
@@ -1332,21 +1483,27 @@
         <v>13</v>
       </c>
       <c r="D13" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E13" t="s">
-        <v>177</v>
+        <v>26</v>
       </c>
       <c r="F13" s="2">
-        <v>15000</v>
+        <v>30000</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>27</v>
       </c>
       <c r="H13" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="51" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+      <c r="J13" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>173</v>
+        <v>162</v>
       </c>
       <c r="B14" t="s">
         <v>10</v>
@@ -1355,298 +1512,310 @@
         <v>13</v>
       </c>
       <c r="D14" t="s">
-        <v>175</v>
+        <v>18</v>
       </c>
       <c r="E14" t="s">
-        <v>107</v>
+        <v>163</v>
       </c>
       <c r="F14" s="2">
+        <v>15000</v>
+      </c>
+      <c r="H14" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="51" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>159</v>
+      </c>
+      <c r="B15" t="s">
+        <v>10</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" t="s">
+        <v>161</v>
+      </c>
+      <c r="E15" t="s">
+        <v>105</v>
+      </c>
+      <c r="F15" s="2">
         <v>40000</v>
       </c>
-      <c r="G14" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="H14" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="34" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>71</v>
-      </c>
-      <c r="B15" t="s">
-        <v>72</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>188</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="F15" s="2">
-        <v>45000</v>
-      </c>
       <c r="G15" s="5" t="s">
-        <v>111</v>
+        <v>160</v>
       </c>
       <c r="H15" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>70</v>
+      </c>
+      <c r="B16" t="s">
+        <v>71</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="F16" s="2">
+        <v>45000</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="H16" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>72</v>
+      </c>
+      <c r="B17" t="s">
+        <v>68</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" t="s">
+        <v>18</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="F17" s="2">
+        <v>10000</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="H17" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="119" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>77</v>
+      </c>
+      <c r="B18" t="s">
+        <v>71</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" t="s">
+        <v>174</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="F18" s="2">
+        <v>100000</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="H18" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="102" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>155</v>
+      </c>
+      <c r="B19" t="s">
+        <v>71</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" t="s">
+        <v>156</v>
+      </c>
+      <c r="E19" t="s">
+        <v>20</v>
+      </c>
+      <c r="F19" s="2">
+        <v>120000</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
         <v>73</v>
       </c>
-      <c r="B16" t="s">
-        <v>69</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D16" t="s">
-        <v>18</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="F16" s="2">
-        <v>10000</v>
-      </c>
-      <c r="H16" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="119" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+      <c r="B20" t="s">
+        <v>10</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" t="s">
+        <v>74</v>
+      </c>
+      <c r="E20" t="s">
+        <v>86</v>
+      </c>
+      <c r="F20" s="2">
+        <v>30000</v>
+      </c>
+      <c r="G20" t="s">
+        <v>108</v>
+      </c>
+      <c r="H20" t="s">
+        <v>34</v>
+      </c>
+      <c r="J20" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>75</v>
+      </c>
+      <c r="B21" t="s">
+        <v>68</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D21" t="s">
+        <v>76</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="F21" s="2">
+        <v>50000</v>
+      </c>
+      <c r="G21" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="H21" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>164</v>
+      </c>
+      <c r="B22" t="s">
+        <v>71</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D22" t="s">
+        <v>161</v>
+      </c>
+      <c r="E22" t="s">
+        <v>105</v>
+      </c>
+      <c r="F22" s="2">
+        <v>25000</v>
+      </c>
+      <c r="G22" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="68" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
         <v>78</v>
       </c>
-      <c r="B17" t="s">
-        <v>72</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D17" t="s">
-        <v>188</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="F17" s="2">
-        <v>100000</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="H17" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="102" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>169</v>
-      </c>
-      <c r="B18" t="s">
-        <v>72</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D18" t="s">
-        <v>170</v>
-      </c>
-      <c r="E18" t="s">
-        <v>21</v>
-      </c>
-      <c r="F18" s="2">
+      <c r="B23" t="s">
+        <v>71</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" t="s">
+        <v>79</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="F23" s="2">
         <v>120000</v>
       </c>
-      <c r="G18" s="5" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>74</v>
-      </c>
-      <c r="B19" t="s">
-        <v>10</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D19" t="s">
-        <v>75</v>
-      </c>
-      <c r="E19" t="s">
-        <v>88</v>
-      </c>
-      <c r="F19" s="2">
-        <v>30000</v>
-      </c>
-      <c r="G19" t="s">
-        <v>112</v>
-      </c>
-      <c r="H19" t="s">
-        <v>35</v>
-      </c>
-      <c r="J19" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="34" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>76</v>
-      </c>
-      <c r="B20" t="s">
-        <v>69</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D20" t="s">
-        <v>77</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="F20" s="2">
-        <v>50000</v>
-      </c>
-      <c r="H20" t="s">
+      <c r="G23" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="H23" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>178</v>
-      </c>
-      <c r="B21" t="s">
-        <v>72</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D21" t="s">
-        <v>175</v>
-      </c>
-      <c r="E21" t="s">
-        <v>107</v>
-      </c>
-      <c r="F21" s="2">
-        <v>25000</v>
-      </c>
-      <c r="G21" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="68" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>79</v>
-      </c>
-      <c r="B22" t="s">
-        <v>72</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D22" t="s">
-        <v>80</v>
-      </c>
-      <c r="E22" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="F22" s="2">
-        <v>120000</v>
-      </c>
-      <c r="G22" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="H22" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="34" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>94</v>
-      </c>
-      <c r="B23" t="s">
-        <v>72</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D23" t="s">
-        <v>188</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="F23" s="2">
+    <row r="24" spans="1:10" ht="68" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>92</v>
+      </c>
+      <c r="B24" t="s">
+        <v>71</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D24" t="s">
+        <v>174</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="F24" s="2">
         <v>80000</v>
       </c>
-      <c r="H23" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="34" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
-        <v>85</v>
-      </c>
-      <c r="B24" t="s">
-        <v>69</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D24" t="s">
-        <v>188</v>
-      </c>
-      <c r="E24" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="F24" s="2">
-        <v>15000</v>
-      </c>
-      <c r="G24" t="s">
-        <v>93</v>
+      <c r="G24" s="5" t="s">
+        <v>190</v>
       </c>
       <c r="H24" t="s">
-        <v>40</v>
+        <v>59</v>
+      </c>
+      <c r="J24" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B25" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D25" t="s">
-        <v>17</v>
+        <v>174</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>187</v>
+        <v>173</v>
       </c>
       <c r="F25" s="2">
-        <v>250000</v>
+        <v>15000</v>
+      </c>
+      <c r="G25" t="s">
+        <v>91</v>
       </c>
       <c r="H25" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="153" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>86</v>
+        <v>191</v>
       </c>
       <c r="B26" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>13</v>
@@ -1655,299 +1824,302 @@
         <v>17</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>187</v>
+        <v>173</v>
       </c>
       <c r="F26" s="2">
         <v>150000</v>
       </c>
-      <c r="G26" t="s">
-        <v>109</v>
+      <c r="G26" s="5" t="s">
+        <v>192</v>
       </c>
       <c r="H26" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="170" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="B27" t="s">
-        <v>10</v>
+        <v>68</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D27" t="s">
-        <v>96</v>
-      </c>
-      <c r="E27" t="s">
-        <v>97</v>
+        <v>17</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>173</v>
       </c>
       <c r="F27" s="2">
-        <v>120000</v>
-      </c>
-      <c r="G27" t="s">
-        <v>98</v>
+        <v>150000</v>
+      </c>
+      <c r="G27" s="5" t="s">
+        <v>193</v>
       </c>
       <c r="H27" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="B28" t="s">
-        <v>69</v>
+        <v>10</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D28" t="s">
-        <v>17</v>
+        <v>94</v>
       </c>
       <c r="E28" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="F28" s="2">
-        <v>60000</v>
+        <v>120000</v>
       </c>
       <c r="G28" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="H28" t="s">
-        <v>46</v>
-      </c>
-      <c r="J28" t="s">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B29" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D29" t="s">
-        <v>77</v>
+        <v>17</v>
       </c>
       <c r="E29" t="s">
-        <v>21</v>
+        <v>99</v>
       </c>
       <c r="F29" s="2">
         <v>60000</v>
       </c>
       <c r="G29" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H29" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="J29" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>180</v>
+        <v>101</v>
       </c>
       <c r="B30" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D30" t="s">
-        <v>21</v>
+        <v>76</v>
       </c>
       <c r="E30" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F30" s="2">
+        <v>60000</v>
+      </c>
+      <c r="G30" t="s">
+        <v>103</v>
+      </c>
+      <c r="H30" t="s">
+        <v>47</v>
+      </c>
+      <c r="J30" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>166</v>
+      </c>
+      <c r="B31" t="s">
+        <v>71</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D31" t="s">
+        <v>20</v>
+      </c>
+      <c r="E31" t="s">
+        <v>20</v>
+      </c>
+      <c r="F31" s="2">
         <v>25000</v>
       </c>
-      <c r="G30" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
-        <v>106</v>
-      </c>
-      <c r="B31" t="s">
-        <v>72</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D31" t="s">
-        <v>21</v>
-      </c>
-      <c r="E31" t="s">
-        <v>21</v>
-      </c>
-      <c r="F31" s="2">
-        <v>35000</v>
-      </c>
-      <c r="G31" s="5" t="s">
-        <v>108</v>
+      <c r="G31" t="s">
+        <v>167</v>
       </c>
       <c r="H31" t="s">
-        <v>55</v>
+        <v>213</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>182</v>
+        <v>104</v>
       </c>
       <c r="B32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D32" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E32" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F32" s="2">
+        <v>35000</v>
+      </c>
+      <c r="G32" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="H32" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>168</v>
+      </c>
+      <c r="B33" t="s">
+        <v>71</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D33" t="s">
+        <v>20</v>
+      </c>
+      <c r="E33" t="s">
+        <v>20</v>
+      </c>
+      <c r="F33" s="2">
         <v>10000</v>
       </c>
-      <c r="G32" s="5" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" ht="119" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
-        <v>114</v>
-      </c>
-      <c r="B33" t="s">
-        <v>72</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D33" t="s">
-        <v>21</v>
-      </c>
-      <c r="E33" t="s">
-        <v>21</v>
-      </c>
-      <c r="F33" s="2">
+      <c r="G33" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="H33" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="51" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>208</v>
+      </c>
+      <c r="B34" t="s">
+        <v>10</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D34" t="s">
+        <v>24</v>
+      </c>
+      <c r="E34" t="s">
+        <v>210</v>
+      </c>
+      <c r="F34" s="2">
+        <v>40000</v>
+      </c>
+      <c r="G34" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="H34" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="119" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>110</v>
+      </c>
+      <c r="B35" t="s">
+        <v>71</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D35" t="s">
+        <v>20</v>
+      </c>
+      <c r="E35" t="s">
+        <v>20</v>
+      </c>
+      <c r="F35" s="2">
         <v>35000</v>
       </c>
-      <c r="G33" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="H33" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
+      <c r="G35" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="H35" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>116</v>
+      </c>
+      <c r="B36" t="s">
+        <v>117</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D36" t="s">
+        <v>118</v>
+      </c>
+      <c r="E36" t="s">
         <v>120</v>
       </c>
-      <c r="B34" t="s">
-        <v>121</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D34" t="s">
-        <v>122</v>
-      </c>
-      <c r="E34" t="s">
+      <c r="F36" s="2">
+        <v>20000</v>
+      </c>
+      <c r="G36" t="s">
+        <v>119</v>
+      </c>
+      <c r="H36" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
         <v>124</v>
       </c>
-      <c r="F34" s="2">
-        <v>20000</v>
-      </c>
-      <c r="G34" t="s">
-        <v>123</v>
-      </c>
-      <c r="H34" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
-        <v>128</v>
-      </c>
-      <c r="B35" t="s">
-        <v>134</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D35" t="s">
-        <v>129</v>
-      </c>
-      <c r="E35" t="s">
+      <c r="B37" t="s">
         <v>130</v>
       </c>
-      <c r="F35" s="2">
+      <c r="C37" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D37" t="s">
+        <v>125</v>
+      </c>
+      <c r="E37" t="s">
+        <v>126</v>
+      </c>
+      <c r="F37" s="2">
         <v>15000</v>
-      </c>
-      <c r="G35" t="s">
-        <v>131</v>
-      </c>
-      <c r="H35" t="s">
-        <v>63</v>
-      </c>
-      <c r="J35" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" ht="34" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
-        <v>117</v>
-      </c>
-      <c r="B36" t="s">
-        <v>69</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D36" t="s">
-        <v>119</v>
-      </c>
-      <c r="E36" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="F36" s="2">
-        <v>8000</v>
-      </c>
-      <c r="G36" t="s">
-        <v>118</v>
-      </c>
-      <c r="H36" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A37" t="s">
-        <v>125</v>
-      </c>
-      <c r="B37" t="s">
-        <v>126</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D37" t="s">
-        <v>21</v>
-      </c>
-      <c r="E37" t="s">
-        <v>21</v>
-      </c>
-      <c r="F37" s="2">
-        <v>10000</v>
       </c>
       <c r="G37" t="s">
         <v>127</v>
@@ -1955,377 +2127,447 @@
       <c r="H37" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J37" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>133</v>
+        <v>113</v>
       </c>
       <c r="B38" t="s">
-        <v>126</v>
+        <v>68</v>
       </c>
       <c r="C38" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D38" t="s">
-        <v>21</v>
-      </c>
-      <c r="E38" t="s">
-        <v>21</v>
+        <v>115</v>
+      </c>
+      <c r="E38" s="5" t="s">
+        <v>173</v>
       </c>
       <c r="F38" s="2">
-        <v>4000</v>
+        <v>8000</v>
       </c>
       <c r="G38" t="s">
-        <v>135</v>
+        <v>114</v>
       </c>
       <c r="H38" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>136</v>
+        <v>121</v>
       </c>
       <c r="B39" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D39" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E39" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F39" s="2">
+        <v>4000</v>
+      </c>
+      <c r="G39" t="s">
+        <v>123</v>
+      </c>
+      <c r="H39" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>129</v>
+      </c>
+      <c r="B40" t="s">
+        <v>122</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D40" t="s">
+        <v>20</v>
+      </c>
+      <c r="E40" t="s">
+        <v>20</v>
+      </c>
+      <c r="F40" s="2">
+        <v>4000</v>
+      </c>
+      <c r="G40" t="s">
+        <v>131</v>
+      </c>
+      <c r="H40" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>132</v>
+      </c>
+      <c r="B41" t="s">
+        <v>122</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D41" t="s">
+        <v>20</v>
+      </c>
+      <c r="E41" t="s">
+        <v>20</v>
+      </c>
+      <c r="F41" s="2">
         <v>2000</v>
       </c>
-      <c r="G39" t="s">
-        <v>137</v>
-      </c>
-      <c r="H39" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" ht="34" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
-        <v>149</v>
-      </c>
-      <c r="B40" t="s">
-        <v>69</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D40" t="s">
-        <v>188</v>
-      </c>
-      <c r="E40" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="F40" s="2">
-        <v>10000</v>
-      </c>
-      <c r="G40" t="s">
-        <v>148</v>
-      </c>
-      <c r="H40" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" ht="34" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
-        <v>150</v>
-      </c>
-      <c r="B41" t="s">
-        <v>134</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D41" t="s">
-        <v>188</v>
-      </c>
-      <c r="E41" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="F41" s="2">
-        <v>0</v>
+      <c r="G41" t="s">
+        <v>133</v>
       </c>
       <c r="H41" t="s">
-        <v>42</v>
+        <v>65</v>
       </c>
     </row>
     <row r="42" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="B42" t="s">
-        <v>134</v>
+        <v>68</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D42" t="s">
-        <v>188</v>
+        <v>174</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>187</v>
+        <v>173</v>
       </c>
       <c r="F42" s="2">
-        <v>0</v>
+        <v>10000</v>
+      </c>
+      <c r="G42" t="s">
+        <v>144</v>
       </c>
       <c r="H42" t="s">
-        <v>43</v>
+        <v>66</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>70</v>
+        <v>146</v>
       </c>
       <c r="B43" t="s">
-        <v>69</v>
+        <v>130</v>
       </c>
       <c r="C43" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D43" t="s">
-        <v>18</v>
+        <v>174</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>187</v>
+        <v>173</v>
       </c>
       <c r="F43" s="2">
         <v>0</v>
       </c>
+      <c r="G43" t="s">
+        <v>194</v>
+      </c>
       <c r="H43" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>15</v>
+        <v>147</v>
       </c>
       <c r="B44" t="s">
-        <v>10</v>
+        <v>130</v>
       </c>
       <c r="C44" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D44" t="s">
-        <v>18</v>
-      </c>
-      <c r="E44" t="s">
-        <v>19</v>
+        <v>174</v>
+      </c>
+      <c r="E44" s="5" t="s">
+        <v>173</v>
       </c>
       <c r="F44" s="2">
         <v>0</v>
       </c>
-      <c r="G44" s="5" t="s">
-        <v>20</v>
+      <c r="G44" t="s">
+        <v>194</v>
+      </c>
+      <c r="H44" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="45" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="B45" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C45" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D45" t="s">
-        <v>82</v>
+        <v>18</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>187</v>
+        <v>173</v>
       </c>
       <c r="F45" s="2">
         <v>0</v>
       </c>
       <c r="G45" t="s">
-        <v>152</v>
+        <v>194</v>
       </c>
       <c r="H45" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
     </row>
     <row r="46" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>142</v>
+        <v>15</v>
       </c>
       <c r="B46" t="s">
-        <v>121</v>
+        <v>10</v>
       </c>
       <c r="C46" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D46" t="s">
-        <v>188</v>
-      </c>
-      <c r="E46" s="5" t="s">
-        <v>187</v>
+        <v>18</v>
+      </c>
+      <c r="E46" t="s">
+        <v>19</v>
       </c>
       <c r="F46" s="2">
         <v>0</v>
       </c>
-      <c r="G46" t="s">
-        <v>153</v>
-      </c>
-      <c r="H46" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="G46" s="5" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>155</v>
+        <v>80</v>
       </c>
       <c r="B47" t="s">
-        <v>134</v>
+        <v>68</v>
       </c>
       <c r="C47" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D47" t="s">
-        <v>188</v>
+        <v>81</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>187</v>
+        <v>173</v>
       </c>
       <c r="F47" s="2">
         <v>0</v>
       </c>
-      <c r="G47" t="s">
-        <v>154</v>
+      <c r="G47" s="5" t="s">
+        <v>196</v>
       </c>
       <c r="H47" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
     </row>
     <row r="48" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="B48" t="s">
-        <v>72</v>
+        <v>117</v>
       </c>
       <c r="C48" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D48" t="s">
-        <v>188</v>
+        <v>174</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>187</v>
+        <v>173</v>
       </c>
       <c r="F48" s="2">
         <v>0</v>
       </c>
-      <c r="G48" t="s">
-        <v>156</v>
+      <c r="G48" s="5" t="s">
+        <v>197</v>
       </c>
       <c r="H48" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" ht="68" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="B49" t="s">
-        <v>10</v>
+        <v>130</v>
       </c>
       <c r="C49" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D49" t="s">
-        <v>188</v>
+        <v>174</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>187</v>
+        <v>173</v>
       </c>
       <c r="F49" s="2">
         <v>0</v>
       </c>
+      <c r="G49" s="5" t="s">
+        <v>198</v>
+      </c>
       <c r="H49" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" ht="170" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="B50" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C50" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D50" t="s">
-        <v>188</v>
+        <v>174</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>187</v>
+        <v>173</v>
       </c>
       <c r="F50" s="2">
         <v>0</v>
       </c>
-      <c r="G50" t="s">
-        <v>157</v>
+      <c r="G50" s="5" t="s">
+        <v>199</v>
       </c>
       <c r="H50" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="B51" t="s">
-        <v>126</v>
+        <v>10</v>
       </c>
       <c r="C51" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D51" t="s">
-        <v>188</v>
+        <v>174</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>187</v>
+        <v>173</v>
       </c>
       <c r="F51" s="2">
         <v>0</v>
       </c>
+      <c r="G51" s="5" t="s">
+        <v>194</v>
+      </c>
       <c r="H51" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" ht="102" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="B52" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C52" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D52" t="s">
-        <v>188</v>
+        <v>174</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>187</v>
+        <v>173</v>
       </c>
       <c r="F52" s="2">
         <v>0</v>
       </c>
-      <c r="G52" t="s">
-        <v>158</v>
+      <c r="G52" s="5" t="s">
+        <v>200</v>
       </c>
       <c r="H52" t="s">
-        <v>53</v>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>142</v>
+      </c>
+      <c r="B53" t="s">
+        <v>122</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D53" t="s">
+        <v>174</v>
+      </c>
+      <c r="E53" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="F53" s="2">
+        <v>0</v>
+      </c>
+      <c r="G53" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="H53" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>143</v>
+      </c>
+      <c r="B54" t="s">
+        <v>68</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D54" t="s">
+        <v>202</v>
+      </c>
+      <c r="E54" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="F54" s="2">
+        <v>0</v>
+      </c>
+      <c r="G54" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="H54" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Arreglando errores y rotacion de fotos 2
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/momuychayis/Documents/Python courses/Ventas_casa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D8DB4CD-CDAB-7E45-9B5E-83D98B19E1FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0945625-1825-3347-95B9-A68E5E4AFA58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{CD00CDD9-C0C8-D147-B0FC-6E5A64DE4059}"/>
   </bookViews>
@@ -730,9 +730,6 @@
     <t>MesitaNoche.jpeg</t>
   </si>
   <si>
-    <t>CoquetaOrig.jpeg</t>
-  </si>
-  <si>
     <t>monstra1.jpeg,monstra2.jpeg,monstra3.jpeg,monstra4.jpeg,monstra5.jpeg</t>
   </si>
   <si>
@@ -748,6 +745,9 @@
   </si>
   <si>
     <t>Incluye el play4 de 500GB, manivela Trustmaster, 2 controles, 3 juegos físicos (Crash, PES2018 y Battlefront II) además de juegos descargados en la consola (Fútbol americano, Fórmula 1, Snipper Elite y Grand Turismo).</t>
+  </si>
+  <si>
+    <t>Coqueta_original.jpeg</t>
   </si>
 </sst>
 </file>
@@ -1290,10 +1290,10 @@
         <v>4000000</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2" t="s">
@@ -1323,7 +1323,7 @@
         <v>184</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
@@ -1487,7 +1487,7 @@
         <v>185</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
@@ -1960,7 +1960,7 @@
         <v>120000</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H28" s="2" t="s">
         <v>50</v>

</xml_diff>

<commit_message>
Corregir arrocera y zancudos
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/momuychayis/Documents/Python courses/Ventas_casa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F287D943-76BC-4D44-91AE-2617DF71E3A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADFE2C29-8173-AE47-9F1E-D59512C3B453}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16460" xr2:uid="{CD00CDD9-C0C8-D147-B0FC-6E5A64DE4059}"/>
+    <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16440" xr2:uid="{CD00CDD9-C0C8-D147-B0FC-6E5A64DE4059}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="223">
   <si>
     <t>Nombre</t>
   </si>
@@ -125,9 +125,6 @@
   </si>
   <si>
     <t>abanico_evapor1.jpeg,controlAbanico.jpeg</t>
-  </si>
-  <si>
-    <t>arrocera_arrriba.jpeg,arrocera_frente.jpeg</t>
   </si>
   <si>
     <t>banco2.jpeg,bancos_metal1.jpeg</t>
@@ -627,9 +624,6 @@
 </t>
   </si>
   <si>
-    <t>Coqueta de muy buena madera, originalmente comprada en Sarchí. Lo pintamos hace algunos años para cambiarle el estilo.</t>
-  </si>
-  <si>
     <t>Batido con tazon y dos aspas, se ha usado una vez :)</t>
   </si>
   <si>
@@ -748,6 +742,25 @@
   </si>
   <si>
     <t>Coqueta_original.jpeg</t>
+  </si>
+  <si>
+    <t>Nuevo dueño</t>
+  </si>
+  <si>
+    <t>Tefy</t>
+  </si>
+  <si>
+    <t>Precio final</t>
+  </si>
+  <si>
+    <t>con licuadora</t>
+  </si>
+  <si>
+    <t>arrocera_frente.jpeg,arrocera_arrriba.jpeg</t>
+  </si>
+  <si>
+    <t>Coqueta de muy buena madera, originalmente comprada en Sarchí. Lo pintamos hace algunos años para cambiarle el estilo.
+La foto muestra la coqueta original, la nueva es azul marino (foto pendiente)</t>
   </si>
 </sst>
 </file>
@@ -797,7 +810,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -820,12 +833,36 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -842,15 +879,26 @@
     <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1166,21 +1214,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60AABAA7-0A6C-104B-82C9-83D30D50B2A2}">
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:M54"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="39.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="32.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" customWidth="1"/>
+    <col min="3" max="3" width="9.6640625" customWidth="1"/>
+    <col min="4" max="4" width="23.6640625" customWidth="1"/>
+    <col min="5" max="5" width="32.33203125" customWidth="1"/>
     <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="31.1640625" customWidth="1"/>
-    <col min="8" max="8" width="76" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31.1640625" style="13" customWidth="1"/>
+    <col min="8" max="8" width="76" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" style="12" customWidth="1"/>
+    <col min="10" max="10" width="10.83203125" style="12" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1202,7 +1252,7 @@
       <c r="G1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="9" t="s">
         <v>4</v>
       </c>
       <c r="I1" s="1" t="s">
@@ -1211,10 +1261,16 @@
       <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" ht="356" x14ac:dyDescent="0.2">
+      <c r="K1" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>7</v>
@@ -1223,26 +1279,26 @@
         <v>13</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="E2" s="4" t="s">
         <v>180</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>181</v>
       </c>
       <c r="F2" s="5">
         <v>40000</v>
       </c>
-      <c r="G2" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>55</v>
+      <c r="G2" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>54</v>
       </c>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>7</v>
@@ -1251,28 +1307,28 @@
         <v>13</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F3" s="5">
         <v>25000</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>38</v>
+        <v>88</v>
+      </c>
+      <c r="H3" s="10" t="s">
+        <v>37</v>
       </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="289" x14ac:dyDescent="0.2">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>7</v>
@@ -1281,28 +1337,28 @@
         <v>13</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>134</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>135</v>
       </c>
       <c r="F4" s="5">
         <v>4000000</v>
       </c>
-      <c r="G4" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>215</v>
+      <c r="G4" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>213</v>
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="221" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>7</v>
@@ -1311,7 +1367,7 @@
         <v>13</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>6</v>
@@ -1319,18 +1375,18 @@
       <c r="F5" s="5">
         <v>3500000</v>
       </c>
-      <c r="G5" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>214</v>
+      <c r="G5" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>212</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
     </row>
-    <row r="6" spans="1:10" ht="153" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>7</v>
@@ -1339,24 +1395,24 @@
         <v>13</v>
       </c>
       <c r="D6" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>150</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>151</v>
       </c>
       <c r="F6" s="5">
         <v>8300000</v>
       </c>
-      <c r="G6" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="H6" s="2"/>
+      <c r="G6" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="H6" s="10"/>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
     </row>
-    <row r="7" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>10</v>
@@ -1368,25 +1424,25 @@
         <v>17</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F7" s="5">
         <v>140000</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H7" s="2" t="s">
-        <v>211</v>
+      <c r="H7" s="10" t="s">
+        <v>209</v>
       </c>
       <c r="I7" s="2"/>
-      <c r="J7" s="7" t="s">
+      <c r="J7" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>10</v>
@@ -1398,23 +1454,23 @@
         <v>17</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F8" s="5">
         <v>120000</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H8" s="2" t="s">
-        <v>48</v>
+      <c r="H8" s="10" t="s">
+        <v>47</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
     </row>
-    <row r="9" spans="1:10" ht="51" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>7</v>
@@ -1423,24 +1479,24 @@
         <v>13</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F9" s="5">
         <v>220000</v>
       </c>
-      <c r="G9" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="H9" s="2"/>
+      <c r="G9" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="H9" s="10"/>
       <c r="I9" s="2"/>
-      <c r="J9" s="7"/>
-    </row>
-    <row r="10" spans="1:10" ht="51" x14ac:dyDescent="0.2">
+      <c r="J9" s="6"/>
+    </row>
+    <row r="10" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>7</v>
@@ -1449,33 +1505,33 @@
         <v>13</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F10" s="5">
         <v>180000</v>
       </c>
-      <c r="G10" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="H10" s="2"/>
+      <c r="G10" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="H10" s="10"/>
       <c r="I10" s="2"/>
-      <c r="J10" s="7"/>
-    </row>
-    <row r="11" spans="1:10" ht="68" x14ac:dyDescent="0.2">
+      <c r="J10" s="6"/>
+    </row>
+    <row r="11" spans="1:12" ht="119" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>14</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>20</v>
@@ -1484,43 +1540,49 @@
         <v>80000</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>218</v>
+        <v>222</v>
+      </c>
+      <c r="H11" s="10" t="s">
+        <v>216</v>
       </c>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
     </row>
-    <row r="12" spans="1:10" ht="102" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="F12" s="5">
         <v>60000</v>
       </c>
-      <c r="G12" s="4" t="s">
-        <v>203</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>206</v>
+      <c r="G12" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="H12" s="10" t="s">
+        <v>204</v>
       </c>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
-    </row>
-    <row r="13" spans="1:10" ht="37" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K12" t="s">
+        <v>218</v>
+      </c>
+      <c r="L12">
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>25</v>
       </c>
@@ -1539,20 +1601,20 @@
       <c r="F13" s="5">
         <v>30000</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="G13" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H13" s="2" t="s">
-        <v>44</v>
+      <c r="H13" s="10" t="s">
+        <v>43</v>
       </c>
       <c r="I13" s="2"/>
       <c r="J13" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>10</v>
@@ -1564,21 +1626,21 @@
         <v>18</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F14" s="5">
         <v>15000</v>
       </c>
       <c r="G14" s="2"/>
-      <c r="H14" s="2" t="s">
+      <c r="H14" s="10" t="s">
         <v>28</v>
       </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
     </row>
-    <row r="15" spans="1:10" ht="51" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>10</v>
@@ -1587,57 +1649,57 @@
         <v>13</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F15" s="5">
         <v>40000</v>
       </c>
-      <c r="G15" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="H15" s="2" t="s">
+      <c r="G15" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="H15" s="10" t="s">
         <v>29</v>
       </c>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
     </row>
-    <row r="16" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>71</v>
-      </c>
       <c r="C16" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D16" s="8" t="s">
-        <v>173</v>
+      <c r="D16" s="7" t="s">
+        <v>172</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F16" s="5">
         <v>45000</v>
       </c>
-      <c r="G16" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>31</v>
+      <c r="G16" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="H16" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
     </row>
-    <row r="17" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>13</v>
@@ -1646,60 +1708,60 @@
         <v>18</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F17" s="5">
         <v>10000</v>
       </c>
-      <c r="G17" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>32</v>
+      <c r="G17" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="H17" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
     </row>
-    <row r="18" spans="1:10" ht="119" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F18" s="5">
         <v>100000</v>
       </c>
-      <c r="G18" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>33</v>
+      <c r="G18" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="H18" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
     </row>
-    <row r="19" spans="1:10" ht="102" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>154</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>155</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>20</v>
@@ -1707,16 +1769,16 @@
       <c r="F19" s="5">
         <v>120000</v>
       </c>
-      <c r="G19" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="H19" s="2"/>
+      <c r="G19" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="H19" s="10"/>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>10</v>
@@ -1725,171 +1787,186 @@
         <v>13</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F20" s="5">
         <v>30000</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>34</v>
+        <v>106</v>
+      </c>
+      <c r="H20" s="10" t="s">
+        <v>33</v>
       </c>
       <c r="I20" s="2"/>
       <c r="J20" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F21" s="5">
         <v>50000</v>
       </c>
-      <c r="G21" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>35</v>
+      <c r="G21" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="H21" s="10" t="s">
+        <v>34</v>
       </c>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K21" s="12" t="s">
+        <v>218</v>
+      </c>
+      <c r="L21">
+        <v>110000</v>
+      </c>
+      <c r="M21" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F22" s="5">
         <v>25000</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="H22" s="2"/>
+        <v>163</v>
+      </c>
+      <c r="H22" s="10"/>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
     </row>
-    <row r="23" spans="1:10" ht="68" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>79</v>
-      </c>
       <c r="E23" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F23" s="5">
         <v>120000</v>
       </c>
-      <c r="G23" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>36</v>
+      <c r="G23" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="H23" s="10" t="s">
+        <v>35</v>
       </c>
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
     </row>
-    <row r="24" spans="1:10" ht="68" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F24" s="5">
         <v>80000</v>
       </c>
-      <c r="G24" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="H24" s="2" t="s">
-        <v>59</v>
+      <c r="G24" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="H24" s="10" t="s">
+        <v>58</v>
       </c>
       <c r="I24" s="2"/>
       <c r="J24" s="2" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F25" s="5">
         <v>15000</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="H25" s="2" t="s">
-        <v>39</v>
+        <v>90</v>
+      </c>
+      <c r="H25" s="10" t="s">
+        <v>38</v>
       </c>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
-    </row>
-    <row r="26" spans="1:10" ht="153" x14ac:dyDescent="0.2">
+      <c r="K25" s="12" t="s">
+        <v>218</v>
+      </c>
+      <c r="L25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>13</v>
@@ -1898,26 +1975,26 @@
         <v>17</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F26" s="5">
         <v>150000</v>
       </c>
-      <c r="G26" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="H26" s="2" t="s">
-        <v>40</v>
+      <c r="G26" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="H26" s="10" t="s">
+        <v>39</v>
       </c>
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
     </row>
-    <row r="27" spans="1:10" ht="170" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>13</v>
@@ -1926,23 +2003,23 @@
         <v>17</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F27" s="5">
         <v>150000</v>
       </c>
-      <c r="G27" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="H27" s="2" t="s">
-        <v>57</v>
+      <c r="G27" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="H27" s="10" t="s">
+        <v>56</v>
       </c>
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>10</v>
@@ -1951,29 +2028,29 @@
         <v>13</v>
       </c>
       <c r="D28" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E28" s="2" t="s">
         <v>94</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>95</v>
       </c>
       <c r="F28" s="5">
         <v>120000</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>50</v>
+        <v>215</v>
+      </c>
+      <c r="H28" s="10" t="s">
+        <v>49</v>
       </c>
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>13</v>
@@ -1982,34 +2059,34 @@
         <v>17</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F29" s="5">
         <v>60000</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="H29" s="2" t="s">
-        <v>45</v>
+        <v>98</v>
+      </c>
+      <c r="H29" s="10" t="s">
+        <v>44</v>
       </c>
       <c r="I29" s="2"/>
       <c r="J29" s="2" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>20</v>
@@ -2018,22 +2095,25 @@
         <v>60000</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="H30" s="2" t="s">
-        <v>47</v>
+        <v>101</v>
+      </c>
+      <c r="H30" s="10" t="s">
+        <v>46</v>
       </c>
       <c r="I30" s="2"/>
       <c r="J30" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+        <v>100</v>
+      </c>
+      <c r="L30">
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>13</v>
@@ -2048,20 +2128,20 @@
         <v>25000</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="H31" s="2" t="s">
-        <v>212</v>
+        <v>165</v>
+      </c>
+      <c r="H31" s="10" t="s">
+        <v>210</v>
       </c>
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
     </row>
-    <row r="32" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:13" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>13</v>
@@ -2075,21 +2155,21 @@
       <c r="F32" s="5">
         <v>35000</v>
       </c>
-      <c r="G32" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="H32" s="2" t="s">
-        <v>54</v>
+      <c r="G32" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="H32" s="10" t="s">
+        <v>53</v>
       </c>
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
     </row>
-    <row r="33" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>13</v>
@@ -2103,18 +2183,18 @@
       <c r="F33" s="5">
         <v>10000</v>
       </c>
-      <c r="G33" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="H33" s="2" t="s">
-        <v>213</v>
+      <c r="G33" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="H33" s="10" t="s">
+        <v>211</v>
       </c>
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
     </row>
-    <row r="34" spans="1:10" ht="51" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>10</v>
@@ -2126,26 +2206,26 @@
         <v>24</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="F34" s="5">
         <v>40000</v>
       </c>
-      <c r="G34" s="4" t="s">
+      <c r="G34" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="H34" s="10" t="s">
         <v>208</v>
-      </c>
-      <c r="H34" s="2" t="s">
-        <v>210</v>
       </c>
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
     </row>
-    <row r="35" spans="1:10" ht="119" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>13</v>
@@ -2159,107 +2239,107 @@
       <c r="F35" s="5">
         <v>35000</v>
       </c>
-      <c r="G35" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="H35" s="2" t="s">
-        <v>53</v>
+      <c r="G35" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="H35" s="10" t="s">
+        <v>52</v>
       </c>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B36" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="C36" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D36" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="C36" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>117</v>
-      </c>
       <c r="E36" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F36" s="5">
         <v>20000</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="H36" s="2" t="s">
-        <v>60</v>
+        <v>117</v>
+      </c>
+      <c r="H36" s="10" t="s">
+        <v>59</v>
       </c>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
     </row>
-    <row r="37" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D37" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="B37" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="C37" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D37" s="2" t="s">
+      <c r="E37" s="2" t="s">
         <v>124</v>
-      </c>
-      <c r="E37" s="2" t="s">
-        <v>125</v>
       </c>
       <c r="F37" s="5">
         <v>15000</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="H37" s="2" t="s">
-        <v>62</v>
+        <v>125</v>
+      </c>
+      <c r="H37" s="10" t="s">
+        <v>61</v>
       </c>
       <c r="I37" s="2"/>
       <c r="J37" s="2" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F38" s="5">
         <v>8000</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="H38" s="2" t="s">
-        <v>56</v>
+        <v>112</v>
+      </c>
+      <c r="H38" s="10" t="s">
+        <v>55</v>
       </c>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B39" s="2" t="s">
         <v>120</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>121</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>13</v>
@@ -2274,20 +2354,20 @@
         <v>4000</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="H39" s="2" t="s">
-        <v>61</v>
+        <v>121</v>
+      </c>
+      <c r="H39" s="10" t="s">
+        <v>60</v>
       </c>
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C40" s="3" t="s">
         <v>13</v>
@@ -2302,20 +2382,20 @@
         <v>4000</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="H40" s="2" t="s">
-        <v>64</v>
+        <v>129</v>
+      </c>
+      <c r="H40" s="10" t="s">
+        <v>63</v>
       </c>
       <c r="I40" s="2"/>
       <c r="J40" s="2"/>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C41" s="3" t="s">
         <v>13</v>
@@ -2330,104 +2410,110 @@
         <v>2000</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="H41" s="2" t="s">
-        <v>65</v>
+        <v>131</v>
+      </c>
+      <c r="H41" s="10" t="s">
+        <v>64</v>
       </c>
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
     </row>
-    <row r="42" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F42" s="5">
         <v>10000</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="H42" s="2" t="s">
-        <v>66</v>
+        <v>142</v>
+      </c>
+      <c r="H42" s="10" t="s">
+        <v>65</v>
       </c>
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
-    </row>
-    <row r="43" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="K42" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="L42">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C43" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F43" s="5">
         <v>0</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="H43" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="H43" s="10" t="s">
         <v>41</v>
       </c>
       <c r="I43" s="2"/>
       <c r="J43" s="2"/>
     </row>
-    <row r="44" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C44" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F44" s="5">
         <v>0</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="H44" s="2" t="s">
-        <v>42</v>
+        <v>191</v>
+      </c>
+      <c r="H44" s="10" t="s">
+        <v>40</v>
       </c>
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
     </row>
-    <row r="45" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C45" s="3" t="s">
         <v>13</v>
@@ -2436,21 +2522,21 @@
         <v>18</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F45" s="5">
         <v>0</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="H45" s="2" t="s">
-        <v>30</v>
+        <v>191</v>
+      </c>
+      <c r="H45" s="10" t="s">
+        <v>221</v>
       </c>
       <c r="I45" s="2"/>
       <c r="J45" s="2"/>
     </row>
-    <row r="46" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>15</v>
       </c>
@@ -2469,128 +2555,128 @@
       <c r="F46" s="5">
         <v>0</v>
       </c>
-      <c r="G46" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="H46" s="2"/>
+      <c r="G46" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="H46" s="10"/>
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
     </row>
-    <row r="47" spans="1:10" ht="51" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D47" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="B47" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C47" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>81</v>
-      </c>
       <c r="E47" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F47" s="5">
         <v>0</v>
       </c>
-      <c r="G47" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="H47" s="2" t="s">
-        <v>37</v>
+      <c r="G47" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="H47" s="10" t="s">
+        <v>36</v>
       </c>
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
     </row>
-    <row r="48" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F48" s="5">
         <v>0</v>
       </c>
-      <c r="G48" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="H48" s="2" t="s">
-        <v>58</v>
+      <c r="G48" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="H48" s="10" t="s">
+        <v>57</v>
       </c>
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
     </row>
-    <row r="49" spans="1:10" ht="68" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C49" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F49" s="5">
         <v>0</v>
       </c>
-      <c r="G49" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="H49" s="2" t="s">
-        <v>51</v>
+      <c r="G49" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="H49" s="10" t="s">
+        <v>50</v>
       </c>
       <c r="I49" s="2"/>
       <c r="J49" s="2"/>
     </row>
-    <row r="50" spans="1:10" ht="170" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C50" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F50" s="5">
         <v>0</v>
       </c>
-      <c r="G50" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="H50" s="2" t="s">
-        <v>43</v>
+      <c r="G50" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="H50" s="10" t="s">
+        <v>42</v>
       </c>
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
     </row>
     <row r="51" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>10</v>
@@ -2599,103 +2685,103 @@
         <v>13</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F51" s="5">
         <v>0</v>
       </c>
-      <c r="G51" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="H51" s="2" t="s">
-        <v>63</v>
+      <c r="G51" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="H51" s="10" t="s">
+        <v>62</v>
       </c>
       <c r="I51" s="2"/>
       <c r="J51" s="2"/>
     </row>
-    <row r="52" spans="1:10" ht="102" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C52" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F52" s="5">
         <v>0</v>
       </c>
-      <c r="G52" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="H52" s="2" t="s">
-        <v>46</v>
+      <c r="G52" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="H52" s="10" t="s">
+        <v>45</v>
       </c>
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
     </row>
     <row r="53" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C53" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F53" s="5">
         <v>0</v>
       </c>
-      <c r="G53" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="H53" s="2" t="s">
-        <v>49</v>
+      <c r="G53" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="H53" s="10" t="s">
+        <v>48</v>
       </c>
       <c r="I53" s="2"/>
       <c r="J53" s="2"/>
     </row>
-    <row r="54" spans="1:10" ht="51" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C54" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F54" s="5">
         <v>0</v>
       </c>
-      <c r="G54" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="H54" s="2" t="s">
-        <v>52</v>
+      <c r="G54" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="H54" s="10" t="s">
+        <v>51</v>
       </c>
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>

</xml_diff>

<commit_message>
Cambio fotos de vespa y actualizar vendidos a Familia
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/momuychayis/Documents/Python courses/Ventas_casa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADFE2C29-8173-AE47-9F1E-D59512C3B453}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1961809-BA98-0743-848B-25EB10E11105}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16440" xr2:uid="{CD00CDD9-C0C8-D147-B0FC-6E5A64DE4059}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$54</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -35,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="228">
   <si>
     <t>Nombre</t>
   </si>
@@ -727,48 +730,64 @@
     <t>monstra1.jpeg,monstra2.jpeg,monstra3.jpeg,monstra4.jpeg,monstra5.jpeg</t>
   </si>
   <si>
-    <t>vespa1.jpeg,vespa2.jpeg,vespa3.jpeg, vespa4.jpeg, vespa5.jpeg, vespaAccesories.jpeg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Poco kilómetraje (3200KM)
-Ha tenido la revisión de los 1000KM y la segunda revisión por tiempo (cambio de aceite, revisión de discos de freno y  revisión general). Ambos hechos en la agencia.
+    <t>Incluye el play4 de 500GB, manivela Trustmaster, 2 controles, 3 juegos físicos (Crash, PES2018 y Battlefront II) además de juegos descargados en la consola (Fútbol americano, Fórmula 1, Snipper Elite y Grand Turismo).</t>
+  </si>
+  <si>
+    <t>Coqueta_original.jpeg</t>
+  </si>
+  <si>
+    <t>Nuevo dueño</t>
+  </si>
+  <si>
+    <t>Tefy</t>
+  </si>
+  <si>
+    <t>Precio final</t>
+  </si>
+  <si>
+    <t>con licuadora</t>
+  </si>
+  <si>
+    <t>arrocera_frente.jpeg,arrocera_arrriba.jpeg</t>
+  </si>
+  <si>
+    <t>Coqueta de muy buena madera, originalmente comprada en Sarchí. Lo pintamos hace algunos años para cambiarle el estilo.
+La foto muestra la coqueta original, la nueva es azul marino (foto pendiente)</t>
+  </si>
+  <si>
+    <t>vespa1.jpeg,vespa2.jpeg,vespa3.jpeg, vespa4.jpeg, vespa5.jpeg, vespa6.jpeg, vespa7.jpeg, vespa8.jpeg, vespaAccesories.jpeg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poco kilómetraje (approx. 3300Km)
+Ha tenido la revisión de los 1000Km y la segunda revisión por tiempo (cambio de aceite, revisión de discos de freno y  revisión general). Ambos hechos en la agencia.
 Encendido con llave por proximidad, pantalla y conexión a bluetooth con el teléfono a través de la aplicación de Vespa.
-Completamente equipada con racks delantero y trasero, baúl, parabrisas, defensas traseras, puños y alfombra.
+Completamente equipada con porta equipajes delantero y trasero, baúl con respaldar, parabrisas, defensas traseras, puños y alfombra.
 Marchamo incluido, traspaso corre por cuenta del comprador.
 </t>
   </si>
   <si>
-    <t>Incluye el play4 de 500GB, manivela Trustmaster, 2 controles, 3 juegos físicos (Crash, PES2018 y Battlefront II) además de juegos descargados en la consola (Fútbol americano, Fórmula 1, Snipper Elite y Grand Turismo).</t>
-  </si>
-  <si>
-    <t>Coqueta_original.jpeg</t>
-  </si>
-  <si>
-    <t>Nuevo dueño</t>
-  </si>
-  <si>
-    <t>Tefy</t>
-  </si>
-  <si>
-    <t>Precio final</t>
-  </si>
-  <si>
-    <t>con licuadora</t>
-  </si>
-  <si>
-    <t>arrocera_frente.jpeg,arrocera_arrriba.jpeg</t>
-  </si>
-  <si>
-    <t>Coqueta de muy buena madera, originalmente comprada en Sarchí. Lo pintamos hace algunos años para cambiarle el estilo.
-La foto muestra la coqueta original, la nueva es azul marino (foto pendiente)</t>
+    <t>Luis</t>
+  </si>
+  <si>
+    <t>Katiria</t>
+  </si>
+  <si>
+    <t>Oso</t>
+  </si>
+  <si>
+    <t>Papi</t>
+  </si>
+  <si>
+    <t>Maria</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="44" formatCode="_(&quot;₡&quot;* #,##0.00_);_(&quot;₡&quot;* \(#,##0.00\);_(&quot;₡&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="&quot;₡&quot;#,##0.00"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -810,7 +829,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -837,17 +856,6 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
       <right/>
       <top style="thin">
         <color indexed="64"/>
@@ -857,12 +865,49 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -885,20 +930,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1214,7 +1257,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60AABAA7-0A6C-104B-82C9-83D30D50B2A2}">
-  <dimension ref="A1:M54"/>
+  <dimension ref="A1:M55"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="39.6640625" bestFit="1" customWidth="1"/>
@@ -1223,11 +1266,12 @@
     <col min="4" max="4" width="23.6640625" customWidth="1"/>
     <col min="5" max="5" width="32.33203125" customWidth="1"/>
     <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="31.1640625" style="13" customWidth="1"/>
-    <col min="8" max="8" width="76" customWidth="1"/>
-    <col min="9" max="9" width="15.6640625" style="12" customWidth="1"/>
-    <col min="10" max="10" width="10.83203125" style="12" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" style="12"/>
+    <col min="7" max="7" width="31.1640625" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="26.83203125" style="9" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" style="8" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="10.83203125" style="15" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" style="17"/>
+    <col min="12" max="12" width="11.33203125" style="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">
@@ -1252,7 +1296,7 @@
       <c r="G1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="H1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="I1" s="1" t="s">
@@ -1261,11 +1305,11 @@
       <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="11" t="s">
+      <c r="K1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="L1" s="11" t="s">
         <v>217</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="34" x14ac:dyDescent="0.2">
@@ -1290,11 +1334,13 @@
       <c r="G2" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="H2" s="10" t="s">
+      <c r="H2" s="2" t="s">
         <v>54</v>
       </c>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
+      <c r="K2" s="8"/>
+      <c r="L2" s="12"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
@@ -1318,15 +1364,17 @@
       <c r="G3" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="H3" s="10" t="s">
+      <c r="H3" s="2" t="s">
         <v>37</v>
       </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="K3" s="8"/>
+      <c r="L3" s="12"/>
+    </row>
+    <row r="4" spans="1:12" ht="289" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>132</v>
       </c>
@@ -1345,16 +1393,18 @@
       <c r="F4" s="5">
         <v>4000000</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="H4" s="10" t="s">
-        <v>213</v>
+      <c r="G4" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>221</v>
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2" t="s">
         <v>135</v>
       </c>
+      <c r="K4" s="8"/>
+      <c r="L4" s="12"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
@@ -1378,11 +1428,13 @@
       <c r="G5" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="H5" s="10" t="s">
+      <c r="H5" s="2" t="s">
         <v>212</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
+      <c r="K5" s="8"/>
+      <c r="L5" s="12"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
@@ -1406,9 +1458,11 @@
       <c r="G6" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="H6" s="10"/>
+      <c r="H6" s="2"/>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="12"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -1418,7 +1472,7 @@
         <v>10</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>17</v>
@@ -1432,13 +1486,14 @@
       <c r="G7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H7" s="10" t="s">
+      <c r="H7" s="2" t="s">
         <v>209</v>
       </c>
       <c r="I7" s="2"/>
       <c r="J7" s="6" t="s">
         <v>9</v>
       </c>
+      <c r="K7" s="8"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
@@ -1448,7 +1503,7 @@
         <v>10</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>17</v>
@@ -1462,11 +1517,17 @@
       <c r="G8" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H8" s="10" t="s">
+      <c r="H8" s="2" t="s">
         <v>47</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
+      <c r="K8" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="L8" s="12">
+        <v>120000</v>
+      </c>
     </row>
     <row r="9" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
@@ -1490,9 +1551,11 @@
       <c r="G9" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="H9" s="10"/>
+      <c r="H9" s="2"/>
       <c r="I9" s="2"/>
       <c r="J9" s="6"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="12"/>
     </row>
     <row r="10" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
@@ -1516,9 +1579,11 @@
       <c r="G10" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="H10" s="10"/>
+      <c r="H10" s="2"/>
       <c r="I10" s="2"/>
       <c r="J10" s="6"/>
+      <c r="K10" s="8"/>
+      <c r="L10" s="12"/>
     </row>
     <row r="11" spans="1:12" ht="119" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
@@ -1540,13 +1605,15 @@
         <v>80000</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>222</v>
-      </c>
-      <c r="H11" s="10" t="s">
-        <v>216</v>
+        <v>220</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>214</v>
       </c>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
+      <c r="K11" s="8"/>
+      <c r="L11" s="12"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
@@ -1570,15 +1637,15 @@
       <c r="G12" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="H12" s="10" t="s">
+      <c r="H12" s="2" t="s">
         <v>204</v>
       </c>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
-      <c r="K12" t="s">
-        <v>218</v>
-      </c>
-      <c r="L12">
+      <c r="K12" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="L12" s="12">
         <v>55000</v>
       </c>
     </row>
@@ -1590,7 +1657,7 @@
         <v>10</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>24</v>
@@ -1604,13 +1671,19 @@
       <c r="G13" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H13" s="10" t="s">
+      <c r="H13" s="2" t="s">
         <v>43</v>
       </c>
       <c r="I13" s="2"/>
       <c r="J13" s="2" t="s">
         <v>23</v>
       </c>
+      <c r="K13" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="L13" s="12">
+        <v>30000</v>
+      </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
@@ -1620,7 +1693,7 @@
         <v>10</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>18</v>
@@ -1632,11 +1705,17 @@
         <v>15000</v>
       </c>
       <c r="G14" s="2"/>
-      <c r="H14" s="10" t="s">
+      <c r="H14" s="2" t="s">
         <v>28</v>
       </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
+      <c r="K14" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="L14" s="12">
+        <v>15000</v>
+      </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
@@ -1660,11 +1739,13 @@
       <c r="G15" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="H15" s="10" t="s">
+      <c r="H15" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
+      <c r="K15" s="8"/>
+      <c r="L15" s="12"/>
     </row>
     <row r="16" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
@@ -1688,11 +1769,13 @@
       <c r="G16" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="H16" s="10" t="s">
+      <c r="H16" s="2" t="s">
         <v>30</v>
       </c>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
+      <c r="K16" s="8"/>
+      <c r="L16" s="12"/>
     </row>
     <row r="17" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
@@ -1716,11 +1799,13 @@
       <c r="G17" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="H17" s="10" t="s">
+      <c r="H17" s="2" t="s">
         <v>31</v>
       </c>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
+      <c r="K17" s="8"/>
+      <c r="L17" s="12"/>
     </row>
     <row r="18" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
@@ -1744,11 +1829,13 @@
       <c r="G18" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="H18" s="10" t="s">
+      <c r="H18" s="2" t="s">
         <v>32</v>
       </c>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
+      <c r="K18" s="8"/>
+      <c r="L18" s="12"/>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
@@ -1772,9 +1859,13 @@
       <c r="G19" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="H19" s="10"/>
+      <c r="H19" s="2"/>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
+      <c r="K19" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="L19" s="12"/>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
@@ -1798,13 +1889,19 @@
       <c r="G20" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="H20" s="10" t="s">
+      <c r="H20" s="2" t="s">
         <v>33</v>
       </c>
       <c r="I20" s="2"/>
       <c r="J20" s="2" t="s">
         <v>86</v>
       </c>
+      <c r="K20" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="L20" s="12">
+        <v>30000</v>
+      </c>
     </row>
     <row r="21" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
@@ -1828,19 +1925,19 @@
       <c r="G21" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="H21" s="10" t="s">
+      <c r="H21" s="2" t="s">
         <v>34</v>
       </c>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
-      <c r="K21" s="12" t="s">
+      <c r="K21" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="L21" s="12">
+        <v>110000</v>
+      </c>
+      <c r="M21" t="s">
         <v>218</v>
-      </c>
-      <c r="L21">
-        <v>110000</v>
-      </c>
-      <c r="M21" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
@@ -1865,9 +1962,11 @@
       <c r="G22" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="H22" s="10"/>
+      <c r="H22" s="2"/>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
+      <c r="K22" s="8"/>
+      <c r="L22" s="12"/>
     </row>
     <row r="23" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
@@ -1891,11 +1990,13 @@
       <c r="G23" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="H23" s="10" t="s">
+      <c r="H23" s="2" t="s">
         <v>35</v>
       </c>
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
+      <c r="K23" s="8"/>
+      <c r="L23" s="12"/>
     </row>
     <row r="24" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
@@ -1919,13 +2020,15 @@
       <c r="G24" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="H24" s="10" t="s">
+      <c r="H24" s="2" t="s">
         <v>58</v>
       </c>
       <c r="I24" s="2"/>
       <c r="J24" s="2" t="s">
         <v>186</v>
       </c>
+      <c r="K24" s="8"/>
+      <c r="L24" s="12"/>
     </row>
     <row r="25" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
@@ -1949,15 +2052,15 @@
       <c r="G25" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="H25" s="10" t="s">
+      <c r="H25" s="2" t="s">
         <v>38</v>
       </c>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
-      <c r="K25" s="12" t="s">
-        <v>218</v>
-      </c>
-      <c r="L25">
+      <c r="K25" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="L25" s="12">
         <v>0</v>
       </c>
     </row>
@@ -1969,7 +2072,7 @@
         <v>67</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>17</v>
@@ -1983,11 +2086,17 @@
       <c r="G26" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="H26" s="10" t="s">
+      <c r="H26" s="2" t="s">
         <v>39</v>
       </c>
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
+      <c r="K26" s="8" t="s">
+        <v>224</v>
+      </c>
+      <c r="L26" s="12">
+        <v>150000</v>
+      </c>
     </row>
     <row r="27" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
@@ -1997,7 +2106,7 @@
         <v>67</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>17</v>
@@ -2011,11 +2120,17 @@
       <c r="G27" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="H27" s="10" t="s">
+      <c r="H27" s="2" t="s">
         <v>56</v>
       </c>
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
+      <c r="K27" s="8" t="s">
+        <v>224</v>
+      </c>
+      <c r="L27" s="12">
+        <v>150000</v>
+      </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
@@ -2037,13 +2152,15 @@
         <v>120000</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="H28" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="H28" s="2" t="s">
         <v>49</v>
       </c>
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
+      <c r="K28" s="8"/>
+      <c r="L28" s="12"/>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
@@ -2067,13 +2184,15 @@
       <c r="G29" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="H29" s="10" t="s">
+      <c r="H29" s="2" t="s">
         <v>44</v>
       </c>
       <c r="I29" s="2"/>
       <c r="J29" s="2" t="s">
         <v>96</v>
       </c>
+      <c r="K29" s="8"/>
+      <c r="L29" s="12"/>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
@@ -2097,14 +2216,17 @@
       <c r="G30" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="H30" s="10" t="s">
+      <c r="H30" s="2" t="s">
         <v>46</v>
       </c>
       <c r="I30" s="2"/>
       <c r="J30" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="L30">
+      <c r="K30" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="L30" s="12">
         <v>55000</v>
       </c>
     </row>
@@ -2130,11 +2252,13 @@
       <c r="G31" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="H31" s="10" t="s">
+      <c r="H31" s="2" t="s">
         <v>210</v>
       </c>
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
+      <c r="K31" s="8"/>
+      <c r="L31" s="12"/>
     </row>
     <row r="32" spans="1:13" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
@@ -2158,11 +2282,13 @@
       <c r="G32" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="H32" s="10" t="s">
+      <c r="H32" s="2" t="s">
         <v>53</v>
       </c>
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
+      <c r="K32" s="8"/>
+      <c r="L32" s="12"/>
     </row>
     <row r="33" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
@@ -2172,7 +2298,7 @@
         <v>70</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>20</v>
@@ -2186,11 +2312,17 @@
       <c r="G33" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="H33" s="10" t="s">
+      <c r="H33" s="2" t="s">
         <v>211</v>
       </c>
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
+      <c r="K33" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="L33" s="12">
+        <v>10000</v>
+      </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
@@ -2200,7 +2332,7 @@
         <v>10</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>24</v>
@@ -2214,11 +2346,17 @@
       <c r="G34" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="H34" s="10" t="s">
+      <c r="H34" s="2" t="s">
         <v>208</v>
       </c>
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
+      <c r="K34" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="L34" s="12">
+        <v>35000</v>
+      </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
@@ -2242,11 +2380,13 @@
       <c r="G35" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="H35" s="10" t="s">
+      <c r="H35" s="2" t="s">
         <v>52</v>
       </c>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
+      <c r="K35" s="8"/>
+      <c r="L35" s="12"/>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
@@ -2270,11 +2410,13 @@
       <c r="G36" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="H36" s="10" t="s">
+      <c r="H36" s="2" t="s">
         <v>59</v>
       </c>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
+      <c r="K36" s="8"/>
+      <c r="L36" s="12"/>
     </row>
     <row r="37" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
@@ -2298,13 +2440,15 @@
       <c r="G37" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="H37" s="10" t="s">
+      <c r="H37" s="2" t="s">
         <v>61</v>
       </c>
       <c r="I37" s="2"/>
       <c r="J37" s="2" t="s">
         <v>126</v>
       </c>
+      <c r="K37" s="8"/>
+      <c r="L37" s="12"/>
     </row>
     <row r="38" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
@@ -2328,11 +2472,13 @@
       <c r="G38" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="H38" s="10" t="s">
+      <c r="H38" s="2" t="s">
         <v>55</v>
       </c>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
+      <c r="K38" s="8"/>
+      <c r="L38" s="12"/>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
@@ -2356,11 +2502,13 @@
       <c r="G39" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="H39" s="10" t="s">
+      <c r="H39" s="2" t="s">
         <v>60</v>
       </c>
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
+      <c r="K39" s="8"/>
+      <c r="L39" s="12"/>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
@@ -2384,11 +2532,13 @@
       <c r="G40" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="H40" s="10" t="s">
+      <c r="H40" s="2" t="s">
         <v>63</v>
       </c>
       <c r="I40" s="2"/>
       <c r="J40" s="2"/>
+      <c r="K40" s="8"/>
+      <c r="L40" s="12"/>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
@@ -2412,11 +2562,13 @@
       <c r="G41" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="H41" s="10" t="s">
+      <c r="H41" s="2" t="s">
         <v>64</v>
       </c>
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
+      <c r="K41" s="8"/>
+      <c r="L41" s="12"/>
     </row>
     <row r="42" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
@@ -2440,15 +2592,15 @@
       <c r="G42" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="H42" s="10" t="s">
+      <c r="H42" s="2" t="s">
         <v>65</v>
       </c>
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
       <c r="K42" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="L42">
+        <v>216</v>
+      </c>
+      <c r="L42" s="12">
         <v>10000</v>
       </c>
     </row>
@@ -2460,7 +2612,7 @@
         <v>128</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>172</v>
@@ -2474,11 +2626,17 @@
       <c r="G43" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="H43" s="10" t="s">
+      <c r="H43" s="2" t="s">
         <v>41</v>
       </c>
       <c r="I43" s="2"/>
       <c r="J43" s="2"/>
+      <c r="K43" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="L43" s="12">
+        <v>0</v>
+      </c>
     </row>
     <row r="44" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
@@ -2488,7 +2646,7 @@
         <v>128</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>172</v>
@@ -2502,11 +2660,17 @@
       <c r="G44" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="H44" s="10" t="s">
+      <c r="H44" s="2" t="s">
         <v>40</v>
       </c>
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
+      <c r="K44" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="L44" s="12">
+        <v>0</v>
+      </c>
     </row>
     <row r="45" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
@@ -2516,7 +2680,7 @@
         <v>67</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>18</v>
@@ -2530,11 +2694,17 @@
       <c r="G45" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="H45" s="10" t="s">
-        <v>221</v>
+      <c r="H45" s="2" t="s">
+        <v>219</v>
       </c>
       <c r="I45" s="2"/>
       <c r="J45" s="2"/>
+      <c r="K45" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="L45" s="12">
+        <v>0</v>
+      </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
@@ -2544,7 +2714,7 @@
         <v>10</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>18</v>
@@ -2558,9 +2728,15 @@
       <c r="G46" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="H46" s="10"/>
+      <c r="H46" s="2"/>
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
+      <c r="K46" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="L46" s="12">
+        <v>0</v>
+      </c>
     </row>
     <row r="47" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
@@ -2584,11 +2760,13 @@
       <c r="G47" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="H47" s="10" t="s">
+      <c r="H47" s="2" t="s">
         <v>36</v>
       </c>
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
+      <c r="K47" s="8"/>
+      <c r="L47" s="12"/>
     </row>
     <row r="48" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
@@ -2612,13 +2790,19 @@
       <c r="G48" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="H48" s="10" t="s">
+      <c r="H48" s="2" t="s">
         <v>57</v>
       </c>
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
-    </row>
-    <row r="49" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="K48" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="L48" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
         <v>146</v>
       </c>
@@ -2640,13 +2824,15 @@
       <c r="G49" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="H49" s="10" t="s">
+      <c r="H49" s="2" t="s">
         <v>50</v>
       </c>
       <c r="I49" s="2"/>
       <c r="J49" s="2"/>
-    </row>
-    <row r="50" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="K49" s="8"/>
+      <c r="L49" s="12"/>
+    </row>
+    <row r="50" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
         <v>137</v>
       </c>
@@ -2668,13 +2854,15 @@
       <c r="G50" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="H50" s="10" t="s">
+      <c r="H50" s="2" t="s">
         <v>42</v>
       </c>
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
-    </row>
-    <row r="51" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="K50" s="8"/>
+      <c r="L50" s="12"/>
+    </row>
+    <row r="51" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
         <v>138</v>
       </c>
@@ -2682,7 +2870,7 @@
         <v>10</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>172</v>
@@ -2696,13 +2884,19 @@
       <c r="G51" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="H51" s="10" t="s">
+      <c r="H51" s="2" t="s">
         <v>62</v>
       </c>
       <c r="I51" s="2"/>
       <c r="J51" s="2"/>
-    </row>
-    <row r="52" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="K51" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="L51" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
         <v>139</v>
       </c>
@@ -2710,7 +2904,7 @@
         <v>70</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D52" s="2" t="s">
         <v>172</v>
@@ -2724,13 +2918,19 @@
       <c r="G52" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="H52" s="10" t="s">
+      <c r="H52" s="2" t="s">
         <v>45</v>
       </c>
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
-    </row>
-    <row r="53" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="K52" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="L52" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
         <v>140</v>
       </c>
@@ -2752,13 +2952,15 @@
       <c r="G53" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="H53" s="10" t="s">
+      <c r="H53" s="2" t="s">
         <v>48</v>
       </c>
       <c r="I53" s="2"/>
       <c r="J53" s="2"/>
-    </row>
-    <row r="54" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+      <c r="K53" s="8"/>
+      <c r="L53" s="12"/>
+    </row>
+    <row r="54" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
         <v>141</v>
       </c>
@@ -2766,7 +2968,7 @@
         <v>67</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>199</v>
@@ -2780,11 +2982,21 @@
       <c r="G54" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="H54" s="10" t="s">
+      <c r="H54" s="2" t="s">
         <v>51</v>
       </c>
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
+      <c r="K54" s="16" t="s">
+        <v>223</v>
+      </c>
+      <c r="L54" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="I55" s="10"/>
+      <c r="J55" s="14"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Cambio fotos de vespa y actualizar vendidos a Familia 2
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/momuychayis/Documents/Python courses/Ventas_casa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1961809-BA98-0743-848B-25EB10E11105}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38F1BB8F-3BA5-6842-9B54-71BE2DBD6B6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16440" xr2:uid="{CD00CDD9-C0C8-D147-B0FC-6E5A64DE4059}"/>
   </bookViews>
@@ -907,7 +907,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -931,7 +931,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -941,7 +940,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1267,11 +1265,10 @@
     <col min="5" max="5" width="32.33203125" customWidth="1"/>
     <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="31.1640625" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="26.83203125" style="9" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="26.83203125" hidden="1" customWidth="1"/>
     <col min="9" max="9" width="15.6640625" style="8" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="10.83203125" style="15" hidden="1" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" style="17"/>
-    <col min="12" max="12" width="11.33203125" style="13" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.83203125" style="14" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="11.33203125" style="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">
@@ -1308,7 +1305,7 @@
       <c r="K1" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="L1" s="11" t="s">
+      <c r="L1" s="10" t="s">
         <v>217</v>
       </c>
     </row>
@@ -1340,7 +1337,7 @@
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
       <c r="K2" s="8"/>
-      <c r="L2" s="12"/>
+      <c r="L2" s="11"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
@@ -1372,7 +1369,7 @@
         <v>89</v>
       </c>
       <c r="K3" s="8"/>
-      <c r="L3" s="12"/>
+      <c r="L3" s="11"/>
     </row>
     <row r="4" spans="1:12" ht="289" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
@@ -1404,7 +1401,7 @@
         <v>135</v>
       </c>
       <c r="K4" s="8"/>
-      <c r="L4" s="12"/>
+      <c r="L4" s="11"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
@@ -1434,7 +1431,7 @@
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
       <c r="K5" s="8"/>
-      <c r="L5" s="12"/>
+      <c r="L5" s="11"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
@@ -1462,7 +1459,7 @@
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
       <c r="K6" s="8"/>
-      <c r="L6" s="12"/>
+      <c r="L6" s="11"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -1472,7 +1469,7 @@
         <v>10</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>17</v>
@@ -1525,7 +1522,7 @@
       <c r="K8" s="8" t="s">
         <v>223</v>
       </c>
-      <c r="L8" s="12">
+      <c r="L8" s="11">
         <v>120000</v>
       </c>
     </row>
@@ -1555,7 +1552,7 @@
       <c r="I9" s="2"/>
       <c r="J9" s="6"/>
       <c r="K9" s="8"/>
-      <c r="L9" s="12"/>
+      <c r="L9" s="11"/>
     </row>
     <row r="10" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
@@ -1583,7 +1580,7 @@
       <c r="I10" s="2"/>
       <c r="J10" s="6"/>
       <c r="K10" s="8"/>
-      <c r="L10" s="12"/>
+      <c r="L10" s="11"/>
     </row>
     <row r="11" spans="1:12" ht="119" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
@@ -1613,7 +1610,7 @@
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
       <c r="K11" s="8"/>
-      <c r="L11" s="12"/>
+      <c r="L11" s="11"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
@@ -1645,7 +1642,7 @@
       <c r="K12" s="8" t="s">
         <v>216</v>
       </c>
-      <c r="L12" s="12">
+      <c r="L12" s="11">
         <v>55000</v>
       </c>
     </row>
@@ -1681,7 +1678,7 @@
       <c r="K13" s="8" t="s">
         <v>225</v>
       </c>
-      <c r="L13" s="12">
+      <c r="L13" s="11">
         <v>30000</v>
       </c>
     </row>
@@ -1713,7 +1710,7 @@
       <c r="K14" s="8" t="s">
         <v>225</v>
       </c>
-      <c r="L14" s="12">
+      <c r="L14" s="11">
         <v>15000</v>
       </c>
     </row>
@@ -1745,7 +1742,7 @@
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
       <c r="K15" s="8"/>
-      <c r="L15" s="12"/>
+      <c r="L15" s="11"/>
     </row>
     <row r="16" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
@@ -1775,7 +1772,7 @@
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
       <c r="K16" s="8"/>
-      <c r="L16" s="12"/>
+      <c r="L16" s="11"/>
     </row>
     <row r="17" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
@@ -1805,7 +1802,7 @@
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
       <c r="K17" s="8"/>
-      <c r="L17" s="12"/>
+      <c r="L17" s="11"/>
     </row>
     <row r="18" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
@@ -1835,7 +1832,7 @@
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
       <c r="K18" s="8"/>
-      <c r="L18" s="12"/>
+      <c r="L18" s="11"/>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
@@ -1865,7 +1862,7 @@
       <c r="K19" s="8" t="s">
         <v>223</v>
       </c>
-      <c r="L19" s="12"/>
+      <c r="L19" s="11"/>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
@@ -1899,7 +1896,7 @@
       <c r="K20" s="8" t="s">
         <v>226</v>
       </c>
-      <c r="L20" s="12">
+      <c r="L20" s="11">
         <v>30000</v>
       </c>
     </row>
@@ -1933,7 +1930,7 @@
       <c r="K21" s="8" t="s">
         <v>216</v>
       </c>
-      <c r="L21" s="12">
+      <c r="L21" s="11">
         <v>110000</v>
       </c>
       <c r="M21" t="s">
@@ -1966,7 +1963,7 @@
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
       <c r="K22" s="8"/>
-      <c r="L22" s="12"/>
+      <c r="L22" s="11"/>
     </row>
     <row r="23" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
@@ -1996,7 +1993,7 @@
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
       <c r="K23" s="8"/>
-      <c r="L23" s="12"/>
+      <c r="L23" s="11"/>
     </row>
     <row r="24" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
@@ -2028,7 +2025,7 @@
         <v>186</v>
       </c>
       <c r="K24" s="8"/>
-      <c r="L24" s="12"/>
+      <c r="L24" s="11"/>
     </row>
     <row r="25" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
@@ -2060,7 +2057,7 @@
       <c r="K25" s="8" t="s">
         <v>216</v>
       </c>
-      <c r="L25" s="12">
+      <c r="L25" s="11">
         <v>0</v>
       </c>
     </row>
@@ -2094,7 +2091,7 @@
       <c r="K26" s="8" t="s">
         <v>224</v>
       </c>
-      <c r="L26" s="12">
+      <c r="L26" s="11">
         <v>150000</v>
       </c>
     </row>
@@ -2128,7 +2125,7 @@
       <c r="K27" s="8" t="s">
         <v>224</v>
       </c>
-      <c r="L27" s="12">
+      <c r="L27" s="11">
         <v>150000</v>
       </c>
     </row>
@@ -2160,7 +2157,7 @@
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
       <c r="K28" s="8"/>
-      <c r="L28" s="12"/>
+      <c r="L28" s="11"/>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
@@ -2192,7 +2189,7 @@
         <v>96</v>
       </c>
       <c r="K29" s="8"/>
-      <c r="L29" s="12"/>
+      <c r="L29" s="11"/>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
@@ -2226,7 +2223,7 @@
       <c r="K30" s="8" t="s">
         <v>216</v>
       </c>
-      <c r="L30" s="12">
+      <c r="L30" s="11">
         <v>55000</v>
       </c>
     </row>
@@ -2258,7 +2255,7 @@
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
       <c r="K31" s="8"/>
-      <c r="L31" s="12"/>
+      <c r="L31" s="11"/>
     </row>
     <row r="32" spans="1:13" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
@@ -2288,7 +2285,7 @@
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
       <c r="K32" s="8"/>
-      <c r="L32" s="12"/>
+      <c r="L32" s="11"/>
     </row>
     <row r="33" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
@@ -2320,7 +2317,7 @@
       <c r="K33" s="8" t="s">
         <v>225</v>
       </c>
-      <c r="L33" s="12">
+      <c r="L33" s="11">
         <v>10000</v>
       </c>
     </row>
@@ -2354,7 +2351,7 @@
       <c r="K34" s="8" t="s">
         <v>225</v>
       </c>
-      <c r="L34" s="12">
+      <c r="L34" s="11">
         <v>35000</v>
       </c>
     </row>
@@ -2386,7 +2383,7 @@
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
       <c r="K35" s="8"/>
-      <c r="L35" s="12"/>
+      <c r="L35" s="11"/>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
@@ -2416,7 +2413,7 @@
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
       <c r="K36" s="8"/>
-      <c r="L36" s="12"/>
+      <c r="L36" s="11"/>
     </row>
     <row r="37" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
@@ -2448,7 +2445,7 @@
         <v>126</v>
       </c>
       <c r="K37" s="8"/>
-      <c r="L37" s="12"/>
+      <c r="L37" s="11"/>
     </row>
     <row r="38" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
@@ -2478,7 +2475,7 @@
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
       <c r="K38" s="8"/>
-      <c r="L38" s="12"/>
+      <c r="L38" s="11"/>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
@@ -2508,7 +2505,7 @@
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
       <c r="K39" s="8"/>
-      <c r="L39" s="12"/>
+      <c r="L39" s="11"/>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
@@ -2538,7 +2535,7 @@
       <c r="I40" s="2"/>
       <c r="J40" s="2"/>
       <c r="K40" s="8"/>
-      <c r="L40" s="12"/>
+      <c r="L40" s="11"/>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
@@ -2568,7 +2565,7 @@
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
       <c r="K41" s="8"/>
-      <c r="L41" s="12"/>
+      <c r="L41" s="11"/>
     </row>
     <row r="42" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
@@ -2600,7 +2597,7 @@
       <c r="K42" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="L42" s="12">
+      <c r="L42" s="11">
         <v>10000</v>
       </c>
     </row>
@@ -2634,7 +2631,7 @@
       <c r="K43" s="8" t="s">
         <v>223</v>
       </c>
-      <c r="L43" s="12">
+      <c r="L43" s="11">
         <v>0</v>
       </c>
     </row>
@@ -2668,7 +2665,7 @@
       <c r="K44" s="8" t="s">
         <v>225</v>
       </c>
-      <c r="L44" s="12">
+      <c r="L44" s="11">
         <v>0</v>
       </c>
     </row>
@@ -2702,7 +2699,7 @@
       <c r="K45" s="8" t="s">
         <v>223</v>
       </c>
-      <c r="L45" s="12">
+      <c r="L45" s="11">
         <v>0</v>
       </c>
     </row>
@@ -2734,7 +2731,7 @@
       <c r="K46" s="8" t="s">
         <v>225</v>
       </c>
-      <c r="L46" s="12">
+      <c r="L46" s="11">
         <v>0</v>
       </c>
     </row>
@@ -2766,7 +2763,7 @@
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
       <c r="K47" s="8"/>
-      <c r="L47" s="12"/>
+      <c r="L47" s="11"/>
     </row>
     <row r="48" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
@@ -2798,7 +2795,7 @@
       <c r="K48" s="8" t="s">
         <v>227</v>
       </c>
-      <c r="L48" s="12">
+      <c r="L48" s="11">
         <v>0</v>
       </c>
     </row>
@@ -2830,7 +2827,7 @@
       <c r="I49" s="2"/>
       <c r="J49" s="2"/>
       <c r="K49" s="8"/>
-      <c r="L49" s="12"/>
+      <c r="L49" s="11"/>
     </row>
     <row r="50" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
@@ -2860,7 +2857,7 @@
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
       <c r="K50" s="8"/>
-      <c r="L50" s="12"/>
+      <c r="L50" s="11"/>
     </row>
     <row r="51" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
@@ -2892,7 +2889,7 @@
       <c r="K51" s="8" t="s">
         <v>225</v>
       </c>
-      <c r="L51" s="12">
+      <c r="L51" s="11">
         <v>0</v>
       </c>
     </row>
@@ -2926,7 +2923,7 @@
       <c r="K52" s="8" t="s">
         <v>223</v>
       </c>
-      <c r="L52" s="12">
+      <c r="L52" s="11">
         <v>0</v>
       </c>
     </row>
@@ -2958,7 +2955,7 @@
       <c r="I53" s="2"/>
       <c r="J53" s="2"/>
       <c r="K53" s="8"/>
-      <c r="L53" s="12"/>
+      <c r="L53" s="11"/>
     </row>
     <row r="54" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
@@ -2987,16 +2984,16 @@
       </c>
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
-      <c r="K54" s="16" t="s">
+      <c r="K54" s="15" t="s">
         <v>223</v>
       </c>
-      <c r="L54" s="12">
+      <c r="L54" s="11">
         <v>0</v>
       </c>
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="I55" s="10"/>
-      <c r="J55" s="14"/>
+      <c r="I55" s="9"/>
+      <c r="J55" s="13"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Limpiando los disponibles, agregando cosas gym y mostrar disponibles
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/momuychayis/Documents/Python courses/Ventas_casa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38F1BB8F-3BA5-6842-9B54-71BE2DBD6B6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26EA9505-304D-934E-868F-15C88ABBFC7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16440" xr2:uid="{CD00CDD9-C0C8-D147-B0FC-6E5A64DE4059}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$57</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="238">
   <si>
     <t>Nombre</t>
   </si>
@@ -365,14 +365,6 @@
   <si>
     <t>Mide 120cmx70cm y la altura se puede variar enter 74 y 120cm.
 Excelente calidad, precio original $500.</t>
-  </si>
-  <si>
-    <t>Rascador de múltiples niveles para gatos</t>
-  </si>
-  <si>
-    <t>Mide 85cm de ancho x 55cm de profundidad y 190cm de alto.
-Tiene cuevitas, repisas y rascadores incorporados. La mayoría de cosas se pueden quitar para ponerlas a lavar.
-Es un hit con los michis!</t>
   </si>
   <si>
     <t>Rodilleras articuladas para motociclista</t>
@@ -779,6 +771,45 @@
   </si>
   <si>
     <t>Maria</t>
+  </si>
+  <si>
+    <t>Ana</t>
+  </si>
+  <si>
+    <t>Adri</t>
+  </si>
+  <si>
+    <t>Amiga de Angie</t>
+  </si>
+  <si>
+    <t>Rascador de múltiples niveles para gatos -Disponible a finales de Enero</t>
+  </si>
+  <si>
+    <t>Mide 85cm de ancho x 55cm de profundidad y 190cm de alto.
+Tiene cuevitas, repisas y rascadores incorporados. La mayoría de cosas se pueden quitar para ponerlas a lavar.
+Es un hit con los michis!
+DISPONIBLE HASTA FINALES DE ENERO</t>
+  </si>
+  <si>
+    <t>Barra olímpica recta</t>
+  </si>
+  <si>
+    <t>Barra olímpica z</t>
+  </si>
+  <si>
+    <t>Gimnasio</t>
+  </si>
+  <si>
+    <t>Juego de discos de metal de varios pesos (2x5, 4x10lbs y 2x25lbs)</t>
+  </si>
+  <si>
+    <t>Similares a los de la foto. Actualizaremos la foto cuando todo lo del gym se haya limpiado</t>
+  </si>
+  <si>
+    <t>discosQuepeño.jpeg</t>
+  </si>
+  <si>
+    <t>barraquepeño.jpeg</t>
   </si>
 </sst>
 </file>
@@ -1255,7 +1286,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60AABAA7-0A6C-104B-82C9-83D30D50B2A2}">
-  <dimension ref="A1:M55"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:M58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="39.6640625" bestFit="1" customWidth="1"/>
@@ -1264,10 +1296,10 @@
     <col min="4" max="4" width="23.6640625" customWidth="1"/>
     <col min="5" max="5" width="32.33203125" customWidth="1"/>
     <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="31.1640625" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="26.83203125" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="15.6640625" style="8" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="10.83203125" style="14" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="48.5" customWidth="1"/>
+    <col min="8" max="8" width="26.83203125" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" style="8" customWidth="1"/>
+    <col min="10" max="10" width="10.83203125" style="14" customWidth="1"/>
     <col min="12" max="12" width="11.33203125" style="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1303,15 +1335,15 @@
         <v>8</v>
       </c>
       <c r="K1" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="L1" s="10" t="s">
         <v>215</v>
-      </c>
-      <c r="L1" s="10" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>7</v>
@@ -1320,16 +1352,16 @@
         <v>13</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="F2" s="5">
         <v>40000</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>54</v>
@@ -1373,7 +1405,7 @@
     </row>
     <row r="4" spans="1:12" ht="289" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>7</v>
@@ -1382,30 +1414,30 @@
         <v>13</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F4" s="5">
         <v>4000000</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="K4" s="8"/>
       <c r="L4" s="11"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>7</v>
@@ -1414,7 +1446,7 @@
         <v>13</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>6</v>
@@ -1423,10 +1455,10 @@
         <v>3500000</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
@@ -1435,7 +1467,7 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>7</v>
@@ -1444,16 +1476,16 @@
         <v>13</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F6" s="5">
         <v>8300000</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
@@ -1461,21 +1493,21 @@
       <c r="K6" s="8"/>
       <c r="L6" s="11"/>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>17</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="F7" s="5">
         <v>140000</v>
@@ -1484,17 +1516,22 @@
         <v>11</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="I7" s="2"/>
       <c r="J7" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="K7" s="8"/>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="K7" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="L7" s="12">
+        <v>130000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>10</v>
@@ -1506,7 +1543,7 @@
         <v>17</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F8" s="5">
         <v>120000</v>
@@ -1520,323 +1557,331 @@
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
       <c r="K8" s="8" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="L8" s="11">
         <v>120000</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>174</v>
+        <v>231</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>7</v>
+        <v>233</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>177</v>
+        <v>201</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>201</v>
       </c>
       <c r="F9" s="5">
-        <v>220000</v>
+        <v>34000</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="H9" s="2"/>
+        <v>235</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>237</v>
+      </c>
       <c r="I9" s="2"/>
-      <c r="J9" s="6"/>
+      <c r="J9" s="2"/>
       <c r="K9" s="8"/>
       <c r="L9" s="11"/>
     </row>
-    <row r="10" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>175</v>
+        <v>232</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>7</v>
+        <v>233</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>176</v>
+        <v>201</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>201</v>
       </c>
       <c r="F10" s="5">
-        <v>180000</v>
+        <v>19000</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="H10" s="2"/>
+        <v>235</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>237</v>
+      </c>
       <c r="I10" s="2"/>
-      <c r="J10" s="6"/>
+      <c r="J10" s="2"/>
       <c r="K10" s="8"/>
       <c r="L10" s="11"/>
     </row>
-    <row r="11" spans="1:12" ht="119" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>14</v>
+        <v>234</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>70</v>
+        <v>233</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>66</v>
+        <v>201</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>20</v>
+        <v>201</v>
       </c>
       <c r="F11" s="5">
-        <v>80000</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>220</v>
+        <v>32000</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>235</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>214</v>
+        <v>236</v>
       </c>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
       <c r="K11" s="8"/>
       <c r="L11" s="11"/>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>200</v>
+        <v>172</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>128</v>
+        <v>7</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>203</v>
+        <v>150</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>175</v>
       </c>
       <c r="F12" s="5">
-        <v>60000</v>
+        <v>220000</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>204</v>
-      </c>
+        <v>171</v>
+      </c>
+      <c r="H12" s="2"/>
       <c r="I12" s="2"/>
-      <c r="J12" s="2"/>
-      <c r="K12" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="L12" s="11">
-        <v>55000</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" ht="37" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="J12" s="6"/>
+      <c r="K12" s="8"/>
+      <c r="L12" s="11"/>
+    </row>
+    <row r="13" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>25</v>
+        <v>173</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>26</v>
+        <v>150</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>174</v>
       </c>
       <c r="F13" s="5">
-        <v>30000</v>
+        <v>180000</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>43</v>
-      </c>
+        <v>176</v>
+      </c>
+      <c r="H13" s="2"/>
       <c r="I13" s="2"/>
-      <c r="J13" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="K13" s="8" t="s">
-        <v>225</v>
-      </c>
-      <c r="L13" s="11">
-        <v>30000</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="J13" s="6"/>
+      <c r="K13" s="8"/>
+      <c r="L13" s="11"/>
+    </row>
+    <row r="14" spans="1:12" ht="119" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>160</v>
+        <v>14</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>10</v>
+        <v>70</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>18</v>
+        <v>66</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>161</v>
+        <v>20</v>
       </c>
       <c r="F14" s="5">
-        <v>15000</v>
-      </c>
-      <c r="G14" s="2"/>
+        <v>80000</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>218</v>
+      </c>
       <c r="H14" s="2" t="s">
-        <v>28</v>
+        <v>212</v>
       </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
       <c r="K14" s="8" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L14" s="11">
-        <v>15000</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+        <v>70000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>157</v>
+        <v>198</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>10</v>
+        <v>126</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>159</v>
+        <v>200</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>103</v>
+        <v>201</v>
       </c>
       <c r="F15" s="5">
-        <v>40000</v>
+        <v>60000</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>158</v>
+        <v>199</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>29</v>
+        <v>202</v>
       </c>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
-      <c r="K15" s="8"/>
-      <c r="L15" s="11"/>
-    </row>
-    <row r="16" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+      <c r="K15" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="L15" s="11">
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="37" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>69</v>
+        <v>25</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>172</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>171</v>
+        <v>21</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>26</v>
       </c>
       <c r="F16" s="5">
-        <v>45000</v>
+        <v>30000</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>105</v>
+        <v>27</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
-      <c r="K16" s="8"/>
-      <c r="L16" s="11"/>
-    </row>
-    <row r="17" spans="1:13" ht="34" x14ac:dyDescent="0.2">
+      <c r="J16" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K16" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="L16" s="11">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>71</v>
+        <v>158</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>67</v>
+        <v>10</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="E17" s="4" t="s">
-        <v>171</v>
+      <c r="E17" s="2" t="s">
+        <v>159</v>
       </c>
       <c r="F17" s="5">
-        <v>10000</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>184</v>
-      </c>
+        <v>15000</v>
+      </c>
+      <c r="G17" s="2"/>
       <c r="H17" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
-      <c r="K17" s="8"/>
-      <c r="L17" s="11"/>
-    </row>
-    <row r="18" spans="1:13" ht="34" x14ac:dyDescent="0.2">
+      <c r="K17" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="L17" s="11">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>76</v>
+        <v>155</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>171</v>
+        <v>157</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>103</v>
       </c>
       <c r="F18" s="5">
-        <v>100000</v>
+        <v>40000</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>156</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
-      <c r="K18" s="8"/>
-      <c r="L18" s="11"/>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K18" s="8" t="s">
+        <v>224</v>
+      </c>
+      <c r="L18" s="11">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>153</v>
+        <v>69</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>70</v>
@@ -1844,356 +1889,356 @@
       <c r="C19" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>20</v>
+      <c r="D19" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>169</v>
       </c>
       <c r="F19" s="5">
-        <v>120000</v>
+        <v>45000</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="H19" s="2"/>
+        <v>105</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>30</v>
+      </c>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
-      <c r="K19" s="8" t="s">
-        <v>223</v>
-      </c>
+      <c r="K19" s="8"/>
       <c r="L19" s="11"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:13" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>10</v>
+        <v>67</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>85</v>
+        <v>18</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>169</v>
       </c>
       <c r="F20" s="5">
-        <v>30000</v>
+        <v>10000</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>106</v>
+        <v>182</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="I20" s="2"/>
-      <c r="J20" s="2" t="s">
-        <v>86</v>
-      </c>
+      <c r="J20" s="2"/>
       <c r="K20" s="8" t="s">
         <v>226</v>
       </c>
       <c r="L20" s="11">
-        <v>30000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>75</v>
+        <v>170</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F21" s="5">
-        <v>50000</v>
+        <v>100000</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>185</v>
+        <v>154</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
-      <c r="K21" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="L21" s="11">
-        <v>110000</v>
-      </c>
-      <c r="M21" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K21" s="8"/>
+      <c r="L21" s="11"/>
+    </row>
+    <row r="22" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>70</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>103</v>
+        <v>20</v>
       </c>
       <c r="F22" s="5">
-        <v>25000</v>
+        <v>120000</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
-      <c r="K22" s="8"/>
-      <c r="L22" s="11"/>
-    </row>
-    <row r="23" spans="1:13" ht="34" x14ac:dyDescent="0.2">
+      <c r="K22" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="L22" s="11">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="F23" s="5">
+        <v>30000</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I23" s="2"/>
+      <c r="J23" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="K23" s="8" t="s">
+        <v>224</v>
+      </c>
+      <c r="L23" s="11">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" ht="34" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="F24" s="5">
+        <v>50000</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
+      <c r="K24" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="L24" s="11">
+        <v>110000</v>
+      </c>
+      <c r="M24" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A25" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>70</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="F23" s="5">
-        <v>120000</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="I23" s="2"/>
-      <c r="J23" s="2"/>
-      <c r="K23" s="8"/>
-      <c r="L23" s="11"/>
-    </row>
-    <row r="24" spans="1:13" ht="34" x14ac:dyDescent="0.2">
-      <c r="A24" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="E24" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="F24" s="5">
-        <v>80000</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="H24" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="I24" s="2"/>
-      <c r="J24" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="K24" s="8"/>
-      <c r="L24" s="11"/>
-    </row>
-    <row r="25" spans="1:13" ht="34" x14ac:dyDescent="0.2">
-      <c r="A25" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>67</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>171</v>
+        <v>157</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>103</v>
       </c>
       <c r="F25" s="5">
-        <v>15000</v>
+        <v>25000</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="H25" s="2" t="s">
-        <v>38</v>
-      </c>
+        <v>161</v>
+      </c>
+      <c r="H25" s="2"/>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
-      <c r="K25" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="L25" s="11">
-        <v>0</v>
-      </c>
+      <c r="K25" s="8"/>
+      <c r="L25" s="11"/>
     </row>
     <row r="26" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>188</v>
+        <v>77</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>17</v>
+        <v>78</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F26" s="5">
-        <v>150000</v>
+        <v>120000</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>189</v>
+        <v>107</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
-      <c r="K26" s="8" t="s">
-        <v>224</v>
-      </c>
-      <c r="L26" s="11">
-        <v>150000</v>
-      </c>
+      <c r="K26" s="8"/>
+      <c r="L26" s="11"/>
     </row>
     <row r="27" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="F27" s="5">
+        <v>80000</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="I27" s="2"/>
+      <c r="J27" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="K27" s="8"/>
+      <c r="L27" s="11"/>
+    </row>
+    <row r="28" spans="1:13" ht="34" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C28" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D27" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="F27" s="5">
-        <v>150000</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="H27" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="I27" s="2"/>
-      <c r="J27" s="2"/>
-      <c r="K27" s="8" t="s">
-        <v>224</v>
-      </c>
-      <c r="L27" s="11">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A28" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>13</v>
-      </c>
       <c r="D28" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>94</v>
+        <v>170</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>169</v>
       </c>
       <c r="F28" s="5">
-        <v>120000</v>
+        <v>15000</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>213</v>
+        <v>90</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
-      <c r="K28" s="8"/>
-      <c r="L28" s="11"/>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K28" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="L28" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
-        <v>95</v>
+        <v>186</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>67</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E29" s="2" t="s">
-        <v>97</v>
+      <c r="E29" s="4" t="s">
+        <v>169</v>
       </c>
       <c r="F29" s="5">
-        <v>60000</v>
+        <v>150000</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>98</v>
+        <v>187</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="I29" s="2"/>
-      <c r="J29" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="K29" s="8"/>
-      <c r="L29" s="11"/>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="J29" s="2"/>
+      <c r="K29" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="L29" s="11">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>67</v>
@@ -2202,162 +2247,160 @@
         <v>21</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>169</v>
       </c>
       <c r="F30" s="5">
-        <v>60000</v>
+        <v>150000</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>101</v>
+        <v>188</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="I30" s="2"/>
-      <c r="J30" s="2" t="s">
-        <v>100</v>
-      </c>
+      <c r="J30" s="2"/>
       <c r="K30" s="8" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="L30" s="11">
-        <v>55000</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
-        <v>164</v>
+        <v>92</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>20</v>
+        <v>93</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>20</v>
+        <v>94</v>
       </c>
       <c r="F31" s="5">
-        <v>25000</v>
+        <v>120000</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>165</v>
+        <v>211</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>210</v>
+        <v>49</v>
       </c>
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
       <c r="K31" s="8"/>
       <c r="L31" s="11"/>
     </row>
-    <row r="32" spans="1:13" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>20</v>
+        <v>97</v>
       </c>
       <c r="F32" s="5">
-        <v>35000</v>
+        <v>60000</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="I32" s="2"/>
-      <c r="J32" s="2"/>
+      <c r="J32" s="2" t="s">
+        <v>96</v>
+      </c>
       <c r="K32" s="8"/>
       <c r="L32" s="11"/>
     </row>
-    <row r="33" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
-        <v>166</v>
+        <v>99</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>20</v>
+        <v>75</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F33" s="5">
-        <v>10000</v>
+        <v>60000</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>167</v>
+        <v>101</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>211</v>
+        <v>46</v>
       </c>
       <c r="I33" s="2"/>
-      <c r="J33" s="2"/>
+      <c r="J33" s="2" t="s">
+        <v>100</v>
+      </c>
       <c r="K33" s="8" t="s">
-        <v>225</v>
+        <v>214</v>
       </c>
       <c r="L33" s="11">
-        <v>10000</v>
+        <v>55000</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
-        <v>205</v>
+        <v>162</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>10</v>
+        <v>70</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>207</v>
+        <v>20</v>
       </c>
       <c r="F34" s="5">
-        <v>40000</v>
+        <v>25000</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>206</v>
+        <v>163</v>
       </c>
       <c r="H34" s="2" t="s">
         <v>208</v>
       </c>
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
-      <c r="K34" s="8" t="s">
-        <v>225</v>
-      </c>
-      <c r="L34" s="11">
-        <v>35000</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="K34" s="8"/>
+      <c r="L34" s="11"/>
+    </row>
+    <row r="35" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>70</v>
@@ -2375,303 +2418,309 @@
         <v>35000</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
       <c r="K35" s="8"/>
       <c r="L35" s="11"/>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:12" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
-        <v>114</v>
+        <v>164</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>115</v>
+        <v>70</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>116</v>
+        <v>20</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>118</v>
+        <v>20</v>
       </c>
       <c r="F36" s="5">
-        <v>20000</v>
+        <v>10000</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>117</v>
+        <v>165</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>59</v>
+        <v>209</v>
       </c>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
-      <c r="K36" s="8"/>
-      <c r="L36" s="11"/>
-    </row>
-    <row r="37" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K36" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="L36" s="11">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
-        <v>122</v>
+        <v>203</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>128</v>
+        <v>10</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>123</v>
+        <v>24</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>124</v>
+        <v>205</v>
       </c>
       <c r="F37" s="5">
-        <v>15000</v>
+        <v>40000</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>125</v>
+        <v>204</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>61</v>
+        <v>206</v>
       </c>
       <c r="I37" s="2"/>
-      <c r="J37" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="K37" s="8"/>
-      <c r="L37" s="11"/>
-    </row>
-    <row r="38" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+      <c r="J37" s="2"/>
+      <c r="K37" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="L37" s="11">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" ht="119" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
-        <v>111</v>
+        <v>229</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="E38" s="4" t="s">
-        <v>171</v>
+        <v>20</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>20</v>
       </c>
       <c r="F38" s="5">
-        <v>8000</v>
-      </c>
-      <c r="G38" s="2" t="s">
-        <v>112</v>
+        <v>35000</v>
+      </c>
+      <c r="G38" s="4" t="s">
+        <v>230</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
       <c r="K38" s="8"/>
       <c r="L38" s="11"/>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>20</v>
+        <v>114</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>20</v>
+        <v>116</v>
       </c>
       <c r="F39" s="5">
-        <v>4000</v>
+        <v>20000</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
-      <c r="K39" s="8"/>
-      <c r="L39" s="11"/>
-    </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="K39" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="L39" s="11">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C40" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>20</v>
+        <v>121</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>20</v>
+        <v>122</v>
       </c>
       <c r="F40" s="5">
-        <v>4000</v>
+        <v>15000</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="I40" s="2"/>
-      <c r="J40" s="2"/>
+      <c r="J40" s="2" t="s">
+        <v>124</v>
+      </c>
       <c r="K40" s="8"/>
       <c r="L40" s="11"/>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
-        <v>130</v>
+        <v>109</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>120</v>
+        <v>67</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E41" s="2" t="s">
-        <v>20</v>
+        <v>111</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>169</v>
       </c>
       <c r="F41" s="5">
-        <v>2000</v>
+        <v>8000</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>131</v>
+        <v>110</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
-      <c r="K41" s="8"/>
-      <c r="L41" s="11"/>
-    </row>
-    <row r="42" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+      <c r="K41" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="L41" s="11">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
-        <v>143</v>
+        <v>117</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>67</v>
+        <v>118</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="E42" s="4" t="s">
-        <v>171</v>
+        <v>20</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>20</v>
       </c>
       <c r="F42" s="5">
-        <v>10000</v>
+        <v>4000</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>142</v>
+        <v>119</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
-      <c r="K42" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="L42" s="11">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+      <c r="K42" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="L42" s="11"/>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
-        <v>144</v>
+        <v>125</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="E43" s="4" t="s">
-        <v>171</v>
+        <v>20</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>20</v>
       </c>
       <c r="F43" s="5">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>191</v>
+        <v>127</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>41</v>
+        <v>63</v>
       </c>
       <c r="I43" s="2"/>
       <c r="J43" s="2"/>
-      <c r="K43" s="8" t="s">
-        <v>223</v>
-      </c>
-      <c r="L43" s="11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+      <c r="K43" s="8"/>
+      <c r="L43" s="11"/>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
-        <v>145</v>
+        <v>128</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="E44" s="4" t="s">
-        <v>171</v>
+        <v>20</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>20</v>
       </c>
       <c r="F44" s="5">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>191</v>
+        <v>129</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>40</v>
+        <v>64</v>
       </c>
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
-      <c r="K44" s="8" t="s">
-        <v>225</v>
-      </c>
-      <c r="L44" s="11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+      <c r="K44" s="8"/>
+      <c r="L44" s="11"/>
+    </row>
+    <row r="45" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
-        <v>68</v>
+        <v>141</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>67</v>
@@ -2680,209 +2729,217 @@
         <v>21</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>18</v>
+        <v>170</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F45" s="5">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>191</v>
+        <v>140</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>219</v>
+        <v>65</v>
       </c>
       <c r="I45" s="2"/>
       <c r="J45" s="2"/>
-      <c r="K45" s="8" t="s">
-        <v>223</v>
+      <c r="K45" s="2" t="s">
+        <v>214</v>
       </c>
       <c r="L45" s="11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
-        <v>15</v>
+        <v>142</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>10</v>
+        <v>126</v>
       </c>
       <c r="C46" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>19</v>
+        <v>170</v>
+      </c>
+      <c r="E46" s="4" t="s">
+        <v>169</v>
       </c>
       <c r="F46" s="5">
         <v>0</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="H46" s="2"/>
+        <v>189</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>41</v>
+      </c>
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
       <c r="K46" s="8" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="L46" s="11">
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
-        <v>79</v>
+        <v>143</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>67</v>
+        <v>126</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>80</v>
+        <v>170</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F47" s="5">
         <v>0</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
-      <c r="K47" s="8"/>
-      <c r="L47" s="11"/>
-    </row>
-    <row r="48" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+      <c r="K47" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="L47" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
-        <v>136</v>
+        <v>68</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>115</v>
+        <v>67</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>172</v>
+        <v>18</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F48" s="5">
         <v>0</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>57</v>
+        <v>217</v>
       </c>
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
       <c r="K48" s="8" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="L48" s="11">
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
-        <v>146</v>
+        <v>15</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>128</v>
+        <v>10</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="E49" s="4" t="s">
-        <v>171</v>
+        <v>18</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>19</v>
       </c>
       <c r="F49" s="5">
         <v>0</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="H49" s="2" t="s">
-        <v>50</v>
-      </c>
+        <v>190</v>
+      </c>
+      <c r="H49" s="2"/>
       <c r="I49" s="2"/>
       <c r="J49" s="2"/>
-      <c r="K49" s="8"/>
-      <c r="L49" s="11"/>
+      <c r="K49" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="L49" s="11">
+        <v>0</v>
+      </c>
     </row>
     <row r="50" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
-        <v>137</v>
+        <v>79</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C50" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>172</v>
+        <v>80</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F50" s="5">
         <v>0</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
       <c r="K50" s="8"/>
       <c r="L50" s="11"/>
     </row>
-    <row r="51" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>10</v>
+        <v>113</v>
       </c>
       <c r="C51" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F51" s="5">
         <v>0</v>
       </c>
       <c r="G51" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="I51" s="2"/>
       <c r="J51" s="2"/>
@@ -2895,107 +2952,212 @@
     </row>
     <row r="52" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>70</v>
+        <v>126</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F52" s="5">
         <v>0</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
-      <c r="K52" s="8" t="s">
-        <v>223</v>
-      </c>
-      <c r="L52" s="11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+      <c r="K52" s="8"/>
+      <c r="L52" s="11"/>
+    </row>
+    <row r="53" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>120</v>
+        <v>70</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F53" s="5">
         <v>0</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="I53" s="2"/>
       <c r="J53" s="2"/>
-      <c r="K53" s="8"/>
-      <c r="L53" s="11"/>
-    </row>
-    <row r="54" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+      <c r="K53" s="8" t="s">
+        <v>228</v>
+      </c>
+      <c r="L53" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>67</v>
+        <v>10</v>
       </c>
       <c r="C54" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>199</v>
+        <v>170</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F54" s="5">
         <v>0</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>51</v>
+        <v>62</v>
       </c>
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
-      <c r="K54" s="15" t="s">
+      <c r="K54" s="8" t="s">
         <v>223</v>
       </c>
       <c r="L54" s="11">
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="I55" s="9"/>
-      <c r="J55" s="13"/>
+    <row r="55" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="F55" s="5">
+        <v>0</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="H55" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I55" s="2"/>
+      <c r="J55" s="2"/>
+      <c r="K55" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="L55" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+      <c r="A56" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="F56" s="5">
+        <v>0</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="H56" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="I56" s="2"/>
+      <c r="J56" s="2"/>
+      <c r="K56" s="8"/>
+      <c r="L56" s="11"/>
+    </row>
+    <row r="57" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E57" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="F57" s="5">
+        <v>0</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="H57" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="I57" s="2"/>
+      <c r="J57" s="2"/>
+      <c r="K57" s="15" t="s">
+        <v>221</v>
+      </c>
+      <c r="L57" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="I58" s="9"/>
+      <c r="J58" s="13"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:M57" xr:uid="{60AABAA7-0A6C-104B-82C9-83D30D50B2A2}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="Disponible"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <hyperlinks>
     <hyperlink ref="J7" r:id="rId1" xr:uid="{C7799A81-F11B-B642-BEF0-047A2E3C329D}"/>
   </hyperlinks>

</xml_diff>

<commit_message>
intentando imagenes gym de nuevo
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/momuychayis/Documents/Python courses/Ventas_casa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26EA9505-304D-934E-868F-15C88ABBFC7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4558231-FCBF-7F4C-B288-3A53E3F6FCAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16440" xr2:uid="{CD00CDD9-C0C8-D147-B0FC-6E5A64DE4059}"/>
+    <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16420" xr2:uid="{CD00CDD9-C0C8-D147-B0FC-6E5A64DE4059}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -304,9 +304,6 @@
     <t>Stella Copper</t>
   </si>
   <si>
-    <t>Completamente nuevos. Talla L</t>
-  </si>
-  <si>
     <t>https://www.alpinestars.com/products/womens-copper-gloves-black?variant=40389898928186</t>
   </si>
   <si>
@@ -560,10 +557,6 @@
     <t>N/A</t>
   </si>
   <si>
-    <t>Talla M
-Tiene muy poco uso. Se venden con mantenimiento hecho por un ciclo.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Mountain Bike Scot Scale 980 </t>
   </si>
   <si>
@@ -576,10 +569,6 @@
   <si>
     <t xml:space="preserve">Scale 980
 </t>
-  </si>
-  <si>
-    <t>Talla S
-Tiene muy poco uso. Se venden con mantenimiento hecho por un ciclo.</t>
   </si>
   <si>
     <t>Zandona</t>
@@ -810,6 +799,15 @@
   </si>
   <si>
     <t>barraquepeño.jpeg</t>
+  </si>
+  <si>
+    <t>Talla M. Tiene muy poco uso. Se venden con mantenimiento hecho por un ciclo.</t>
+  </si>
+  <si>
+    <t>Talla S. Tiene muy poco uso. Se venden con mantenimiento hecho por un ciclo.</t>
+  </si>
+  <si>
+    <t>Completamente nuevos. Talla L de mujer</t>
   </si>
 </sst>
 </file>
@@ -1295,8 +1293,8 @@
     <col min="3" max="3" width="9.6640625" customWidth="1"/>
     <col min="4" max="4" width="23.6640625" customWidth="1"/>
     <col min="5" max="5" width="32.33203125" customWidth="1"/>
-    <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="48.5" customWidth="1"/>
+    <col min="6" max="6" width="40.83203125" customWidth="1"/>
+    <col min="7" max="7" width="140.1640625" customWidth="1"/>
     <col min="8" max="8" width="26.83203125" customWidth="1"/>
     <col min="9" max="9" width="15.6640625" style="8" customWidth="1"/>
     <col min="10" max="10" width="10.83203125" style="14" customWidth="1"/>
@@ -1335,15 +1333,15 @@
         <v>8</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="L1" s="10" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>7</v>
@@ -1352,16 +1350,16 @@
         <v>13</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="F2" s="5">
         <v>40000</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>54</v>
@@ -1391,21 +1389,21 @@
         <v>25000</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>88</v>
+        <v>237</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>37</v>
       </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="K3" s="8"/>
       <c r="L3" s="11"/>
     </row>
-    <row r="4" spans="1:12" ht="289" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" ht="238" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>7</v>
@@ -1414,30 +1412,30 @@
         <v>13</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>131</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>132</v>
       </c>
       <c r="F4" s="5">
         <v>4000000</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K4" s="8"/>
       <c r="L4" s="11"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>7</v>
@@ -1446,7 +1444,7 @@
         <v>13</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>6</v>
@@ -1455,10 +1453,10 @@
         <v>3500000</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
@@ -1467,7 +1465,7 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>7</v>
@@ -1476,16 +1474,16 @@
         <v>13</v>
       </c>
       <c r="D6" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>147</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>148</v>
       </c>
       <c r="F6" s="5">
         <v>8300000</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
@@ -1495,7 +1493,7 @@
     </row>
     <row r="7" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>10</v>
@@ -1507,7 +1505,7 @@
         <v>17</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F7" s="5">
         <v>140000</v>
@@ -1516,14 +1514,14 @@
         <v>11</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="I7" s="2"/>
       <c r="J7" s="6" t="s">
         <v>9</v>
       </c>
       <c r="K7" s="8" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="L7" s="12">
         <v>130000</v>
@@ -1531,7 +1529,7 @@
     </row>
     <row r="8" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>10</v>
@@ -1543,7 +1541,7 @@
         <v>17</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F8" s="5">
         <v>120000</v>
@@ -1557,7 +1555,7 @@
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
       <c r="K8" s="8" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="L8" s="11">
         <v>120000</v>
@@ -1565,28 +1563,28 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="F9" s="5">
         <v>34000</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
@@ -1595,28 +1593,28 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="F10" s="5">
         <v>19000</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
@@ -1625,28 +1623,28 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="F11" s="5">
         <v>32000</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
@@ -1655,7 +1653,7 @@
     </row>
     <row r="12" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>7</v>
@@ -1664,16 +1662,16 @@
         <v>13</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F12" s="5">
         <v>220000</v>
       </c>
-      <c r="G12" s="2" t="s">
-        <v>171</v>
+      <c r="G12" s="4" t="s">
+        <v>235</v>
       </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
@@ -1683,7 +1681,7 @@
     </row>
     <row r="13" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>7</v>
@@ -1692,16 +1690,16 @@
         <v>13</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="F13" s="5">
         <v>180000</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>176</v>
+        <v>236</v>
       </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
@@ -1729,15 +1727,15 @@
         <v>80000</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
       <c r="K14" s="8" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="L14" s="11">
         <v>70000</v>
@@ -1745,33 +1743,33 @@
     </row>
     <row r="15" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="F15" s="5">
         <v>60000</v>
       </c>
       <c r="G15" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="H15" s="2" t="s">
         <v>199</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>202</v>
       </c>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
       <c r="K15" s="8" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="L15" s="11">
         <v>55000</v>
@@ -1807,7 +1805,7 @@
         <v>23</v>
       </c>
       <c r="K16" s="8" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="L16" s="11">
         <v>30000</v>
@@ -1815,7 +1813,7 @@
     </row>
     <row r="17" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>10</v>
@@ -1827,7 +1825,7 @@
         <v>18</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F17" s="5">
         <v>15000</v>
@@ -1839,7 +1837,7 @@
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
       <c r="K17" s="8" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="L17" s="11">
         <v>15000</v>
@@ -1847,7 +1845,7 @@
     </row>
     <row r="18" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>10</v>
@@ -1856,16 +1854,16 @@
         <v>21</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F18" s="5">
         <v>40000</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H18" s="2" t="s">
         <v>29</v>
@@ -1873,7 +1871,7 @@
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
       <c r="K18" s="8" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="L18" s="11">
         <v>35000</v>
@@ -1890,16 +1888,16 @@
         <v>13</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F19" s="5">
         <v>45000</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H19" s="2" t="s">
         <v>30</v>
@@ -1923,13 +1921,13 @@
         <v>18</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F20" s="5">
         <v>10000</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="H20" s="2" t="s">
         <v>31</v>
@@ -1937,7 +1935,7 @@
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
       <c r="K20" s="8" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="L20" s="11">
         <v>10000</v>
@@ -1954,16 +1952,16 @@
         <v>13</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F21" s="5">
         <v>100000</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="H21" s="2" t="s">
         <v>32</v>
@@ -1975,7 +1973,7 @@
     </row>
     <row r="22" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>70</v>
@@ -1984,7 +1982,7 @@
         <v>21</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>20</v>
@@ -1993,13 +1991,13 @@
         <v>120000</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
       <c r="K22" s="8" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="L22" s="11">
         <v>100000</v>
@@ -2025,7 +2023,7 @@
         <v>30000</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H23" s="2" t="s">
         <v>33</v>
@@ -2035,7 +2033,7 @@
         <v>86</v>
       </c>
       <c r="K23" s="8" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="L23" s="11">
         <v>25000</v>
@@ -2055,13 +2053,13 @@
         <v>75</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F24" s="5">
         <v>50000</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="H24" s="2" t="s">
         <v>34</v>
@@ -2069,18 +2067,18 @@
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
       <c r="K24" s="8" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="L24" s="11">
         <v>110000</v>
       </c>
       <c r="M24" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>70</v>
@@ -2089,16 +2087,16 @@
         <v>13</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F25" s="5">
         <v>25000</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H25" s="2"/>
       <c r="I25" s="2"/>
@@ -2120,13 +2118,13 @@
         <v>78</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F26" s="5">
         <v>120000</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H26" s="2" t="s">
         <v>35</v>
@@ -2138,7 +2136,7 @@
     </row>
     <row r="27" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>70</v>
@@ -2147,23 +2145,23 @@
         <v>13</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F27" s="5">
         <v>80000</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="H27" s="2" t="s">
         <v>58</v>
       </c>
       <c r="I27" s="2"/>
       <c r="J27" s="2" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="K27" s="8"/>
       <c r="L27" s="11"/>
@@ -2179,16 +2177,16 @@
         <v>21</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F28" s="5">
         <v>15000</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H28" s="2" t="s">
         <v>38</v>
@@ -2196,7 +2194,7 @@
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
       <c r="K28" s="8" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="L28" s="11">
         <v>0</v>
@@ -2204,7 +2202,7 @@
     </row>
     <row r="29" spans="1:13" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>67</v>
@@ -2216,13 +2214,13 @@
         <v>17</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F29" s="5">
         <v>150000</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="H29" s="2" t="s">
         <v>39</v>
@@ -2230,7 +2228,7 @@
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
       <c r="K29" s="8" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="L29" s="11">
         <v>150000</v>
@@ -2250,13 +2248,13 @@
         <v>17</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F30" s="5">
         <v>150000</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="H30" s="2" t="s">
         <v>56</v>
@@ -2264,7 +2262,7 @@
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
       <c r="K30" s="8" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="L30" s="11">
         <v>150000</v>
@@ -2272,7 +2270,7 @@
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>10</v>
@@ -2281,16 +2279,16 @@
         <v>13</v>
       </c>
       <c r="D31" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E31" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>94</v>
       </c>
       <c r="F31" s="5">
         <v>120000</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="H31" s="2" t="s">
         <v>49</v>
@@ -2302,7 +2300,7 @@
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>67</v>
@@ -2314,27 +2312,27 @@
         <v>17</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F32" s="5">
         <v>60000</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H32" s="2" t="s">
         <v>44</v>
       </c>
       <c r="I32" s="2"/>
       <c r="J32" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="K32" s="8"/>
       <c r="L32" s="11"/>
     </row>
     <row r="33" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>67</v>
@@ -2352,17 +2350,17 @@
         <v>60000</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H33" s="2" t="s">
         <v>46</v>
       </c>
       <c r="I33" s="2"/>
       <c r="J33" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K33" s="8" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="L33" s="11">
         <v>55000</v>
@@ -2370,7 +2368,7 @@
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>70</v>
@@ -2388,10 +2386,10 @@
         <v>25000</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
@@ -2400,7 +2398,7 @@
     </row>
     <row r="35" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>70</v>
@@ -2418,7 +2416,7 @@
         <v>35000</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H35" s="2" t="s">
         <v>53</v>
@@ -2430,7 +2428,7 @@
     </row>
     <row r="36" spans="1:12" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>70</v>
@@ -2448,15 +2446,15 @@
         <v>10000</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
       <c r="K36" s="8" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="L36" s="11">
         <v>10000</v>
@@ -2464,7 +2462,7 @@
     </row>
     <row r="37" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>10</v>
@@ -2476,21 +2474,21 @@
         <v>24</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="F37" s="5">
         <v>40000</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
       <c r="K37" s="8" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="L37" s="11">
         <v>35000</v>
@@ -2498,7 +2496,7 @@
     </row>
     <row r="38" spans="1:12" ht="119" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>70</v>
@@ -2516,7 +2514,7 @@
         <v>35000</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="H38" s="2" t="s">
         <v>52</v>
@@ -2528,25 +2526,25 @@
     </row>
     <row r="39" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B39" s="2" t="s">
         <v>112</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>113</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F39" s="5">
         <v>20000</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H39" s="2" t="s">
         <v>59</v>
@@ -2554,7 +2552,7 @@
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
       <c r="K39" s="8" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="L39" s="11">
         <v>20000</v>
@@ -2562,39 +2560,39 @@
     </row>
     <row r="40" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C40" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D40" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="E40" s="2" t="s">
         <v>121</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>122</v>
       </c>
       <c r="F40" s="5">
         <v>15000</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H40" s="2" t="s">
         <v>61</v>
       </c>
       <c r="I40" s="2"/>
       <c r="J40" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="K40" s="8"/>
       <c r="L40" s="11"/>
     </row>
     <row r="41" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>67</v>
@@ -2603,16 +2601,16 @@
         <v>21</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F41" s="5">
         <v>8000</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H41" s="2" t="s">
         <v>55</v>
@@ -2620,7 +2618,7 @@
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
       <c r="K41" s="8" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="L41" s="11">
         <v>8000</v>
@@ -2628,10 +2626,10 @@
     </row>
     <row r="42" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B42" s="2" t="s">
         <v>117</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>118</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>21</v>
@@ -2646,7 +2644,7 @@
         <v>4000</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H42" s="2" t="s">
         <v>60</v>
@@ -2654,16 +2652,16 @@
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
       <c r="K42" s="8" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="L42" s="11"/>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C43" s="3" t="s">
         <v>13</v>
@@ -2678,7 +2676,7 @@
         <v>4000</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H43" s="2" t="s">
         <v>63</v>
@@ -2690,10 +2688,10 @@
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C44" s="3" t="s">
         <v>13</v>
@@ -2708,7 +2706,7 @@
         <v>2000</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="H44" s="2" t="s">
         <v>64</v>
@@ -2720,7 +2718,7 @@
     </row>
     <row r="45" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>67</v>
@@ -2729,16 +2727,16 @@
         <v>21</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F45" s="5">
         <v>10000</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="H45" s="2" t="s">
         <v>65</v>
@@ -2746,7 +2744,7 @@
       <c r="I45" s="2"/>
       <c r="J45" s="2"/>
       <c r="K45" s="2" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="L45" s="11">
         <v>10000</v>
@@ -2754,25 +2752,25 @@
     </row>
     <row r="46" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C46" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F46" s="5">
         <v>0</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="H46" s="2" t="s">
         <v>41</v>
@@ -2780,7 +2778,7 @@
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
       <c r="K46" s="8" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="L46" s="11">
         <v>0</v>
@@ -2788,25 +2786,25 @@
     </row>
     <row r="47" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C47" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F47" s="5">
         <v>0</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="H47" s="2" t="s">
         <v>40</v>
@@ -2814,7 +2812,7 @@
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
       <c r="K47" s="8" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="L47" s="11">
         <v>0</v>
@@ -2834,21 +2832,21 @@
         <v>18</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F48" s="5">
         <v>0</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
       <c r="K48" s="8" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="L48" s="11">
         <v>0</v>
@@ -2874,13 +2872,13 @@
         <v>0</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="H49" s="2"/>
       <c r="I49" s="2"/>
       <c r="J49" s="2"/>
       <c r="K49" s="8" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="L49" s="11">
         <v>0</v>
@@ -2900,13 +2898,13 @@
         <v>80</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F50" s="5">
         <v>0</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="H50" s="2" t="s">
         <v>36</v>
@@ -2918,25 +2916,25 @@
     </row>
     <row r="51" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C51" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F51" s="5">
         <v>0</v>
       </c>
       <c r="G51" s="2" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="H51" s="2" t="s">
         <v>57</v>
@@ -2944,7 +2942,7 @@
       <c r="I51" s="2"/>
       <c r="J51" s="2"/>
       <c r="K51" s="8" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="L51" s="11">
         <v>0</v>
@@ -2952,25 +2950,25 @@
     </row>
     <row r="52" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C52" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F52" s="5">
         <v>0</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="H52" s="2" t="s">
         <v>50</v>
@@ -2982,7 +2980,7 @@
     </row>
     <row r="53" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>70</v>
@@ -2991,16 +2989,16 @@
         <v>21</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F53" s="5">
         <v>0</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="H53" s="2" t="s">
         <v>42</v>
@@ -3008,7 +3006,7 @@
       <c r="I53" s="2"/>
       <c r="J53" s="2"/>
       <c r="K53" s="8" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="L53" s="11">
         <v>0</v>
@@ -3016,7 +3014,7 @@
     </row>
     <row r="54" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>10</v>
@@ -3025,16 +3023,16 @@
         <v>21</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F54" s="5">
         <v>0</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="H54" s="2" t="s">
         <v>62</v>
@@ -3042,7 +3040,7 @@
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
       <c r="K54" s="8" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="L54" s="11">
         <v>0</v>
@@ -3050,7 +3048,7 @@
     </row>
     <row r="55" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>70</v>
@@ -3059,16 +3057,16 @@
         <v>21</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F55" s="5">
         <v>0</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="H55" s="2" t="s">
         <v>45</v>
@@ -3076,7 +3074,7 @@
       <c r="I55" s="2"/>
       <c r="J55" s="2"/>
       <c r="K55" s="8" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="L55" s="11">
         <v>0</v>
@@ -3084,25 +3082,25 @@
     </row>
     <row r="56" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C56" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F56" s="5">
         <v>0</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="H56" s="2" t="s">
         <v>48</v>
@@ -3114,7 +3112,7 @@
     </row>
     <row r="57" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>67</v>
@@ -3123,16 +3121,16 @@
         <v>21</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="E57" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F57" s="5">
         <v>0</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="H57" s="2" t="s">
         <v>51</v>
@@ -3140,7 +3138,7 @@
       <c r="I57" s="2"/>
       <c r="J57" s="2"/>
       <c r="K57" s="15" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="L57" s="11">
         <v>0</v>

</xml_diff>

<commit_message>
intentando imagenes gym de nuevo sin ñ
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/momuychayis/Documents/Python courses/Ventas_casa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4558231-FCBF-7F4C-B288-3A53E3F6FCAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CDBB9C6-501A-594B-A615-C3CAC7BB5200}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16420" xr2:uid="{CD00CDD9-C0C8-D147-B0FC-6E5A64DE4059}"/>
   </bookViews>
@@ -795,12 +795,6 @@
     <t>Similares a los de la foto. Actualizaremos la foto cuando todo lo del gym se haya limpiado</t>
   </si>
   <si>
-    <t>discosQuepeño.jpeg</t>
-  </si>
-  <si>
-    <t>barraquepeño.jpeg</t>
-  </si>
-  <si>
     <t>Talla M. Tiene muy poco uso. Se venden con mantenimiento hecho por un ciclo.</t>
   </si>
   <si>
@@ -808,6 +802,12 @@
   </si>
   <si>
     <t>Completamente nuevos. Talla L de mujer</t>
+  </si>
+  <si>
+    <t>barraquepeno.jpeg</t>
+  </si>
+  <si>
+    <t>discosQuepeno.jpeg</t>
   </si>
 </sst>
 </file>
@@ -1389,7 +1389,7 @@
         <v>25000</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>37</v>
@@ -1401,7 +1401,7 @@
       <c r="K3" s="8"/>
       <c r="L3" s="11"/>
     </row>
-    <row r="4" spans="1:12" ht="238" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" ht="102" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>129</v>
       </c>
@@ -1584,7 +1584,7 @@
         <v>232</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
@@ -1614,7 +1614,7 @@
         <v>232</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
@@ -1644,7 +1644,7 @@
         <v>232</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
@@ -1671,7 +1671,7 @@
         <v>220000</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
@@ -1699,7 +1699,7 @@
         <v>180000</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
@@ -2494,7 +2494,7 @@
         <v>35000</v>
       </c>
     </row>
-    <row r="38" spans="1:12" ht="119" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:12" ht="68" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>226</v>
       </c>

</xml_diff>

<commit_message>
vendido escritorio y rascado
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/momuychayis/Documents/Python courses/Ventas_casa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CDBB9C6-501A-594B-A615-C3CAC7BB5200}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B2068EE-4A34-C54D-8B0A-2FA91EC94BC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16420" xr2:uid="{CD00CDD9-C0C8-D147-B0FC-6E5A64DE4059}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="240">
   <si>
     <t>Nombre</t>
   </si>
@@ -808,6 +808,12 @@
   </si>
   <si>
     <t>discosQuepeno.jpeg</t>
+  </si>
+  <si>
+    <t>Isaac</t>
+  </si>
+  <si>
+    <t>Ully</t>
   </si>
 </sst>
 </file>
@@ -2112,7 +2118,7 @@
         <v>70</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>78</v>
@@ -2131,8 +2137,12 @@
       </c>
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
-      <c r="K26" s="8"/>
-      <c r="L26" s="11"/>
+      <c r="K26" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="L26" s="11">
+        <v>120000</v>
+      </c>
     </row>
     <row r="27" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
@@ -2502,7 +2512,7 @@
         <v>70</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>20</v>
@@ -2521,8 +2531,12 @@
       </c>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
-      <c r="K38" s="8"/>
-      <c r="L38" s="11"/>
+      <c r="K38" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="L38" s="11">
+        <v>35000</v>
+      </c>
     </row>
     <row r="39" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">

</xml_diff>

<commit_message>
quitando la monstra temporalmente
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/momuychayis/Documents/Python courses/Ventas_casa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0E6E5DC-8563-6942-9205-626EC0B18831}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C36006C0-C9BC-0944-AD17-0FC2D5C28631}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16420" xr2:uid="{CD00CDD9-C0C8-D147-B0FC-6E5A64DE4059}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$56</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="236">
   <si>
     <t>Nombre</t>
   </si>
@@ -56,9 +56,6 @@
   </si>
   <si>
     <t>Video</t>
-  </si>
-  <si>
-    <t>Multistrada 950</t>
   </si>
   <si>
     <t>Vehículos</t>
@@ -472,9 +469,6 @@
     <t>Portaretratos</t>
   </si>
   <si>
-    <t>Multistrada 950 2017</t>
-  </si>
-  <si>
     <t>Tucson Elegant AWD 2000cc-2017</t>
   </si>
   <si>
@@ -482,9 +476,6 @@
   </si>
   <si>
     <t>Elegant -2017</t>
-  </si>
-  <si>
-    <t>Ducati</t>
   </si>
   <si>
     <t>Scot</t>
@@ -593,18 +584,6 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">-Kilometraje: 56000km
-Incluye:
-1. Pantalla inteligente Chigee AIO-5 lite
-2. Cámara trasera y delantera
-3. Medidor de presión de llantas
-4. Defensas SW-Motech
-5. Tank bag marca Ducati
-6. Baúl Ducati (problema de cierre, usa un candado :) )
-7.Marchamo incluido, traspaso corre por cuenta del comprador.
-</t>
-  </si>
-  <si>
     <t>Batido con tazon y dos aspas, se ha usado una vez :)</t>
   </si>
   <si>
@@ -703,9 +682,6 @@
   </si>
   <si>
     <t>MesitaNoche.jpeg</t>
-  </si>
-  <si>
-    <t>monstra1.jpeg,monstra2.jpeg,monstra3.jpeg,monstra4.jpeg,monstra5.jpeg</t>
   </si>
   <si>
     <t>Incluye el play4 de 500GB, manivela Trustmaster, 2 controles, 3 juegos físicos (Crash, PES2018 y Battlefront II) además de juegos descargados en la consola (Fútbol americano, Fórmula 1, Snipper Elite y Grand Turismo).</t>
@@ -945,7 +921,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -978,9 +954,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1297,7 +1270,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60AABAA7-0A6C-104B-82C9-83D30D50B2A2}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:M58"/>
+  <dimension ref="A1:M57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="39.6640625" bestFit="1" customWidth="1"/>
@@ -1318,13 +1291,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>1</v>
@@ -1342,39 +1315,39 @@
         <v>5</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="L1" s="10" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="F2" s="5">
         <v>40000</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
@@ -1383,220 +1356,220 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>81</v>
-      </c>
       <c r="E3" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F3" s="5">
         <v>25000</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="K3" s="8"/>
       <c r="L3" s="11"/>
     </row>
     <row r="4" spans="1:12" ht="102" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>129</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>130</v>
       </c>
       <c r="F4" s="5">
         <v>4000000</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="K4" s="8"/>
       <c r="L4" s="11"/>
     </row>
-    <row r="5" spans="1:12" ht="170" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>147</v>
-      </c>
       <c r="E5" s="2" t="s">
-        <v>6</v>
+        <v>144</v>
       </c>
       <c r="F5" s="5">
-        <v>3500000</v>
-      </c>
-      <c r="G5" s="16" t="s">
-        <v>177</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>206</v>
-      </c>
+        <v>8300000</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="H5" s="2"/>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
       <c r="K5" s="8"/>
       <c r="L5" s="11"/>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>144</v>
+        <v>161</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>145</v>
+        <v>16</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>146</v>
+        <v>162</v>
       </c>
       <c r="F6" s="5">
-        <v>8300000</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>176</v>
-      </c>
-      <c r="H6" s="2"/>
+        <v>140000</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>199</v>
+      </c>
       <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="8"/>
-      <c r="L6" s="11"/>
+      <c r="J6" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="K6" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="L6" s="12">
+        <v>130000</v>
+      </c>
     </row>
     <row r="7" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="F7" s="5">
+        <v>120000</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="F7" s="5">
-        <v>140000</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>11</v>
-      </c>
       <c r="H7" s="2" t="s">
-        <v>203</v>
+        <v>46</v>
       </c>
       <c r="I7" s="2"/>
-      <c r="J7" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="J7" s="2"/>
       <c r="K7" s="8" t="s">
-        <v>221</v>
-      </c>
-      <c r="L7" s="12">
-        <v>130000</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+        <v>212</v>
+      </c>
+      <c r="L7" s="11">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>164</v>
+        <v>222</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>10</v>
+        <v>224</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>17</v>
+        <v>193</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>166</v>
+        <v>193</v>
       </c>
       <c r="F8" s="5">
-        <v>120000</v>
+        <v>34000</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>11</v>
+        <v>226</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>47</v>
+        <v>230</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
-      <c r="K8" s="8" t="s">
-        <v>217</v>
-      </c>
-      <c r="L8" s="11">
-        <v>120000</v>
-      </c>
+      <c r="K8" s="8"/>
+      <c r="L8" s="11"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="F9" s="5">
-        <v>34000</v>
+        <v>19000</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
@@ -1605,85 +1578,83 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="F10" s="5">
-        <v>19000</v>
+        <v>32000</v>
       </c>
       <c r="G10" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="H10" s="2" t="s">
         <v>231</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>235</v>
       </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
       <c r="K10" s="8"/>
       <c r="L10" s="11"/>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>230</v>
+        <v>166</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>229</v>
+        <v>6</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>197</v>
+        <v>145</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>169</v>
       </c>
       <c r="F11" s="5">
-        <v>32000</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>236</v>
-      </c>
+        <v>220000</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="H11" s="2"/>
       <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
+      <c r="J11" s="6"/>
       <c r="K11" s="8"/>
       <c r="L11" s="11"/>
     </row>
     <row r="12" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="F12" s="5">
-        <v>220000</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>232</v>
+        <v>180000</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>228</v>
       </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
@@ -1691,255 +1662,261 @@
       <c r="K12" s="8"/>
       <c r="L12" s="11"/>
     </row>
-    <row r="13" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:12" ht="119" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>170</v>
+        <v>13</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>7</v>
+        <v>69</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>171</v>
+        <v>65</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>19</v>
       </c>
       <c r="F13" s="5">
-        <v>180000</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="H13" s="2"/>
+        <v>80000</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>203</v>
+      </c>
       <c r="I13" s="2"/>
-      <c r="J13" s="6"/>
-      <c r="K13" s="8"/>
-      <c r="L13" s="11"/>
-    </row>
-    <row r="14" spans="1:12" ht="119" hidden="1" x14ac:dyDescent="0.2">
+      <c r="J13" s="2"/>
+      <c r="K13" s="8" t="s">
+        <v>215</v>
+      </c>
+      <c r="L13" s="11">
+        <v>70000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>14</v>
+        <v>190</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>70</v>
+        <v>123</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>66</v>
+        <v>192</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>20</v>
+        <v>193</v>
       </c>
       <c r="F14" s="5">
-        <v>80000</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>214</v>
+        <v>60000</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>191</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>208</v>
+        <v>194</v>
       </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
       <c r="K14" s="8" t="s">
-        <v>220</v>
+        <v>205</v>
       </c>
       <c r="L14" s="11">
-        <v>70000</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="37" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>194</v>
+        <v>24</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>124</v>
+        <v>9</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>196</v>
+        <v>23</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>197</v>
+        <v>25</v>
       </c>
       <c r="F15" s="5">
-        <v>60000</v>
+        <v>30000</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>195</v>
+        <v>26</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>198</v>
+        <v>42</v>
       </c>
       <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
+      <c r="J15" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="K15" s="8" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="L15" s="11">
-        <v>55000</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" ht="37" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>25</v>
+        <v>153</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>26</v>
+        <v>154</v>
       </c>
       <c r="F16" s="5">
-        <v>30000</v>
-      </c>
-      <c r="G16" s="2" t="s">
+        <v>15000</v>
+      </c>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H16" s="2" t="s">
-        <v>43</v>
-      </c>
       <c r="I16" s="2"/>
-      <c r="J16" s="2" t="s">
-        <v>23</v>
-      </c>
+      <c r="J16" s="2"/>
       <c r="K16" s="8" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="L16" s="11">
-        <v>30000</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="17" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>18</v>
+        <v>152</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>157</v>
+        <v>100</v>
       </c>
       <c r="F17" s="5">
-        <v>15000</v>
-      </c>
-      <c r="G17" s="2"/>
+        <v>40000</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>151</v>
+      </c>
       <c r="H17" s="2" t="s">
         <v>28</v>
       </c>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
       <c r="K17" s="8" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="L17" s="11">
-        <v>15000</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>153</v>
+        <v>68</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>10</v>
+        <v>69</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>101</v>
+        <v>12</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>164</v>
       </c>
       <c r="F18" s="5">
-        <v>40000</v>
+        <v>45000</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>154</v>
+        <v>102</v>
       </c>
       <c r="H18" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
-      <c r="K18" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="L18" s="11">
-        <v>35000</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" ht="34" x14ac:dyDescent="0.2">
+      <c r="K18" s="8"/>
+      <c r="L18" s="11"/>
+    </row>
+    <row r="19" spans="1:13" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D19" s="7" t="s">
-        <v>168</v>
+        <v>20</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>17</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="F19" s="5">
-        <v>45000</v>
+        <v>10000</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>103</v>
+        <v>174</v>
       </c>
       <c r="H19" s="2" t="s">
         <v>30</v>
       </c>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
-      <c r="K19" s="8"/>
-      <c r="L19" s="11"/>
-    </row>
-    <row r="20" spans="1:13" ht="34" hidden="1" x14ac:dyDescent="0.2">
+      <c r="K19" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="L19" s="11">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>71</v>
+        <v>234</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>18</v>
+        <v>165</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="F20" s="5">
-        <v>10000</v>
+        <v>100000</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>178</v>
+        <v>149</v>
       </c>
       <c r="H20" s="2" t="s">
         <v>31</v>
@@ -1947,41 +1924,39 @@
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
       <c r="K20" s="8" t="s">
-        <v>222</v>
+        <v>235</v>
       </c>
       <c r="L20" s="11">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" ht="34" x14ac:dyDescent="0.2">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>239</v>
+        <v>146</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>167</v>
+        <v>147</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>19</v>
       </c>
       <c r="F21" s="5">
-        <v>100000</v>
+        <v>120000</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>32</v>
-      </c>
+        <v>148</v>
+      </c>
+      <c r="H21" s="2"/>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
       <c r="K21" s="8" t="s">
-        <v>240</v>
+        <v>218</v>
       </c>
       <c r="L21" s="11">
         <v>100000</v>
@@ -1989,224 +1964,226 @@
     </row>
     <row r="22" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>149</v>
+        <v>71</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>70</v>
+        <v>9</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>150</v>
+        <v>72</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>20</v>
+        <v>83</v>
       </c>
       <c r="F22" s="5">
-        <v>120000</v>
+        <v>30000</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="H22" s="2"/>
+        <v>103</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>32</v>
+      </c>
       <c r="I22" s="2"/>
-      <c r="J22" s="2"/>
+      <c r="J22" s="2" t="s">
+        <v>84</v>
+      </c>
       <c r="K22" s="8" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="L22" s="11">
-        <v>100000</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>10</v>
+        <v>66</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>164</v>
       </c>
       <c r="F23" s="5">
-        <v>30000</v>
+        <v>50000</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>104</v>
+        <v>175</v>
       </c>
       <c r="H23" s="2" t="s">
         <v>33</v>
       </c>
       <c r="I23" s="2"/>
-      <c r="J23" s="2" t="s">
-        <v>85</v>
-      </c>
+      <c r="J23" s="2"/>
       <c r="K23" s="8" t="s">
-        <v>220</v>
+        <v>205</v>
       </c>
       <c r="L23" s="11">
+        <v>110000</v>
+      </c>
+      <c r="M23" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F24" s="5">
         <v>25000</v>
       </c>
-    </row>
-    <row r="24" spans="1:13" ht="34" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="E24" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="F24" s="5">
-        <v>50000</v>
-      </c>
       <c r="G24" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="H24" s="2" t="s">
-        <v>34</v>
-      </c>
+        <v>156</v>
+      </c>
+      <c r="H24" s="2"/>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
-      <c r="K24" s="8" t="s">
-        <v>210</v>
-      </c>
-      <c r="L24" s="11">
-        <v>110000</v>
-      </c>
-      <c r="M24" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K24" s="8"/>
+      <c r="L24" s="11"/>
+    </row>
+    <row r="25" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>158</v>
+        <v>75</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>101</v>
+        <v>76</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>164</v>
       </c>
       <c r="F25" s="5">
-        <v>25000</v>
+        <v>120000</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="H25" s="2"/>
+        <v>104</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>34</v>
+      </c>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
-      <c r="K25" s="8"/>
-      <c r="L25" s="11"/>
+      <c r="K25" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="L25" s="11">
+        <v>120000</v>
+      </c>
     </row>
     <row r="26" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>77</v>
+        <v>165</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="F26" s="5">
-        <v>120000</v>
+        <v>80000</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>105</v>
+        <v>177</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>35</v>
+        <v>57</v>
       </c>
       <c r="I26" s="2"/>
-      <c r="J26" s="2"/>
-      <c r="K26" s="8" t="s">
-        <v>237</v>
-      </c>
-      <c r="L26" s="11">
-        <v>120000</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13" ht="34" x14ac:dyDescent="0.2">
+      <c r="J26" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="K26" s="8"/>
+      <c r="L26" s="11"/>
+    </row>
+    <row r="27" spans="1:13" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="F27" s="5">
-        <v>80000</v>
+        <v>15000</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>181</v>
+        <v>87</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>58</v>
+        <v>37</v>
       </c>
       <c r="I27" s="2"/>
-      <c r="J27" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="K27" s="8"/>
-      <c r="L27" s="11"/>
+      <c r="J27" s="2"/>
+      <c r="K27" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="L27" s="11">
+        <v>0</v>
+      </c>
     </row>
     <row r="28" spans="1:13" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>82</v>
+        <v>178</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>168</v>
+        <v>16</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="F28" s="5">
-        <v>15000</v>
+        <v>150000</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>88</v>
+        <v>179</v>
       </c>
       <c r="H28" s="2" t="s">
         <v>38</v>
@@ -2214,497 +2191,493 @@
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
       <c r="K28" s="8" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="L28" s="11">
-        <v>0</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="29" spans="1:13" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
-        <v>182</v>
+        <v>82</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="F29" s="5">
         <v>150000</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>39</v>
+        <v>55</v>
       </c>
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
       <c r="K29" s="8" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="L29" s="11">
         <v>150000</v>
       </c>
     </row>
-    <row r="30" spans="1:13" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>67</v>
+        <v>9</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E30" s="4" t="s">
-        <v>167</v>
+        <v>90</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>91</v>
       </c>
       <c r="F30" s="5">
-        <v>150000</v>
+        <v>120000</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>184</v>
+        <v>202</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
-      <c r="K30" s="8" t="s">
-        <v>218</v>
-      </c>
-      <c r="L30" s="11">
-        <v>150000</v>
-      </c>
+      <c r="K30" s="8"/>
+      <c r="L30" s="11"/>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>10</v>
+        <v>66</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>91</v>
+        <v>16</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F31" s="5">
-        <v>120000</v>
+        <v>60000</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>207</v>
+        <v>95</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="I31" s="2"/>
-      <c r="J31" s="2"/>
+      <c r="J31" s="2" t="s">
+        <v>93</v>
+      </c>
       <c r="K31" s="8"/>
       <c r="L31" s="11"/>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>17</v>
+        <v>74</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>95</v>
+        <v>19</v>
       </c>
       <c r="F32" s="5">
         <v>60000</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I32" s="2"/>
       <c r="J32" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="K32" s="8"/>
-      <c r="L32" s="11"/>
-    </row>
-    <row r="33" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+        <v>97</v>
+      </c>
+      <c r="K32" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="L32" s="11">
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
-        <v>97</v>
+        <v>157</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>75</v>
+        <v>19</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F33" s="5">
-        <v>60000</v>
+        <v>25000</v>
       </c>
       <c r="G33" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="I33" s="2"/>
+      <c r="J33" s="2"/>
+      <c r="K33" s="8"/>
+      <c r="L33" s="11"/>
+    </row>
+    <row r="34" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="H33" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I33" s="2"/>
-      <c r="J33" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="K33" s="8" t="s">
-        <v>210</v>
-      </c>
-      <c r="L33" s="11">
-        <v>55000</v>
-      </c>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A34" s="2" t="s">
-        <v>160</v>
-      </c>
       <c r="B34" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F34" s="5">
-        <v>25000</v>
+        <v>35000</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>161</v>
+        <v>101</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>204</v>
+        <v>52</v>
       </c>
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
-      <c r="K34" s="8"/>
-      <c r="L34" s="11"/>
-    </row>
-    <row r="35" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K34" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="L34" s="11">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
-        <v>100</v>
+        <v>159</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F35" s="5">
-        <v>35000</v>
+        <v>10000</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>102</v>
+        <v>160</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>53</v>
+        <v>201</v>
       </c>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
       <c r="K35" s="8" t="s">
-        <v>240</v>
+        <v>214</v>
       </c>
       <c r="L35" s="11">
-        <v>35000</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
-        <v>162</v>
+        <v>195</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>70</v>
+        <v>9</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>20</v>
+        <v>197</v>
       </c>
       <c r="F36" s="5">
-        <v>10000</v>
+        <v>40000</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>163</v>
+        <v>196</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
       <c r="K36" s="8" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="L36" s="11">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" ht="68" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
-        <v>199</v>
+        <v>220</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>10</v>
+        <v>69</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>201</v>
+        <v>19</v>
       </c>
       <c r="F37" s="5">
-        <v>40000</v>
-      </c>
-      <c r="G37" s="2" t="s">
-        <v>200</v>
+        <v>35000</v>
+      </c>
+      <c r="G37" s="4" t="s">
+        <v>221</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>202</v>
+        <v>51</v>
       </c>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
       <c r="K37" s="8" t="s">
-        <v>219</v>
+        <v>233</v>
       </c>
       <c r="L37" s="11">
         <v>35000</v>
       </c>
     </row>
-    <row r="38" spans="1:12" ht="68" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
-        <v>225</v>
+        <v>109</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>70</v>
+        <v>110</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>20</v>
+        <v>111</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>20</v>
+        <v>113</v>
       </c>
       <c r="F38" s="5">
-        <v>35000</v>
-      </c>
-      <c r="G38" s="4" t="s">
-        <v>226</v>
+        <v>20000</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>112</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
       <c r="K38" s="8" t="s">
-        <v>238</v>
+        <v>213</v>
       </c>
       <c r="L38" s="11">
-        <v>35000</v>
-      </c>
-    </row>
-    <row r="39" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="E39" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="F39" s="5">
+        <v>15000</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="I39" s="2"/>
+      <c r="J39" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="K39" s="8"/>
+      <c r="L39" s="11"/>
+    </row>
+    <row r="40" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="F40" s="5">
+        <v>8000</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="I40" s="2"/>
+      <c r="J40" s="2"/>
+      <c r="K40" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="L40" s="11">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="F39" s="5">
-        <v>20000</v>
-      </c>
-      <c r="G39" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="H39" s="2" t="s">
+      <c r="B41" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F41" s="5">
+        <v>4000</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="H41" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="I39" s="2"/>
-      <c r="J39" s="2"/>
-      <c r="K39" s="8" t="s">
-        <v>218</v>
-      </c>
-      <c r="L39" s="11">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="40" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="C40" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="F40" s="5">
-        <v>15000</v>
-      </c>
-      <c r="G40" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="H40" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="I40" s="2"/>
-      <c r="J40" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="K40" s="8"/>
-      <c r="L40" s="11"/>
-    </row>
-    <row r="41" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C41" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="E41" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="F41" s="5">
-        <v>8000</v>
-      </c>
-      <c r="G41" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="H41" s="2" t="s">
-        <v>55</v>
       </c>
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
       <c r="K41" s="8" t="s">
-        <v>222</v>
-      </c>
-      <c r="L41" s="11">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+        <v>217</v>
+      </c>
+      <c r="L41" s="11"/>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B42" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="B42" s="2" t="s">
-        <v>116</v>
-      </c>
       <c r="C42" s="3" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F42" s="5">
         <v>4000</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
-      <c r="K42" s="8" t="s">
-        <v>222</v>
-      </c>
+      <c r="K42" s="8"/>
       <c r="L42" s="11"/>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F43" s="5">
-        <v>4000</v>
+        <v>2000</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H43" s="2" t="s">
         <v>63</v>
@@ -2714,68 +2687,72 @@
       <c r="K43" s="8"/>
       <c r="L43" s="11"/>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>116</v>
+        <v>66</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>20</v>
+        <v>165</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>164</v>
       </c>
       <c r="F44" s="5">
-        <v>2000</v>
+        <v>10000</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="H44" s="2" t="s">
         <v>64</v>
       </c>
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
-      <c r="K44" s="8"/>
-      <c r="L44" s="11"/>
+      <c r="K44" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="L44" s="11">
+        <v>10000</v>
+      </c>
     </row>
     <row r="45" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>139</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>67</v>
+        <v>123</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="F45" s="5">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>138</v>
+        <v>181</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>65</v>
+        <v>40</v>
       </c>
       <c r="I45" s="2"/>
       <c r="J45" s="2"/>
-      <c r="K45" s="2" t="s">
-        <v>210</v>
+      <c r="K45" s="8" t="s">
+        <v>212</v>
       </c>
       <c r="L45" s="11">
-        <v>10000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
@@ -2783,30 +2760,30 @@
         <v>140</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="F46" s="5">
         <v>0</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
       <c r="K46" s="8" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="L46" s="11">
         <v>0</v>
@@ -2814,227 +2791,227 @@
     </row>
     <row r="47" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
-        <v>141</v>
+        <v>67</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>124</v>
+        <v>66</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>168</v>
+        <v>17</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="F47" s="5">
         <v>0</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>40</v>
+        <v>208</v>
       </c>
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
       <c r="K47" s="8" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="L47" s="11">
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
-        <v>68</v>
+        <v>14</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>67</v>
+        <v>9</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D48" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E48" s="2" t="s">
         <v>18</v>
-      </c>
-      <c r="E48" s="4" t="s">
-        <v>167</v>
       </c>
       <c r="F48" s="5">
         <v>0</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="H48" s="2" t="s">
-        <v>213</v>
-      </c>
+        <v>182</v>
+      </c>
+      <c r="H48" s="2"/>
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
       <c r="K48" s="8" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="L48" s="11">
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
-        <v>15</v>
+        <v>77</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>10</v>
+        <v>66</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E49" s="2" t="s">
-        <v>19</v>
+        <v>78</v>
+      </c>
+      <c r="E49" s="4" t="s">
+        <v>164</v>
       </c>
       <c r="F49" s="5">
         <v>0</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="H49" s="2"/>
+        <v>183</v>
+      </c>
+      <c r="H49" s="2" t="s">
+        <v>35</v>
+      </c>
       <c r="I49" s="2"/>
       <c r="J49" s="2"/>
-      <c r="K49" s="8" t="s">
-        <v>219</v>
-      </c>
-      <c r="L49" s="11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+      <c r="K49" s="8"/>
+      <c r="L49" s="11"/>
+    </row>
+    <row r="50" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
-        <v>78</v>
+        <v>131</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>67</v>
+        <v>110</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>79</v>
+        <v>165</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="F50" s="5">
         <v>0</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>36</v>
+        <v>56</v>
       </c>
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
-      <c r="K50" s="8"/>
-      <c r="L50" s="11"/>
-    </row>
-    <row r="51" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
+      <c r="K50" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="L50" s="11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="F51" s="5">
         <v>0</v>
       </c>
       <c r="G51" s="2" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="I51" s="2"/>
       <c r="J51" s="2"/>
-      <c r="K51" s="8" t="s">
-        <v>221</v>
-      </c>
-      <c r="L51" s="11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+      <c r="K51" s="8"/>
+      <c r="L51" s="11"/>
+    </row>
+    <row r="52" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>124</v>
+        <v>69</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="F52" s="5">
         <v>0</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
-      <c r="K52" s="8"/>
-      <c r="L52" s="11"/>
+      <c r="K52" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="L52" s="11">
+        <v>0</v>
+      </c>
     </row>
     <row r="53" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
         <v>133</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>70</v>
+        <v>9</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="F53" s="5">
         <v>0</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="I53" s="2"/>
       <c r="J53" s="2"/>
       <c r="K53" s="8" t="s">
-        <v>224</v>
+        <v>214</v>
       </c>
       <c r="L53" s="11">
         <v>0</v>
@@ -3045,139 +3022,105 @@
         <v>134</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>10</v>
+        <v>69</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="F54" s="5">
         <v>0</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
       <c r="K54" s="8" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="L54" s="11">
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
         <v>135</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>70</v>
+        <v>115</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="F55" s="5">
         <v>0</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="H55" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="I55" s="2"/>
       <c r="J55" s="2"/>
-      <c r="K55" s="8" t="s">
-        <v>217</v>
-      </c>
-      <c r="L55" s="11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+      <c r="K55" s="8"/>
+      <c r="L55" s="11"/>
+    </row>
+    <row r="56" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
         <v>136</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>116</v>
+        <v>66</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>168</v>
+        <v>189</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="F56" s="5">
         <v>0</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="I56" s="2"/>
       <c r="J56" s="2"/>
-      <c r="K56" s="8"/>
-      <c r="L56" s="11"/>
-    </row>
-    <row r="57" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="B57" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C57" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D57" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="E57" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="F57" s="5">
+      <c r="K56" s="15" t="s">
+        <v>212</v>
+      </c>
+      <c r="L56" s="11">
         <v>0</v>
       </c>
-      <c r="G57" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="H57" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="I57" s="2"/>
-      <c r="J57" s="2"/>
-      <c r="K57" s="15" t="s">
-        <v>217</v>
-      </c>
-      <c r="L57" s="11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="I58" s="9"/>
-      <c r="J58" s="13"/>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="I57" s="9"/>
+      <c r="J57" s="13"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M57" xr:uid="{60AABAA7-0A6C-104B-82C9-83D30D50B2A2}">
+  <autoFilter ref="A1:M56" xr:uid="{60AABAA7-0A6C-104B-82C9-83D30D50B2A2}">
     <filterColumn colId="2">
       <filters>
         <filter val="Disponible"/>
@@ -3185,7 +3128,7 @@
     </filterColumn>
   </autoFilter>
   <hyperlinks>
-    <hyperlink ref="J7" r:id="rId1" xr:uid="{C7799A81-F11B-B642-BEF0-047A2E3C329D}"/>
+    <hyperlink ref="J6" r:id="rId1" xr:uid="{C7799A81-F11B-B642-BEF0-047A2E3C329D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Venta de pesas, freidora, carpa playa y agregando sillones y aspiradora
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/momuychayis/Documents/Python courses/Ventas_casa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C36006C0-C9BC-0944-AD17-0FC2D5C28631}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12E7BFF7-0819-F948-8731-3E55A586055A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16420" xr2:uid="{CD00CDD9-C0C8-D147-B0FC-6E5A64DE4059}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{CD00CDD9-C0C8-D147-B0FC-6E5A64DE4059}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$58</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="247">
   <si>
     <t>Nombre</t>
   </si>
@@ -618,10 +618,6 @@
   </si>
   <si>
     <t>Gratis
-Esta en perfecto estado, solo tiene muchos años de uso constante</t>
-  </si>
-  <si>
-    <t>Gratis
 Practicamente nuevo</t>
   </si>
   <si>
@@ -793,6 +789,44 @@
   </si>
   <si>
     <t>Andres S</t>
+  </si>
+  <si>
+    <t>Gratis!
+Esta en perfecto estado, solo tiene muchos años de uso constante</t>
+  </si>
+  <si>
+    <t>Joselyn-Fabi</t>
+  </si>
+  <si>
+    <t>Martín</t>
+  </si>
+  <si>
+    <t>Sillones de exterior</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aspiradora </t>
+  </si>
+  <si>
+    <t>Sillones de mimbre para exteriores</t>
+  </si>
+  <si>
+    <t>Shark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No recuerdo
+</t>
+  </si>
+  <si>
+    <t>David</t>
+  </si>
+  <si>
+    <t>Nosotros ponemos 70mel por los regalos de cumple</t>
+  </si>
+  <si>
+    <t>Aspiradora de mano</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/-/es/Shark-CZ2001-Vertex-Aspiradora-autolimpiante/dp/B0C257RFWZ</t>
   </si>
 </sst>
 </file>
@@ -843,7 +877,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -870,43 +904,6 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -921,7 +918,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -945,15 +942,32 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1270,7 +1284,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60AABAA7-0A6C-104B-82C9-83D30D50B2A2}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:M57"/>
+  <dimension ref="A1:M58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="39.6640625" bestFit="1" customWidth="1"/>
@@ -1281,9 +1295,9 @@
     <col min="6" max="6" width="40.83203125" customWidth="1"/>
     <col min="7" max="7" width="140.1640625" customWidth="1"/>
     <col min="8" max="8" width="26.83203125" customWidth="1"/>
-    <col min="9" max="9" width="15.6640625" style="8" customWidth="1"/>
-    <col min="10" max="10" width="10.83203125" style="14" customWidth="1"/>
-    <col min="12" max="12" width="21.33203125" style="12" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" style="20" customWidth="1"/>
+    <col min="10" max="10" width="10.83203125" style="20" customWidth="1"/>
+    <col min="12" max="12" width="21.33203125" style="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">
@@ -1318,10 +1332,10 @@
         <v>7</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="L1" s="10" t="s">
-        <v>206</v>
+        <v>203</v>
+      </c>
+      <c r="L1" s="9" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="34" x14ac:dyDescent="0.2">
@@ -1352,7 +1366,7 @@
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
       <c r="K2" s="8"/>
-      <c r="L2" s="11"/>
+      <c r="L2" s="10"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
@@ -1374,7 +1388,7 @@
         <v>25000</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>36</v>
@@ -1384,7 +1398,7 @@
         <v>86</v>
       </c>
       <c r="K3" s="8"/>
-      <c r="L3" s="11"/>
+      <c r="L3" s="10"/>
     </row>
     <row r="4" spans="1:12" ht="102" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
@@ -1406,17 +1420,17 @@
         <v>4000000</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2" t="s">
         <v>130</v>
       </c>
       <c r="K4" s="8"/>
-      <c r="L4" s="11"/>
+      <c r="L4" s="10"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
@@ -1444,7 +1458,7 @@
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
       <c r="K5" s="8"/>
-      <c r="L5" s="11"/>
+      <c r="L5" s="10"/>
     </row>
     <row r="6" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
@@ -1469,16 +1483,16 @@
         <v>10</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="6" t="s">
         <v>8</v>
       </c>
       <c r="K6" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="L6" s="12">
+        <v>215</v>
+      </c>
+      <c r="L6" s="11">
         <v>130000</v>
       </c>
     </row>
@@ -1510,101 +1524,113 @@
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
       <c r="K7" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="L7" s="11">
+        <v>211</v>
+      </c>
+      <c r="L7" s="10">
         <v>120000</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F8" s="5">
         <v>34000</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
-      <c r="K8" s="8"/>
-      <c r="L8" s="11"/>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="K8" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="L8" s="10">
+        <v>34000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>224</v>
-      </c>
       <c r="C9" s="3" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F9" s="5">
         <v>19000</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
-      <c r="K9" s="8"/>
-      <c r="L9" s="11"/>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="K9" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="L9" s="10">
+        <v>19000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F10" s="5">
         <v>32000</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
-      <c r="K10" s="8"/>
-      <c r="L10" s="11"/>
+      <c r="K10" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="L10" s="10">
+        <v>32000</v>
+      </c>
     </row>
     <row r="11" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
@@ -1626,13 +1652,13 @@
         <v>220000</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
       <c r="J11" s="6"/>
       <c r="K11" s="8"/>
-      <c r="L11" s="11"/>
+      <c r="L11" s="10"/>
     </row>
     <row r="12" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
@@ -1654,13 +1680,13 @@
         <v>180000</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="6"/>
       <c r="K12" s="8"/>
-      <c r="L12" s="11"/>
+      <c r="L12" s="10"/>
     </row>
     <row r="13" spans="1:12" ht="119" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
@@ -1682,23 +1708,23 @@
         <v>80000</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
       <c r="K13" s="8" t="s">
-        <v>215</v>
-      </c>
-      <c r="L13" s="11">
+        <v>214</v>
+      </c>
+      <c r="L13" s="10">
         <v>70000</v>
       </c>
     </row>
     <row r="14" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>123</v>
@@ -1707,26 +1733,26 @@
         <v>20</v>
       </c>
       <c r="D14" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>192</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>193</v>
       </c>
       <c r="F14" s="5">
         <v>60000</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
       <c r="K14" s="8" t="s">
-        <v>205</v>
-      </c>
-      <c r="L14" s="11">
+        <v>204</v>
+      </c>
+      <c r="L14" s="10">
         <v>55000</v>
       </c>
     </row>
@@ -1760,9 +1786,9 @@
         <v>22</v>
       </c>
       <c r="K15" s="8" t="s">
-        <v>214</v>
-      </c>
-      <c r="L15" s="11">
+        <v>213</v>
+      </c>
+      <c r="L15" s="10">
         <v>30000</v>
       </c>
     </row>
@@ -1792,9 +1818,9 @@
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
       <c r="K16" s="8" t="s">
-        <v>214</v>
-      </c>
-      <c r="L16" s="11">
+        <v>213</v>
+      </c>
+      <c r="L16" s="10">
         <v>15000</v>
       </c>
     </row>
@@ -1826,9 +1852,9 @@
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
       <c r="K17" s="8" t="s">
-        <v>215</v>
-      </c>
-      <c r="L17" s="11">
+        <v>214</v>
+      </c>
+      <c r="L17" s="10">
         <v>35000</v>
       </c>
     </row>
@@ -1860,7 +1886,7 @@
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
       <c r="K18" s="8"/>
-      <c r="L18" s="11"/>
+      <c r="L18" s="10"/>
     </row>
     <row r="19" spans="1:13" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
@@ -1890,15 +1916,15 @@
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
       <c r="K19" s="8" t="s">
-        <v>217</v>
-      </c>
-      <c r="L19" s="11">
+        <v>216</v>
+      </c>
+      <c r="L19" s="10">
         <v>10000</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="34" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:13" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>69</v>
@@ -1924,9 +1950,9 @@
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
       <c r="K20" s="8" t="s">
-        <v>235</v>
-      </c>
-      <c r="L20" s="11">
+        <v>234</v>
+      </c>
+      <c r="L20" s="10">
         <v>100000</v>
       </c>
     </row>
@@ -1956,9 +1982,9 @@
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
       <c r="K21" s="8" t="s">
-        <v>218</v>
-      </c>
-      <c r="L21" s="11">
+        <v>217</v>
+      </c>
+      <c r="L21" s="10">
         <v>100000</v>
       </c>
     </row>
@@ -1992,9 +2018,9 @@
         <v>84</v>
       </c>
       <c r="K22" s="8" t="s">
-        <v>215</v>
-      </c>
-      <c r="L22" s="11">
+        <v>214</v>
+      </c>
+      <c r="L22" s="10">
         <v>25000</v>
       </c>
     </row>
@@ -2026,13 +2052,13 @@
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
       <c r="K23" s="8" t="s">
-        <v>205</v>
-      </c>
-      <c r="L23" s="11">
+        <v>204</v>
+      </c>
+      <c r="L23" s="10">
         <v>110000</v>
       </c>
       <c r="M23" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
@@ -2061,9 +2087,9 @@
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
       <c r="K24" s="8"/>
-      <c r="L24" s="11"/>
-    </row>
-    <row r="25" spans="1:13" ht="34" x14ac:dyDescent="0.2">
+      <c r="L24" s="10"/>
+    </row>
+    <row r="25" spans="1:13" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>75</v>
       </c>
@@ -2091,9 +2117,9 @@
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
       <c r="K25" s="8" t="s">
-        <v>232</v>
-      </c>
-      <c r="L25" s="11">
+        <v>231</v>
+      </c>
+      <c r="L25" s="10">
         <v>120000</v>
       </c>
     </row>
@@ -2127,7 +2153,7 @@
         <v>176</v>
       </c>
       <c r="K26" s="8"/>
-      <c r="L26" s="11"/>
+      <c r="L26" s="10"/>
     </row>
     <row r="27" spans="1:13" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
@@ -2157,9 +2183,9 @@
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
       <c r="K27" s="8" t="s">
-        <v>205</v>
-      </c>
-      <c r="L27" s="11">
+        <v>204</v>
+      </c>
+      <c r="L27" s="10">
         <v>0</v>
       </c>
     </row>
@@ -2191,9 +2217,9 @@
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
       <c r="K28" s="8" t="s">
-        <v>213</v>
-      </c>
-      <c r="L28" s="11">
+        <v>212</v>
+      </c>
+      <c r="L28" s="10">
         <v>150000</v>
       </c>
     </row>
@@ -2225,13 +2251,13 @@
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
       <c r="K29" s="8" t="s">
-        <v>213</v>
-      </c>
-      <c r="L29" s="11">
+        <v>212</v>
+      </c>
+      <c r="L29" s="10">
         <v>150000</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>89</v>
       </c>
@@ -2239,7 +2265,7 @@
         <v>9</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>90</v>
@@ -2251,15 +2277,22 @@
         <v>120000</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="H30" s="2" t="s">
         <v>48</v>
       </c>
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
-      <c r="K30" s="8"/>
-      <c r="L30" s="11"/>
+      <c r="K30" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="L30" s="10">
+        <v>50000</v>
+      </c>
+      <c r="M30" t="s">
+        <v>244</v>
+      </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
@@ -2291,7 +2324,7 @@
         <v>93</v>
       </c>
       <c r="K31" s="8"/>
-      <c r="L31" s="11"/>
+      <c r="L31" s="10"/>
     </row>
     <row r="32" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
@@ -2323,9 +2356,9 @@
         <v>97</v>
       </c>
       <c r="K32" s="8" t="s">
-        <v>205</v>
-      </c>
-      <c r="L32" s="11">
+        <v>204</v>
+      </c>
+      <c r="L32" s="10">
         <v>55000</v>
       </c>
     </row>
@@ -2352,14 +2385,14 @@
         <v>158</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
       <c r="K33" s="8"/>
-      <c r="L33" s="11"/>
-    </row>
-    <row r="34" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L33" s="10"/>
+    </row>
+    <row r="34" spans="1:12" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>99</v>
       </c>
@@ -2387,9 +2420,9 @@
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
       <c r="K34" s="8" t="s">
-        <v>235</v>
-      </c>
-      <c r="L34" s="11">
+        <v>234</v>
+      </c>
+      <c r="L34" s="10">
         <v>35000</v>
       </c>
     </row>
@@ -2416,20 +2449,20 @@
         <v>160</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
       <c r="K35" s="8" t="s">
-        <v>214</v>
-      </c>
-      <c r="L35" s="11">
+        <v>213</v>
+      </c>
+      <c r="L35" s="10">
         <v>10000</v>
       </c>
     </row>
     <row r="36" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>9</v>
@@ -2441,29 +2474,29 @@
         <v>23</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F36" s="5">
         <v>40000</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
       <c r="K36" s="8" t="s">
-        <v>214</v>
-      </c>
-      <c r="L36" s="11">
+        <v>213</v>
+      </c>
+      <c r="L36" s="10">
         <v>35000</v>
       </c>
     </row>
-    <row r="37" spans="1:12" ht="68" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:12" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>69</v>
@@ -2481,7 +2514,7 @@
         <v>35000</v>
       </c>
       <c r="G37" s="4" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H37" s="2" t="s">
         <v>51</v>
@@ -2489,9 +2522,9 @@
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
       <c r="K37" s="8" t="s">
-        <v>233</v>
-      </c>
-      <c r="L37" s="11">
+        <v>232</v>
+      </c>
+      <c r="L37" s="10">
         <v>35000</v>
       </c>
     </row>
@@ -2523,13 +2556,13 @@
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
       <c r="K38" s="8" t="s">
-        <v>213</v>
-      </c>
-      <c r="L38" s="11">
+        <v>212</v>
+      </c>
+      <c r="L38" s="10">
         <v>20000</v>
       </c>
     </row>
-    <row r="39" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:12" ht="28" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>117</v>
       </c>
@@ -2537,7 +2570,7 @@
         <v>123</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>118</v>
@@ -2558,8 +2591,12 @@
       <c r="J39" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="K39" s="8"/>
-      <c r="L39" s="11"/>
+      <c r="K39" s="8" t="s">
+        <v>236</v>
+      </c>
+      <c r="L39" s="10">
+        <v>15000</v>
+      </c>
     </row>
     <row r="40" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
@@ -2589,9 +2626,9 @@
       <c r="I40" s="2"/>
       <c r="J40" s="2"/>
       <c r="K40" s="8" t="s">
-        <v>217</v>
-      </c>
-      <c r="L40" s="11">
+        <v>216</v>
+      </c>
+      <c r="L40" s="10">
         <v>8000</v>
       </c>
     </row>
@@ -2623,9 +2660,9 @@
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
       <c r="K41" s="8" t="s">
-        <v>217</v>
-      </c>
-      <c r="L41" s="11"/>
+        <v>216</v>
+      </c>
+      <c r="L41" s="10"/>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
@@ -2655,7 +2692,7 @@
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
       <c r="K42" s="8"/>
-      <c r="L42" s="11"/>
+      <c r="L42" s="10"/>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
@@ -2685,7 +2722,7 @@
       <c r="I43" s="2"/>
       <c r="J43" s="2"/>
       <c r="K43" s="8"/>
-      <c r="L43" s="11"/>
+      <c r="L43" s="10"/>
     </row>
     <row r="44" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
@@ -2715,9 +2752,9 @@
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
       <c r="K44" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="L44" s="11">
+        <v>204</v>
+      </c>
+      <c r="L44" s="10">
         <v>10000</v>
       </c>
     </row>
@@ -2749,9 +2786,9 @@
       <c r="I45" s="2"/>
       <c r="J45" s="2"/>
       <c r="K45" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="L45" s="11">
+        <v>211</v>
+      </c>
+      <c r="L45" s="10">
         <v>0</v>
       </c>
     </row>
@@ -2783,9 +2820,9 @@
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
       <c r="K46" s="8" t="s">
-        <v>214</v>
-      </c>
-      <c r="L46" s="11">
+        <v>213</v>
+      </c>
+      <c r="L46" s="10">
         <v>0</v>
       </c>
     </row>
@@ -2812,14 +2849,14 @@
         <v>181</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
       <c r="K47" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="L47" s="11">
+        <v>211</v>
+      </c>
+      <c r="L47" s="10">
         <v>0</v>
       </c>
     </row>
@@ -2849,13 +2886,13 @@
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
       <c r="K48" s="8" t="s">
-        <v>214</v>
-      </c>
-      <c r="L48" s="11">
+        <v>213</v>
+      </c>
+      <c r="L48" s="10">
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
         <v>77</v>
       </c>
@@ -2863,7 +2900,7 @@
         <v>66</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>78</v>
@@ -2874,16 +2911,20 @@
       <c r="F49" s="5">
         <v>0</v>
       </c>
-      <c r="G49" s="2" t="s">
-        <v>183</v>
+      <c r="G49" s="4" t="s">
+        <v>235</v>
       </c>
       <c r="H49" s="2" t="s">
         <v>35</v>
       </c>
       <c r="I49" s="2"/>
       <c r="J49" s="2"/>
-      <c r="K49" s="8"/>
-      <c r="L49" s="11"/>
+      <c r="K49" s="8" t="s">
+        <v>236</v>
+      </c>
+      <c r="L49" s="10">
+        <v>0</v>
+      </c>
     </row>
     <row r="50" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
@@ -2905,7 +2946,7 @@
         <v>0</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="H50" s="2" t="s">
         <v>56</v>
@@ -2913,9 +2954,9 @@
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
       <c r="K50" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="L50" s="11">
+        <v>215</v>
+      </c>
+      <c r="L50" s="10">
         <v>0</v>
       </c>
     </row>
@@ -2939,7 +2980,7 @@
         <v>0</v>
       </c>
       <c r="G51" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="H51" s="2" t="s">
         <v>49</v>
@@ -2947,7 +2988,7 @@
       <c r="I51" s="2"/>
       <c r="J51" s="2"/>
       <c r="K51" s="8"/>
-      <c r="L51" s="11"/>
+      <c r="L51" s="10"/>
     </row>
     <row r="52" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
@@ -2969,7 +3010,7 @@
         <v>0</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="H52" s="2" t="s">
         <v>41</v>
@@ -2977,9 +3018,9 @@
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
       <c r="K52" s="8" t="s">
-        <v>219</v>
-      </c>
-      <c r="L52" s="11">
+        <v>218</v>
+      </c>
+      <c r="L52" s="10">
         <v>0</v>
       </c>
     </row>
@@ -3011,9 +3052,9 @@
       <c r="I53" s="2"/>
       <c r="J53" s="2"/>
       <c r="K53" s="8" t="s">
-        <v>214</v>
-      </c>
-      <c r="L53" s="11">
+        <v>213</v>
+      </c>
+      <c r="L53" s="10">
         <v>0</v>
       </c>
     </row>
@@ -3037,7 +3078,7 @@
         <v>0</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H54" s="2" t="s">
         <v>44</v>
@@ -3045,9 +3086,9 @@
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
       <c r="K54" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="L54" s="11">
+        <v>211</v>
+      </c>
+      <c r="L54" s="10">
         <v>0</v>
       </c>
     </row>
@@ -3079,48 +3120,110 @@
       <c r="I55" s="2"/>
       <c r="J55" s="2"/>
       <c r="K55" s="8"/>
-      <c r="L55" s="11"/>
+      <c r="L55" s="10"/>
     </row>
     <row r="56" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="2" t="s">
+      <c r="A56" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="B56" s="2" t="s">
+      <c r="B56" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="C56" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D56" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="E56" s="4" t="s">
+      <c r="C56" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D56" s="13" t="s">
+        <v>188</v>
+      </c>
+      <c r="E56" s="15" t="s">
         <v>164</v>
       </c>
-      <c r="F56" s="5">
+      <c r="F56" s="16">
         <v>0</v>
       </c>
-      <c r="G56" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="H56" s="2" t="s">
+      <c r="G56" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="H56" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="I56" s="2"/>
-      <c r="J56" s="2"/>
-      <c r="K56" s="15" t="s">
-        <v>212</v>
-      </c>
-      <c r="L56" s="11">
+      <c r="I56" s="13"/>
+      <c r="J56" s="13"/>
+      <c r="K56" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="L56" s="17">
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="I57" s="9"/>
-      <c r="J57" s="13"/>
+    <row r="57" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="18" t="s">
+        <v>238</v>
+      </c>
+      <c r="B57" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="C57" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E57" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="F57" s="5">
+        <v>20000</v>
+      </c>
+      <c r="G57" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="H57" s="8"/>
+      <c r="I57" s="8"/>
+      <c r="J57" s="8"/>
+      <c r="K57" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="L57" s="10">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" ht="34" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A58" s="18" t="s">
+        <v>239</v>
+      </c>
+      <c r="B58" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="C58" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="E58" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="F58" s="5">
+        <v>30000</v>
+      </c>
+      <c r="G58" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="H58" s="8"/>
+      <c r="I58" s="8"/>
+      <c r="J58" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="K58" s="8" t="s">
+        <v>243</v>
+      </c>
+      <c r="L58" s="10">
+        <v>30000</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M56" xr:uid="{60AABAA7-0A6C-104B-82C9-83D30D50B2A2}">
+  <autoFilter ref="A1:M58" xr:uid="{60AABAA7-0A6C-104B-82C9-83D30D50B2A2}">
     <filterColumn colId="2">
       <filters>
         <filter val="Disponible"/>

</xml_diff>